<commit_message>
shes ready to run
when I leave we will run the better sim and we can graph the results tomorrow for jake. should be a good time.
</commit_message>
<xml_diff>
--- a/offlineSimStuff/my_data.xlsx
+++ b/offlineSimStuff/my_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,7 +493,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>["S", 3]</t>
+          <t>['J', 3]</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -509,7 +509,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>NAN</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -519,7 +519,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>NAN</t>
+          <t>118.97412589514015</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -529,12 +529,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 16.0, 14.0, 11.0], [10.0, 14.0, 14.0, 10.0, 13.0, 10.0, 13.0, 13.0, 10.0, 13.0], [11.0, 14.0, 13.0, 10.0, 11.0, 13.0, 13.0, 13.0, 11.0, 11.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0]]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[[112.44641447647095, 114.85031037720012, 116.52791248674896, 115.85891140329656, 113.21864613940429, 110.97868750731607, 124.9841913773291, 119.2764553046238, 138.05880621062366, 123.65559715238055], [109.15885981568007, 127.90376913190084, 120.75050335770874, 125.21758830070394, 116.71002512007499, 119.50860497013846, 124.58658020111304, 123.52741675881569, 107.43687392616323, 115.42785667430499], [119.07485783560861, 126.79031263604321, 121.60307482277855, 120.13756089700493, 121.75609992823942, 109.23196407872541, 102.46261787986393, 120.63894261963637, 116.21218191096142, 133.10838739113834], [110.80652615784173, 130.21007348415472, 116.28454104215362, 124.37471905809966, 126.01936710248594, 117.79974505101194, 111.92366083505647, 116.7349094070488, 127.37202276761556, 109.49043509453175], [117.70136650103746, 123.62061326616035, 136.51940054110864, 113.81043523213455, 111.60943058133154, 103.19420122321401, 124.29239443949106, 123.92476956612742, 118.28789613435993, 113.62977658004425]]</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>["S", 3]</t>
+          <t>['S', 3]</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -555,14 +555,14 @@
         </is>
       </c>
       <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="b">
         <v>1</v>
       </c>
-      <c r="E3" t="b">
-        <v>0</v>
-      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>[[21.0, 19.0, 15.0, 15.0, 16.0, 14.0, 18.0, 12.0, 14.0, 16.0], [17.0, 17.0, 10.0, 17.0, 21.0, 18.0, 17.0, 10.0, 13.0, 20.0], [16.0, 15.0, 16.0, 17.0, 16.0, 14.0, 15.0, 16.0, 13.0, 22.0], [10.0, 21.0, 17.0, 13.0, 16.0, 11.0, 22.0, 20.0, 14.0, 16.0], [19.0, 15.0, 15.0, 18.0, 16.0, 15.0, 14.0, 14.0, 20.0, 14.0]]</t>
+          <t>[[10.0, 11.0, 11.0, 15.0, 13.0, 11.0, 13.0, 10.0, 13.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [13.0, 10.0, 12.0, 13.0, 13.0, 13.0, 13.0, 13.0, 10.0, 10.0], [16.0, 15.0, 14.0, 15.0, 12.0, 13.0, 14.0, 15.0, 14.0, 12.0], [13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 10.0]]</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>["J", 3]</t>
+          <t>['S', 3]</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -608,14 +608,14 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>NAN</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>119.10160000000003</t>
+          <t>NAN</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -635,12 +635,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
+          <t>[[17.0, 13.0, 12.0, 20.0, 17.0, 20.0, 14.0, 19.0, 15.0, 13.0], [14.0, 23.0, 16.0, 17.0, 20.0, 16.0, 13.0, 10.0, 14.0, 17.0], [14.0, 21.0, 16.0, 15.0, 18.0, 20.0, 11.0, 19.0, 16.0, 10.0], [13.0, 23.0, 18.0, 10.0, 21.0, 17.0, 14.0, 19.0, 14.0, 11.0], [16.0, 15.0, 18.0, 21.0, 16.0, 14.0, 15.0, 21.0, 10.0, 14.0]]</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
           <t>[]</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>[[114.17171163796559, 128.2630175467319, 124.5590043831875, 114.67634150040169, 110.40772912949686, 119.04747696068904, 127.60773831250162, 122.86591142260593, 112.20306141209522, 117.21400769432486], [114.17171163796559, 128.2630175467319, 124.5590043831875, 114.67634150040169, 110.40772912949686, 119.04747696068904, 127.60773831250162, 122.86591142260593, 112.20306141209522, 117.21400769432486], [114.17171163796559, 128.2630175467319, 124.5590043831875, 114.67634150040169, 110.40772912949686, 119.04747696068904, 127.60773831250162, 122.86591142260593, 112.20306141209522, 117.21400769432486], [114.17171163796559, 128.2630175467319, 124.5590043831875, 114.67634150040169, 110.40772912949686, 119.04747696068904, 127.60773831250162, 122.86591142260593, 112.20306141209522, 117.21400769432486], [114.17171163796559, 128.2630175467319, 124.5590043831875, 114.67634150040169, 110.40772912949686, 119.04747696068904, 127.60773831250162, 122.86591142260593, 112.20306141209522, 117.21400769432486]]</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>["J", 3]</t>
+          <t>[4, 3]</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -661,14 +661,14 @@
         </is>
       </c>
       <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="b">
         <v>1</v>
       </c>
-      <c r="E5" t="b">
-        <v>0</v>
-      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>NAN</t>
+          <t>11.600000000000001</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>119.10160000000003</t>
+          <t>150.26451265447554</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -688,12 +688,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 13.0, 13.0, 10.0], [12.0, 13.0, 12.0, 12.0, 12.0, 10.0, 12.0, 13.0, 12.0, 12.0], [15.0, 15.0, 16.0, 10.0, 13.0, 15.0, 13.0, 12.0, 16.0, 15.0]]</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>[[114.17171163796559, 128.2630175467319, 124.5590043831875, 114.67634150040169, 110.40772912949686, 119.04747696068904, 127.60773831250162, 122.86591142260593, 112.20306141209522, 117.21400769432486], [114.17171163796559, 128.2630175467319, 124.5590043831875, 114.67634150040169, 110.40772912949686, 119.04747696068904, 127.60773831250162, 122.86591142260593, 112.20306141209522, 117.21400769432486], [114.17171163796559, 128.2630175467319, 124.5590043831875, 114.67634150040169, 110.40772912949686, 119.04747696068904, 127.60773831250162, 122.86591142260593, 112.20306141209522, 117.21400769432486], [114.17171163796559, 128.2630175467319, 124.5590043831875, 114.67634150040169, 110.40772912949686, 119.04747696068904, 127.60773831250162, 122.86591142260593, 112.20306141209522, 117.21400769432486], [114.17171163796559, 128.2630175467319, 124.5590043831875, 114.67634150040169, 110.40772912949686, 119.04747696068904, 127.60773831250162, 122.86591142260593, 112.20306141209522, 117.21400769432486]]</t>
+          <t>[[135.2457612834003, 163.77341261986552, 162.40873381961111, 149.0994458362992, 156.82713559415382, 156.55912292433126, 113.50697504554023, 147.08762598241657, 163.34408183743966, 154.7404136687867], [159.30703654821008, 168.71723329384707, 148.13701007934066, 163.19968819985738, 159.7403841492182, 148.91971687619866, 147.48371687123245, 155.01342814276515, 157.90099002233933, 95.21105480835163], [161.26236091728572, 142.23010800471286, 135.46921531236518, 144.45609105172423, 157.6163836363749, 146.57023212864834, 153.96565701706126, 156.29974033174463, 158.97572506742313, 146.7847455240203], [165.01242687247526, 147.08180046812632, 155.45399660967865, 125.20426212794568, 157.68533728928213, 153.77449072584156, 154.84186505197957, 134.12948874071932, 161.445786218799, 149.0008048865131], [150.46986956421856, 169.39743466601539, 156.2356799658897, 127.85759069894185, 150.55713958438218, 161.0238665035684, 143.3258585600864, 131.74692866727162, 157.22867671517298, 151.89910221230426]]</t>
         </is>
       </c>
     </row>
@@ -714,14 +714,14 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>13.6</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>[[15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0]]</t>
+          <t>[[14.0, 14.0, 15.0, 15.0, 14.0, 14.0, 14.0, 14.0, 14.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0]]</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>[[144.17921313809367, 166.35220031338423, 141.22171984560214, 145.3855231073463, 144.90639468917507, 147.27238158198946, 154.3238228233656, 157.98766645630056, 148.09405833559518, 153.9072787005084], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959]]</t>
+          <t>[[153.17813738809068, 142.1654240481266, 161.089145166602, 153.67519683450485, 108.13579453286296, 155.2568836160391, 158.39700298915312, 156.1530879435942, 154.40968571816396, 161.16990075422314], [163.11110857806625, 149.9599480216834, 148.08195220221242, 143.91916324278904, 163.244325816204, 143.90515283961517, 161.3213293273694, 131.0840215308905, 161.5045914549302, 137.49866597760015], [154.72875285614313, 162.049171180831, 146.4895599726681, 160.9448635688605, 152.22921063346593, 154.02788565810914, 158.05488293943534, 160.58325472105608, 106.8581862774655, 147.66449118332577], [158.72313985353253, 131.23792951204507, 140.1461826418081, 161.3803764579432, 155.98126290666482, 155.0049759155173, 125.18100527967182, 152.1554354946612, 159.02827742458913, 164.7916735049274], [137.14422511107904, 129.30969233850746, 171.72531315982874, 129.654523283093, 178.25881870518367, 139.60269678368365, 133.46443895339144, 164.56452054581794, 161.9527514221011, 157.95327868867457]]</t>
         </is>
       </c>
     </row>
@@ -767,14 +767,14 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>13.4</t>
+          <t>11.200000000000001</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>150.13653127648766</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -794,12 +794,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>[[15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 13.0, 12.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0]]</t>
+          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 12.0, 12.0, 12.0, 12.0, 10.0, 12.0, 13.0, 12.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [14.0, 17.0, 12.0, 14.0, 14.0, 12.0, 15.0, 16.0, 12.0, 14.0]]</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>[[144.17921313809367, 166.35220031338423, 141.22171984560214, 145.3855231073463, 144.90639468917507, 147.27238158198946, 154.3238228233656, 157.98766645630056, 148.09405833559518, 153.9072787005084], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [144.30117409217885, 172.14729779439898, 142.40331771791733, 144.8190493875945, 163.38871241541744, 138.37602675777651, 145.19294131188033, 153.81985957820902, 145.16959966818743, 154.01228026780007], [138.5950961011988, 159.93270578904753, 145.68391375185405, 142.55305687560497, 151.24177471797898, 147.22991933251757, 155.39988729281495, 164.16938949754916, 152.11914188605147, 146.7053737467431], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959]]</t>
+          <t>[[154.36344535215304, 163.52982756793426, 146.9025445694372, 142.66416523350992, 148.29514298519496, 148.070996571783, 156.73145526719205, 146.90501471231136, 149.14692502008475, 147.02074171175997], [159.06291866347968, 152.74469351810455, 138.97276733048787, 162.29841231241943, 136.20700277766468, 136.30253318487186, 144.94198749708056, 155.70030063218982, 162.34915590595784, 155.0504871691043], [160.66568024432038, 157.47470609321786, 149.39590312047022, 130.4463821294525, 153.7827944374896, 156.48325416066206, 149.5729700634638, 140.0711270733987, 152.32467372239284, 153.41276794649258], [141.1064897126365, 149.18034444326906, 138.6775410344389, 127.9319560448643, 145.393821839696, 137.5447659626759, 166.42190622024893, 143.7918186376209, 173.5921030473251, 168.66478091616472], [163.42885191900396, 168.85020200484772, 129.3845840149361, 154.46688144539283, 140.55090586468302, 148.60449966196364, 155.8975179393106, 141.15607525895066, 163.78772492331126, 137.5030159589607]]</t>
         </is>
       </c>
     </row>
@@ -820,14 +820,14 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.333333333333334</t>
+          <t>12.000000000000002</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>150.30653170277293</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -847,12 +847,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>[[15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 13.0, 12.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 10.0, 12.0, 14.0, 13.0, 12.0, 12.0, 13.0, 10.0, 12.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0]]</t>
+          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 12.0, 12.0, 12.0, 10.0, 12.0, 13.0, 13.0, 12.0, 12.0], [10.0, 12.0, 13.0, 12.0, 12.0, 13.0, 12.0, 12.0, 12.0, 12.0], [13.0, 10.0, 13.0, 10.0, 10.0, 13.0, 14.0, 10.0, 13.0, 14.0], [14.0, 15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 15.0, 14.0, 12.0]]</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>[[144.17921313809367, 166.35220031338423, 141.22171984560214, 145.3855231073463, 144.90639468917507, 147.27238158198946, 154.3238228233656, 157.98766645630056, 148.09405833559518, 153.9072787005084], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [144.30117409217885, 172.14729779439898, 142.40331771791733, 144.8190493875945, 163.38871241541744, 138.37602675777651, 145.19294131188033, 153.81985957820902, 145.16959966818743, 154.01228026780007], [138.5950961011988, 159.93270578904753, 145.68391375185405, 142.55305687560497, 151.24177471797898, 147.22991933251757, 155.39988729281495, 164.16938949754916, 152.11914188605147, 146.7053737467431], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.08136289158472, 160.49623667828618, 145.4987985222077, 141.43986050360445, 157.9292714840807, 150.70287516416076, 161.7472400092508, 153.70033433406178, 149.3168725093424, 131.7174068947811], [140.98959900595693, 162.99321023852437, 140.38278876177927, 149.78099912120337, 160.5570071317603, 144.82442509913304, 158.9031371435798, 149.6418701897537, 146.87052710478156, 148.68669519488822], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [143.74044209255126, 161.8910669627725, 140.14184098297, 143.18716101161152, 164.7169006038425, 143.71132625069296, 157.7794211144888, 151.17537657648876, 142.12314403742783, 155.16357935851443], [138.30012114995344, 155.1088900607881, 133.72029570587694, 158.18967098930176, 157.62917959053266, 151.43673509842776, 151.9013337518322, 150.7223156274309, 150.6337752637292, 155.98794175348755]]</t>
+          <t>[[143.9365010009627, 157.98235095462442, 167.910854506371, 161.60083468044155, 100.14555174214257, 133.16135541779263, 166.5032285621916, 157.48128705312192, 161.0427083006713, 153.86558677304092], [156.3095011969217, 144.28072290451644, 134.93124983737604, 155.34255892631518, 156.35597334323265, 157.62323254879874, 143.79228582528162, 147.04124583465563, 155.208481007529, 152.74500756673362], [144.09116681052726, 150.76240896878033, 155.5310942238963, 162.07931153203845, 119.82517838267107, 151.31203656985218, 155.41578631061242, 141.82707669471853, 160.27415024700616, 162.51204925125782], [132.67162830264147, 164.6458461289911, 114.17684385938405, 172.30556789541166, 139.96358506354014, 153.4767815638743, 137.23585278346997, 161.6756748247832, 166.50178686783983, 160.976691701425], [155.72608205118942, 155.28022078580207, 137.25188611270423, 147.81174874362063, 144.9789624109234, 154.1697814216385, 166.71361912747716, 131.10571638899197, 168.70089503885902, 139.06663709199654]]</t>
         </is>
       </c>
     </row>
@@ -873,14 +873,14 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.0</t>
+          <t>12.8</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>149.55529385010266</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -900,12 +900,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>[[15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 13.0, 12.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 10.0, 12.0, 14.0, 13.0, 12.0, 12.0, 13.0, 10.0, 12.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 12.0, 12.0, 13.0, 12.0, 12.0, 12.0, 13.0, 12.0, 10.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0]]</t>
+          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 16.0, 14.0, 14.0, 14.0], [17.0, 14.0, 12.0, 12.0, 16.0, 15.0, 13.0, 13.0, 15.0, 13.0], [10.0, 12.0, 14.0, 12.0, 12.0, 12.0, 12.0, 13.0, 10.0, 13.0], [14.0, 16.0, 15.0, 12.0, 15.0, 13.0, 15.0, 12.0, 13.0, 15.0]]</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>[[144.17921313809367, 166.35220031338423, 141.22171984560214, 145.3855231073463, 144.90639468917507, 147.27238158198946, 154.3238228233656, 157.98766645630056, 148.09405833559518, 153.9072787005084], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [144.30117409217885, 172.14729779439898, 142.40331771791733, 144.8190493875945, 163.38871241541744, 138.37602675777651, 145.19294131188033, 153.81985957820902, 145.16959966818743, 154.01228026780007], [138.5950961011988, 159.93270578904753, 145.68391375185405, 142.55305687560497, 151.24177471797898, 147.22991933251757, 155.39988729281495, 164.16938949754916, 152.11914188605147, 146.7053737467431], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.08136289158472, 160.49623667828618, 145.4987985222077, 141.43986050360445, 157.9292714840807, 150.70287516416076, 161.7472400092508, 153.70033433406178, 149.3168725093424, 131.7174068947811], [140.98959900595693, 162.99321023852437, 140.38278876177927, 149.78099912120337, 160.5570071317603, 144.82442509913304, 158.9031371435798, 149.6418701897537, 146.87052710478156, 148.68669519488822], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [143.74044209255126, 161.8910669627725, 140.14184098297, 143.18716101161152, 164.7169006038425, 143.71132625069296, 157.7794211144888, 151.17537657648876, 142.12314403742783, 155.16357935851443], [138.30012114995344, 155.1088900607881, 133.72029570587694, 158.18967098930176, 157.62917959053266, 151.43673509842776, 151.9013337518322, 150.7223156274309, 150.6337752637292, 155.98794175348755], [141.69795868289765, 160.13482094842018, 142.09099875306856, 156.48707979343624, 164.16136161273224, 140.3901466759431, 151.0647504374702, 156.86462005597053, 146.45522413259854, 144.28329789882335], [148.2009552205627, 165.08780994485082, 152.3765345193727, 138.4276094077305, 150.13832991527178, 141.69081770545236, 158.60760144277467, 154.45947443059003, 140.62344799303048, 154.01767841172455], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [118.5901570276999, 164.29670634824816, 134.45811446512846, 143.58298645856215, 160.18352050060176, 149.6417928032472, 160.83886619545365, 172.6790173465758, 142.53701433592758, 156.82208350991596], [150.03780013362507, 157.96129209120093, 130.14080628606516, 146.83174460066198, 152.76236912074017, 152.49716682824345, 165.95665916466442, 146.33538452449912, 151.00434467421977, 150.10269156744056]]</t>
+          <t>[[142.5646497707894, 154.60165175532154, 120.42984201645552, 152.7725152088831, 157.24021495771333, 152.2112742345671, 153.85581973250174, 158.43764566886486, 157.21892729716325, 154.2977183491007], [163.11383666444496, 108.34146247009433, 151.5206943223244, 155.16161095210393, 163.3771234010503, 153.92292529524437, 156.51473811801426, 135.35998941519583, 162.97423779420842, 152.89582611571313], [177.08158709106598, 146.46687415538491, 116.0053308306409, 127.92310255543612, 162.31260809998463, 158.54766305926756, 146.02017522354853, 132.68260220690527, 162.7754647856039, 151.5037888551013], [141.20218440168742, 151.872688826403, 152.42019383668494, 147.54030585617357, 155.2653499072652, 157.3553526600218, 138.1534182716993, 160.2322868689816, 137.24186913366788, 162.34660922877586], [109.4937868388256, 144.3921699368205, 138.96928863981987, 175.4396603761238, 157.18174275354377, 139.68823753493, 149.8368586133563, 149.6388602488837, 155.34474977733584, 166.01717839143936]]</t>
         </is>
       </c>
     </row>
@@ -926,14 +926,14 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.040000000000001</t>
+          <t>11.599999999999998</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>150.36302589913603</t>
+          <t>150.14489772036896</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -953,12 +953,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>[[15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 13.0, 12.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 10.0, 12.0, 14.0, 13.0, 12.0, 12.0, 13.0, 10.0, 12.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 12.0, 12.0, 13.0, 12.0, 12.0, 12.0, 13.0, 12.0, 10.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0], [14.0, 14.0, 14.0, 16.0, 13.0, 14.0, 14.0, 14.0, 15.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 15.0, 10.0, 16.0], [13.0, 13.0, 12.0, 12.0, 12.0, 10.0, 12.0, 12.0, 12.0, 12.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0]]</t>
+          <t>[[12.0, 12.0, 12.0, 13.0, 12.0, 12.0, 12.0, 13.0, 12.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 12.0, 12.0, 13.0, 12.0, 10.0, 13.0, 12.0, 12.0, 12.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0]]</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>[[144.17921313809367, 166.35220031338423, 141.22171984560214, 145.3855231073463, 144.90639468917507, 147.27238158198946, 154.3238228233656, 157.98766645630056, 148.09405833559518, 153.9072787005084], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [144.30117409217885, 172.14729779439898, 142.40331771791733, 144.8190493875945, 163.38871241541744, 138.37602675777651, 145.19294131188033, 153.81985957820902, 145.16959966818743, 154.01228026780007], [138.5950961011988, 159.93270578904753, 145.68391375185405, 142.55305687560497, 151.24177471797898, 147.22991933251757, 155.39988729281495, 164.16938949754916, 152.11914188605147, 146.7053737467431], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.08136289158472, 160.49623667828618, 145.4987985222077, 141.43986050360445, 157.9292714840807, 150.70287516416076, 161.7472400092508, 153.70033433406178, 149.3168725093424, 131.7174068947811], [140.98959900595693, 162.99321023852437, 140.38278876177927, 149.78099912120337, 160.5570071317603, 144.82442509913304, 158.9031371435798, 149.6418701897537, 146.87052710478156, 148.68669519488822], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [143.74044209255126, 161.8910669627725, 140.14184098297, 143.18716101161152, 164.7169006038425, 143.71132625069296, 157.7794211144888, 151.17537657648876, 142.12314403742783, 155.16357935851443], [138.30012114995344, 155.1088900607881, 133.72029570587694, 158.18967098930176, 157.62917959053266, 151.43673509842776, 151.9013337518322, 150.7223156274309, 150.6337752637292, 155.98794175348755], [141.69795868289765, 160.13482094842018, 142.09099875306856, 156.48707979343624, 164.16136161273224, 140.3901466759431, 151.0647504374702, 156.86462005597053, 146.45522413259854, 144.28329789882335], [148.2009552205627, 165.08780994485082, 152.3765345193727, 138.4276094077305, 150.13832991527178, 141.69081770545236, 158.60760144277467, 154.45947443059003, 140.62344799303048, 154.01767841172455], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [118.5901570276999, 164.29670634824816, 134.45811446512846, 143.58298645856215, 160.18352050060176, 149.6417928032472, 160.83886619545365, 172.6790173465758, 142.53701433592758, 156.82208350991596], [150.03780013362507, 157.96129209120093, 130.14080628606516, 146.83174460066198, 152.76236912074017, 152.49716682824345, 165.95665916466442, 146.33538452449912, 151.00434467421977, 150.10269156744056], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [142.3175565041156, 157.07966095880727, 140.65243589292643, 146.39006015317656, 158.84130944106187, 143.41892367687444, 144.7012664163339, 170.44697427144183, 140.0615524164133, 159.72051926020941], [143.1609562614084, 152.080137850226, 146.5439872986877, 148.60330294578583, 159.51872916684874, 126.47997850559219, 147.3184981101908, 171.5368382288596, 156.186595413062, 152.20123521069925], [129.19861613587076, 165.00393668186683, 146.03750532321607, 138.08157977216175, 164.05997105719132, 159.2035061403781, 158.91703991686694, 160.55240623428136, 133.36065538477132, 149.21504234475606], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809]]</t>
+          <t>[[151.72145293488995, 158.6767179438192, 152.81526641052443, 144.90541010398505, 113.53737580322012, 161.64331232737538, 155.9955514216545, 161.14347017102355, 160.16148205443548, 143.03021982043288], [145.16896269401914, 161.1985821615475, 161.85009535966708, 127.5123723202587, 163.01545988629712, 154.30000801009263, 154.773243586621, 128.6405522110852, 160.85080453443194, 146.32017822734022], [150.75060518995346, 157.0381242428861, 143.6076181507443, 156.87348636732764, 144.96275402289078, 148.13824874524016, 125.11546779356085, 159.04033207095466, 161.94016082952263, 156.16346157827994], [138.29434235319417, 147.42185445615496, 132.56417263937888, 146.29255644629106, 158.1055998134475, 155.05057072384892, 158.96808688618864, 147.7451950263281, 159.22751976469112, 159.49501109687358], [152.95530830945626, 151.68711290851584, 146.19437316572473, 158.02131346825573, 149.27502488341514, 122.3587918286342, 145.72220749832312, 159.4534607370966, 146.15604211758355, 161.36556492096398]]</t>
         </is>
       </c>
     </row>
@@ -979,14 +979,14 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="E11" t="b">
         <v>1</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>13.066666666666666</t>
+          <t>12.000000000000002</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>150.1807921428966</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1006,12 +1006,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>[[15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 13.0, 12.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 10.0, 12.0, 14.0, 13.0, 12.0, 12.0, 13.0, 10.0, 12.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 12.0, 12.0, 13.0, 12.0, 12.0, 12.0, 13.0, 12.0, 10.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0], [14.0, 14.0, 14.0, 16.0, 13.0, 14.0, 14.0, 14.0, 15.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 15.0, 10.0, 16.0], [13.0, 13.0, 12.0, 12.0, 12.0, 10.0, 12.0, 12.0, 12.0, 12.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0], [14.0, 14.0, 14.0, 15.0, 15.0, 15.0, 15.0, 14.0, 14.0, 10.0], [14.0, 12.0, 14.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [13.0, 10.0, 10.0, 13.0, 13.0, 12.0, 13.0, 13.0, 10.0, 13.0]]</t>
+          <t>[[12.0, 12.0, 12.0, 12.0, 10.0, 12.0, 13.0, 12.0, 13.0, 12.0], [15.0, 15.0, 15.0, 13.0, 15.0, 13.0, 12.0, 12.0, 15.0, 15.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 10.0]]</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>[[144.17921313809367, 166.35220031338423, 141.22171984560214, 145.3855231073463, 144.90639468917507, 147.27238158198946, 154.3238228233656, 157.98766645630056, 148.09405833559518, 153.9072787005084], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [144.30117409217885, 172.14729779439898, 142.40331771791733, 144.8190493875945, 163.38871241541744, 138.37602675777651, 145.19294131188033, 153.81985957820902, 145.16959966818743, 154.01228026780007], [138.5950961011988, 159.93270578904753, 145.68391375185405, 142.55305687560497, 151.24177471797898, 147.22991933251757, 155.39988729281495, 164.16938949754916, 152.11914188605147, 146.7053737467431], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.08136289158472, 160.49623667828618, 145.4987985222077, 141.43986050360445, 157.9292714840807, 150.70287516416076, 161.7472400092508, 153.70033433406178, 149.3168725093424, 131.7174068947811], [140.98959900595693, 162.99321023852437, 140.38278876177927, 149.78099912120337, 160.5570071317603, 144.82442509913304, 158.9031371435798, 149.6418701897537, 146.87052710478156, 148.68669519488822], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [143.74044209255126, 161.8910669627725, 140.14184098297, 143.18716101161152, 164.7169006038425, 143.71132625069296, 157.7794211144888, 151.17537657648876, 142.12314403742783, 155.16357935851443], [138.30012114995344, 155.1088900607881, 133.72029570587694, 158.18967098930176, 157.62917959053266, 151.43673509842776, 151.9013337518322, 150.7223156274309, 150.6337752637292, 155.98794175348755], [141.69795868289765, 160.13482094842018, 142.09099875306856, 156.48707979343624, 164.16136161273224, 140.3901466759431, 151.0647504374702, 156.86462005597053, 146.45522413259854, 144.28329789882335], [148.2009552205627, 165.08780994485082, 152.3765345193727, 138.4276094077305, 150.13832991527178, 141.69081770545236, 158.60760144277467, 154.45947443059003, 140.62344799303048, 154.01767841172455], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [118.5901570276999, 164.29670634824816, 134.45811446512846, 143.58298645856215, 160.18352050060176, 149.6417928032472, 160.83886619545365, 172.6790173465758, 142.53701433592758, 156.82208350991596], [150.03780013362507, 157.96129209120093, 130.14080628606516, 146.83174460066198, 152.76236912074017, 152.49716682824345, 165.95665916466442, 146.33538452449912, 151.00434467421977, 150.10269156744056], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [142.3175565041156, 157.07966095880727, 140.65243589292643, 146.39006015317656, 158.84130944106187, 143.41892367687444, 144.7012664163339, 170.44697427144183, 140.0615524164133, 159.72051926020941], [143.1609562614084, 152.080137850226, 146.5439872986877, 148.60330294578583, 159.51872916684874, 126.47997850559219, 147.3184981101908, 171.5368382288596, 156.186595413062, 152.20123521069925], [129.19861613587076, 165.00393668186683, 146.03750532321607, 138.08157977216175, 164.05997105719132, 159.2035061403781, 158.91703991686694, 160.55240623428136, 133.36065538477132, 149.21504234475606], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [138.64000650561, 151.86873674340978, 138.32456021370763, 161.7335877936576, 151.6848443573904, 136.28496273135173, 151.04700607126532, 160.00284567116378, 150.87959157390125, 163.1641173299031], [143.48850037839307, 155.4933055473404, 140.58853020416862, 159.85835524368773, 164.78432821434643, 126.41020852112312, 151.1747917241475, 163.2933719101649, 149.21610263858187, 149.32276460940685], [139.87991413377017, 161.49924507831477, 140.27796357727996, 154.66410937869347, 144.83977940148063, 142.96223798876127, 159.0317739406516, 158.2554937467503, 147.191755098787, 155.02798664687145], [148.3011917158448, 152.24135327016148, 138.24322771433754, 159.91265087419478, 157.75302017067696, 158.5786808938281, 147.92743000516273, 133.41406355031097, 153.4502590576199, 153.80838173922336]]</t>
+          <t>[[155.91145631396216, 139.58254814469186, 153.91485014245944, 155.93643163721967, 159.2506586215597, 131.1461382764836, 154.00860602878268, 152.8244395130185, 159.4516955890683, 141.6034347241146], [146.9876252886497, 132.29818977510797, 180.7969192679678, 164.31527003741695, 138.30850821043535, 114.11296290457743, 173.66294769365012, 171.21578068306616, 141.48178211241017, 138.64961584331007], [153.53580644367003, 165.87315230754749, 158.1382138365809, 148.14341324089773, 135.54860727045968, 154.6400441866743, 148.6051461769168, 156.44176320947676, 130.34219055553237, 145.50869689569714], [139.8754638479635, 197.55288278093713, 136.19417340761478, 154.64116557696843, 139.1166064115473, 147.2060006353052, 143.6783990992699, 144.46298790766198, 165.77374200820947, 134.67103154658525], [184.99612434302418, 159.57372429976425, 124.23443097974597, 148.39767694924805, 165.8174998394593, 150.19162034106506, 152.87531788741384, 126.37437547373712, 131.42069204894497, 159.7487968289579]]</t>
         </is>
       </c>
     </row>
@@ -1032,14 +1032,14 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="E12" t="b">
         <v>1</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13.085714285714285</t>
+          <t>12.400000000000002</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>150.1796305779208</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1059,12 +1059,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>[[15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 13.0, 12.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 10.0, 12.0, 14.0, 13.0, 12.0, 12.0, 13.0, 10.0, 12.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 12.0, 12.0, 13.0, 12.0, 12.0, 12.0, 13.0, 12.0, 10.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0], [14.0, 14.0, 14.0, 16.0, 13.0, 14.0, 14.0, 14.0, 15.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 15.0, 10.0, 16.0], [13.0, 13.0, 12.0, 12.0, 12.0, 10.0, 12.0, 12.0, 12.0, 12.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0], [14.0, 14.0, 14.0, 15.0, 15.0, 15.0, 15.0, 14.0, 14.0, 10.0], [14.0, 12.0, 14.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [13.0, 10.0, 10.0, 13.0, 13.0, 12.0, 13.0, 13.0, 10.0, 13.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 16.0, 12.0, 12.0], [13.0, 13.0, 12.0, 12.0, 12.0, 10.0, 12.0, 12.0, 12.0, 12.0], [12.0, 14.0, 14.0, 16.0, 15.0, 14.0, 14.0, 16.0, 12.0, 13.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0]]</t>
+          <t>[[13.0, 10.0, 13.0, 12.0, 12.0, 12.0, 13.0, 10.0, 13.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [14.0, 12.0, 16.0, 15.0, 14.0, 15.0, 12.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 13.0, 16.0, 13.0, 15.0, 14.0, 15.0, 16.0, 14.0, 12.0]]</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>[[144.17921313809367, 166.35220031338423, 141.22171984560214, 145.3855231073463, 144.90639468917507, 147.27238158198946, 154.3238228233656, 157.98766645630056, 148.09405833559518, 153.9072787005084], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [144.30117409217885, 172.14729779439898, 142.40331771791733, 144.8190493875945, 163.38871241541744, 138.37602675777651, 145.19294131188033, 153.81985957820902, 145.16959966818743, 154.01228026780007], [138.5950961011988, 159.93270578904753, 145.68391375185405, 142.55305687560497, 151.24177471797898, 147.22991933251757, 155.39988729281495, 164.16938949754916, 152.11914188605147, 146.7053737467431], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.08136289158472, 160.49623667828618, 145.4987985222077, 141.43986050360445, 157.9292714840807, 150.70287516416076, 161.7472400092508, 153.70033433406178, 149.3168725093424, 131.7174068947811], [140.98959900595693, 162.99321023852437, 140.38278876177927, 149.78099912120337, 160.5570071317603, 144.82442509913304, 158.9031371435798, 149.6418701897537, 146.87052710478156, 148.68669519488822], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [143.74044209255126, 161.8910669627725, 140.14184098297, 143.18716101161152, 164.7169006038425, 143.71132625069296, 157.7794211144888, 151.17537657648876, 142.12314403742783, 155.16357935851443], [138.30012114995344, 155.1088900607881, 133.72029570587694, 158.18967098930176, 157.62917959053266, 151.43673509842776, 151.9013337518322, 150.7223156274309, 150.6337752637292, 155.98794175348755], [141.69795868289765, 160.13482094842018, 142.09099875306856, 156.48707979343624, 164.16136161273224, 140.3901466759431, 151.0647504374702, 156.86462005597053, 146.45522413259854, 144.28329789882335], [148.2009552205627, 165.08780994485082, 152.3765345193727, 138.4276094077305, 150.13832991527178, 141.69081770545236, 158.60760144277467, 154.45947443059003, 140.62344799303048, 154.01767841172455], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [118.5901570276999, 164.29670634824816, 134.45811446512846, 143.58298645856215, 160.18352050060176, 149.6417928032472, 160.83886619545365, 172.6790173465758, 142.53701433592758, 156.82208350991596], [150.03780013362507, 157.96129209120093, 130.14080628606516, 146.83174460066198, 152.76236912074017, 152.49716682824345, 165.95665916466442, 146.33538452449912, 151.00434467421977, 150.10269156744056], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [142.3175565041156, 157.07966095880727, 140.65243589292643, 146.39006015317656, 158.84130944106187, 143.41892367687444, 144.7012664163339, 170.44697427144183, 140.0615524164133, 159.72051926020941], [143.1609562614084, 152.080137850226, 146.5439872986877, 148.60330294578583, 159.51872916684874, 126.47997850559219, 147.3184981101908, 171.5368382288596, 156.186595413062, 152.20123521069925], [129.19861613587076, 165.00393668186683, 146.03750532321607, 138.08157977216175, 164.05997105719132, 159.2035061403781, 158.91703991686694, 160.55240623428136, 133.36065538477132, 149.21504234475606], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [138.64000650561, 151.86873674340978, 138.32456021370763, 161.7335877936576, 151.6848443573904, 136.28496273135173, 151.04700607126532, 160.00284567116378, 150.87959157390125, 163.1641173299031], [143.48850037839307, 155.4933055473404, 140.58853020416862, 159.85835524368773, 164.78432821434643, 126.41020852112312, 151.1747917241475, 163.2933719101649, 149.21610263858187, 149.32276460940685], [139.87991413377017, 161.49924507831477, 140.27796357727996, 154.66410937869347, 144.83977940148063, 142.96223798876127, 159.0317739406516, 158.2554937467503, 147.191755098787, 155.02798664687145], [148.3011917158448, 152.24135327016148, 138.24322771433754, 159.91265087419478, 157.75302017067696, 158.5786808938281, 147.92743000516273, 133.41406355031097, 153.4502590576199, 153.80838173922336], [142.47324381977754, 159.75391385863625, 139.89686476919496, 145.92151539200015, 165.15378792221145, 141.8884481702422, 147.56315632618478, 157.37789100557123, 152.37492819700643, 151.2265095305356], [151.77483014045058, 157.36992639649077, 145.1618572256677, 158.0463074247516, 156.45693331800123, 120.78821544824784, 148.9198164926133, 152.63719450795264, 157.35176560591893, 155.12341243126613], [122.56086781889486, 153.33018154775155, 138.73316026639344, 162.8616151383083, 160.47717131128687, 144.43501925639598, 153.8554606392985, 160.9905612202666, 141.2595350303938, 165.12668676237058], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992]]</t>
+          <t>[[137.45214988332003, 117.32273171879662, 151.95131782480888, 160.71957861359766, 157.08001203957724, 152.16618601697434, 168.97136573215377, 148.4424836050697, 160.4282205706354, 149.09621298642708], [141.5813086142579, 157.45287978407345, 157.4269475809512, 155.57412391598717, 150.2632437202302, 157.43826063954947, 123.3221444982746, 142.63029827864364, 163.86181095373334, 154.0792410056597], [155.55409319471985, 146.22882559890937, 161.95160545732227, 132.5173879064515, 159.31973134549426, 156.86411112419577, 152.02018604464484, 140.76955817481803, 148.39130005479987, 150.01346009000474], [155.9718635998441, 156.92779829112703, 135.03163729519343, 158.9466621615339, 153.12509089564654, 158.20216943775617, 125.42912945985944, 153.14578067210718, 148.71920569520543, 148.96115542232312], [167.6179359529006, 147.1585369439073, 155.5404851292476, 144.89517762225708, 162.65348200936361, 162.0000319544627, 157.69067369633433, 146.36809202663585, 117.380735210085, 142.3251084461665]]</t>
         </is>
       </c>
     </row>
@@ -1085,14 +1085,14 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="E13" t="b">
         <v>1</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>13.1</t>
+          <t>10.4</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>149.69164070568888</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1112,12 +1112,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>[[15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 13.0, 12.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 10.0, 12.0, 14.0, 13.0, 12.0, 12.0, 13.0, 10.0, 12.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 12.0, 12.0, 13.0, 12.0, 12.0, 12.0, 13.0, 12.0, 10.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0], [14.0, 14.0, 14.0, 16.0, 13.0, 14.0, 14.0, 14.0, 15.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 15.0, 10.0, 16.0], [13.0, 13.0, 12.0, 12.0, 12.0, 10.0, 12.0, 12.0, 12.0, 12.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0], [14.0, 14.0, 14.0, 15.0, 15.0, 15.0, 15.0, 14.0, 14.0, 10.0], [14.0, 12.0, 14.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [13.0, 10.0, 10.0, 13.0, 13.0, 12.0, 13.0, 13.0, 10.0, 13.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 16.0, 12.0, 12.0], [13.0, 13.0, 12.0, 12.0, 12.0, 10.0, 12.0, 12.0, 12.0, 12.0], [12.0, 14.0, 14.0, 16.0, 15.0, 14.0, 14.0, 16.0, 12.0, 13.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [10.0, 14.0, 12.0, 10.0, 12.0, 13.0, 13.0, 11.0, 12.0, 13.0], [14.0, 14.0, 12.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0]]</t>
+          <t>[[10.0, 12.0, 13.0, 12.0, 12.0, 12.0, 12.0, 13.0, 12.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0]]</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>[[144.17921313809367, 166.35220031338423, 141.22171984560214, 145.3855231073463, 144.90639468917507, 147.27238158198946, 154.3238228233656, 157.98766645630056, 148.09405833559518, 153.9072787005084], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [144.30117409217885, 172.14729779439898, 142.40331771791733, 144.8190493875945, 163.38871241541744, 138.37602675777651, 145.19294131188033, 153.81985957820902, 145.16959966818743, 154.01228026780007], [138.5950961011988, 159.93270578904753, 145.68391375185405, 142.55305687560497, 151.24177471797898, 147.22991933251757, 155.39988729281495, 164.16938949754916, 152.11914188605147, 146.7053737467431], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.08136289158472, 160.49623667828618, 145.4987985222077, 141.43986050360445, 157.9292714840807, 150.70287516416076, 161.7472400092508, 153.70033433406178, 149.3168725093424, 131.7174068947811], [140.98959900595693, 162.99321023852437, 140.38278876177927, 149.78099912120337, 160.5570071317603, 144.82442509913304, 158.9031371435798, 149.6418701897537, 146.87052710478156, 148.68669519488822], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [143.74044209255126, 161.8910669627725, 140.14184098297, 143.18716101161152, 164.7169006038425, 143.71132625069296, 157.7794211144888, 151.17537657648876, 142.12314403742783, 155.16357935851443], [138.30012114995344, 155.1088900607881, 133.72029570587694, 158.18967098930176, 157.62917959053266, 151.43673509842776, 151.9013337518322, 150.7223156274309, 150.6337752637292, 155.98794175348755], [141.69795868289765, 160.13482094842018, 142.09099875306856, 156.48707979343624, 164.16136161273224, 140.3901466759431, 151.0647504374702, 156.86462005597053, 146.45522413259854, 144.28329789882335], [148.2009552205627, 165.08780994485082, 152.3765345193727, 138.4276094077305, 150.13832991527178, 141.69081770545236, 158.60760144277467, 154.45947443059003, 140.62344799303048, 154.01767841172455], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [118.5901570276999, 164.29670634824816, 134.45811446512846, 143.58298645856215, 160.18352050060176, 149.6417928032472, 160.83886619545365, 172.6790173465758, 142.53701433592758, 156.82208350991596], [150.03780013362507, 157.96129209120093, 130.14080628606516, 146.83174460066198, 152.76236912074017, 152.49716682824345, 165.95665916466442, 146.33538452449912, 151.00434467421977, 150.10269156744056], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [142.3175565041156, 157.07966095880727, 140.65243589292643, 146.39006015317656, 158.84130944106187, 143.41892367687444, 144.7012664163339, 170.44697427144183, 140.0615524164133, 159.72051926020941], [143.1609562614084, 152.080137850226, 146.5439872986877, 148.60330294578583, 159.51872916684874, 126.47997850559219, 147.3184981101908, 171.5368382288596, 156.186595413062, 152.20123521069925], [129.19861613587076, 165.00393668186683, 146.03750532321607, 138.08157977216175, 164.05997105719132, 159.2035061403781, 158.91703991686694, 160.55240623428136, 133.36065538477132, 149.21504234475606], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [138.64000650561, 151.86873674340978, 138.32456021370763, 161.7335877936576, 151.6848443573904, 136.28496273135173, 151.04700607126532, 160.00284567116378, 150.87959157390125, 163.1641173299031], [143.48850037839307, 155.4933055473404, 140.58853020416862, 159.85835524368773, 164.78432821434643, 126.41020852112312, 151.1747917241475, 163.2933719101649, 149.21610263858187, 149.32276460940685], [139.87991413377017, 161.49924507831477, 140.27796357727996, 154.66410937869347, 144.83977940148063, 142.96223798876127, 159.0317739406516, 158.2554937467503, 147.191755098787, 155.02798664687145], [148.3011917158448, 152.24135327016148, 138.24322771433754, 159.91265087419478, 157.75302017067696, 158.5786808938281, 147.92743000516273, 133.41406355031097, 153.4502590576199, 153.80838173922336], [142.47324381977754, 159.75391385863625, 139.89686476919496, 145.92151539200015, 165.15378792221145, 141.8884481702422, 147.56315632618478, 157.37789100557123, 152.37492819700643, 151.2265095305356], [151.77483014045058, 157.36992639649077, 145.1618572256677, 158.0463074247516, 156.45693331800123, 120.78821544824784, 148.9198164926133, 152.63719450795264, 157.35176560591893, 155.12341243126613], [122.56086781889486, 153.33018154775155, 138.73316026639344, 162.8616151383083, 160.47717131128687, 144.43501925639598, 153.8554606392985, 160.9905612202666, 141.2595350303938, 165.12668676237058], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [137.71140916636776, 159.04502682053018, 146.36776204231367, 137.6717594479347, 149.78346457725695, 149.8343764514719, 156.96511399072568, 165.1925738690632, 151.00844474590428, 150.0503278797923], [138.69691740865682, 161.36899676610903, 141.0319809300706, 142.05497300143577, 151.9853314935421, 150.1777877692477, 158.95250888203665, 158.09076104019178, 150.52377473544067, 150.74722696462945], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [148.2009552205627, 165.08780994485082, 152.3765345193727, 138.4276094077305, 150.13832991527178, 141.69081770545236, 158.60760144277467, 154.45947443059003, 140.62344799303048, 154.01767841172455], [138.68858555784465, 155.72401439258195, 130.9195634604849, 164.28562240424654, 170.29051638672433, 139.7351254814477, 149.6251369865507, 161.88719987536257, 156.7102103479174, 135.7642840981997]]</t>
+          <t>[[158.62041885331553, 158.23383960084414, 166.97624552411918, 149.97124882336453, 154.14136870762104, 134.3229584931898, 129.9478644072818, 155.30510841039376, 142.9494992782937, 153.1617068929371], [151.1958646435784, 161.84783569430147, 138.37095370616584, 157.5056829002396, 98.45353404666847, 151.49960774624148, 158.56948785946344, 159.1102110803948, 168.0097060945943, 159.06737521971283], [149.40815605527584, 148.59337676491242, 158.92241884689602, 166.80350913822008, 159.72698284719294, 150.66927251043597, 161.56114590987318, 159.48294884219067, 99.77183718839709, 148.69061088796633], [147.76157068122038, 147.97840546452133, 138.48312260155762, 146.16478033600677, 138.29404923753583, 161.30939477598423, 143.87208646917998, 168.40587157611935, 145.6502074870022, 148.58262567395386], [151.01110222414994, 156.90050126190806, 132.49301037136476, 150.77211922652214, 147.14023219694178, 146.81381772839663, 143.42289714121983, 132.93131490235015, 154.3967684029704, 171.3073805514561]]</t>
         </is>
       </c>
     </row>
@@ -1138,14 +1138,14 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="E14" t="b">
         <v>1</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>13.066666666666666</t>
+          <t>11.599999999999998</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>150.03221041627856</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,12 +1165,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>[[15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 13.0, 12.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 10.0, 12.0, 14.0, 13.0, 12.0, 12.0, 13.0, 10.0, 12.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 12.0, 12.0, 13.0, 12.0, 12.0, 12.0, 13.0, 12.0, 10.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0], [14.0, 14.0, 14.0, 16.0, 13.0, 14.0, 14.0, 14.0, 15.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 15.0, 10.0, 16.0], [13.0, 13.0, 12.0, 12.0, 12.0, 10.0, 12.0, 12.0, 12.0, 12.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0], [14.0, 14.0, 14.0, 15.0, 15.0, 15.0, 15.0, 14.0, 14.0, 10.0], [14.0, 12.0, 14.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [13.0, 10.0, 10.0, 13.0, 13.0, 12.0, 13.0, 13.0, 10.0, 13.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 16.0, 12.0, 12.0], [13.0, 13.0, 12.0, 12.0, 12.0, 10.0, 12.0, 12.0, 12.0, 12.0], [12.0, 14.0, 14.0, 16.0, 15.0, 14.0, 14.0, 16.0, 12.0, 13.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [10.0, 14.0, 12.0, 10.0, 12.0, 13.0, 13.0, 11.0, 12.0, 13.0], [14.0, 14.0, 12.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 14.0, 15.0, 12.0], [10.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 13.0, 10.0, 13.0], [10.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 13.0, 10.0, 13.0], [13.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0]]</t>
+          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 12.0, 10.0], [12.0, 12.0, 13.0, 12.0, 12.0, 12.0, 12.0, 12.0, 13.0, 10.0], [15.0, 16.0, 15.0, 15.0, 12.0, 12.0, 14.0, 12.0, 14.0, 15.0]]</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>[[144.17921313809367, 166.35220031338423, 141.22171984560214, 145.3855231073463, 144.90639468917507, 147.27238158198946, 154.3238228233656, 157.98766645630056, 148.09405833559518, 153.9072787005084], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [144.30117409217885, 172.14729779439898, 142.40331771791733, 144.8190493875945, 163.38871241541744, 138.37602675777651, 145.19294131188033, 153.81985957820902, 145.16959966818743, 154.01228026780007], [138.5950961011988, 159.93270578904753, 145.68391375185405, 142.55305687560497, 151.24177471797898, 147.22991933251757, 155.39988729281495, 164.16938949754916, 152.11914188605147, 146.7053737467431], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.08136289158472, 160.49623667828618, 145.4987985222077, 141.43986050360445, 157.9292714840807, 150.70287516416076, 161.7472400092508, 153.70033433406178, 149.3168725093424, 131.7174068947811], [140.98959900595693, 162.99321023852437, 140.38278876177927, 149.78099912120337, 160.5570071317603, 144.82442509913304, 158.9031371435798, 149.6418701897537, 146.87052710478156, 148.68669519488822], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [143.74044209255126, 161.8910669627725, 140.14184098297, 143.18716101161152, 164.7169006038425, 143.71132625069296, 157.7794211144888, 151.17537657648876, 142.12314403742783, 155.16357935851443], [138.30012114995344, 155.1088900607881, 133.72029570587694, 158.18967098930176, 157.62917959053266, 151.43673509842776, 151.9013337518322, 150.7223156274309, 150.6337752637292, 155.98794175348755], [141.69795868289765, 160.13482094842018, 142.09099875306856, 156.48707979343624, 164.16136161273224, 140.3901466759431, 151.0647504374702, 156.86462005597053, 146.45522413259854, 144.28329789882335], [148.2009552205627, 165.08780994485082, 152.3765345193727, 138.4276094077305, 150.13832991527178, 141.69081770545236, 158.60760144277467, 154.45947443059003, 140.62344799303048, 154.01767841172455], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [118.5901570276999, 164.29670634824816, 134.45811446512846, 143.58298645856215, 160.18352050060176, 149.6417928032472, 160.83886619545365, 172.6790173465758, 142.53701433592758, 156.82208350991596], [150.03780013362507, 157.96129209120093, 130.14080628606516, 146.83174460066198, 152.76236912074017, 152.49716682824345, 165.95665916466442, 146.33538452449912, 151.00434467421977, 150.10269156744056], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [142.3175565041156, 157.07966095880727, 140.65243589292643, 146.39006015317656, 158.84130944106187, 143.41892367687444, 144.7012664163339, 170.44697427144183, 140.0615524164133, 159.72051926020941], [143.1609562614084, 152.080137850226, 146.5439872986877, 148.60330294578583, 159.51872916684874, 126.47997850559219, 147.3184981101908, 171.5368382288596, 156.186595413062, 152.20123521069925], [129.19861613587076, 165.00393668186683, 146.03750532321607, 138.08157977216175, 164.05997105719132, 159.2035061403781, 158.91703991686694, 160.55240623428136, 133.36065538477132, 149.21504234475606], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [138.64000650561, 151.86873674340978, 138.32456021370763, 161.7335877936576, 151.6848443573904, 136.28496273135173, 151.04700607126532, 160.00284567116378, 150.87959157390125, 163.1641173299031], [143.48850037839307, 155.4933055473404, 140.58853020416862, 159.85835524368773, 164.78432821434643, 126.41020852112312, 151.1747917241475, 163.2933719101649, 149.21610263858187, 149.32276460940685], [139.87991413377017, 161.49924507831477, 140.27796357727996, 154.66410937869347, 144.83977940148063, 142.96223798876127, 159.0317739406516, 158.2554937467503, 147.191755098787, 155.02798664687145], [148.3011917158448, 152.24135327016148, 138.24322771433754, 159.91265087419478, 157.75302017067696, 158.5786808938281, 147.92743000516273, 133.41406355031097, 153.4502590576199, 153.80838173922336], [142.47324381977754, 159.75391385863625, 139.89686476919496, 145.92151539200015, 165.15378792221145, 141.8884481702422, 147.56315632618478, 157.37789100557123, 152.37492819700643, 151.2265095305356], [151.77483014045058, 157.36992639649077, 145.1618572256677, 158.0463074247516, 156.45693331800123, 120.78821544824784, 148.9198164926133, 152.63719450795264, 157.35176560591893, 155.12341243126613], [122.56086781889486, 153.33018154775155, 138.73316026639344, 162.8616151383083, 160.47717131128687, 144.43501925639598, 153.8554606392985, 160.9905612202666, 141.2595350303938, 165.12668676237058], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [137.71140916636776, 159.04502682053018, 146.36776204231367, 137.6717594479347, 149.78346457725695, 149.8343764514719, 156.96511399072568, 165.1925738690632, 151.00844474590428, 150.0503278797923], [138.69691740865682, 161.36899676610903, 141.0319809300706, 142.05497300143577, 151.9853314935421, 150.1777877692477, 158.95250888203665, 158.09076104019178, 150.52377473544067, 150.74722696462945], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [148.2009552205627, 165.08780994485082, 152.3765345193727, 138.4276094077305, 150.13832991527178, 141.69081770545236, 158.60760144277467, 154.45947443059003, 140.62344799303048, 154.01767841172455], [138.68858555784465, 155.72401439258195, 130.9195634604849, 164.28562240424654, 170.29051638672433, 139.7351254814477, 149.6251369865507, 161.88719987536257, 156.7102103479174, 135.7642840981997], [146.96819049514585, 166.07135480306746, 149.9806344602439, 143.10317688672225, 153.82144256053363, 123.85796945663141, 162.44295163751056, 164.80514965374246, 141.46778093293213, 151.111608104831], [142.3175565041156, 157.07966095880727, 140.65243589292643, 146.39006015317656, 158.84130944106187, 143.41892367687444, 144.7012664163339, 170.44697427144183, 140.0615524164133, 159.72051926020941], [142.3175565041156, 157.07966095880727, 140.65243589292643, 146.39006015317656, 158.84130944106187, 143.41892367687444, 144.7012664163339, 170.44697427144183, 140.0615524164133, 159.72051926020941], [128.2589192837509, 166.08527098056226, 140.48593481787083, 156.75657747977493, 158.97455500840914, 150.1259112681928, 157.30358706207375, 160.5979410069489, 132.26593227072797, 152.77562981304905], [138.68858555784465, 155.72401439258195, 130.9195634604849, 164.28562240424654, 170.29051638672433, 139.7351254814477, 149.6251369865507, 161.88719987536257, 156.7102103479174, 135.7642840981997]]</t>
+          <t>[[147.68711990105024, 154.1608702059313, 150.11438828966982, 163.3491545802869, 155.42608430572844, 122.88615127290804, 148.12308458955792, 154.67068072714693, 151.1917169846608, 156.02100813442027], [159.8779975444673, 100.68775332362057, 162.8652578260208, 131.4788355672065, 156.2560621629521, 153.86663508485728, 147.89759324013917, 152.43536526834788, 174.02458161006243, 163.10753663795748], [159.82056010567388, 160.01000594783497, 163.1605690494393, 158.19744479878037, 145.56980118269308, 148.63414776013764, 143.63276304735638, 140.6983659276353, 140.68515415810884, 143.2214470137008], [142.55268731993388, 124.86185543304715, 158.88800996062557, 151.57040718734578, 167.22765665088872, 151.89697457766647, 147.92595724546806, 132.99210151466932, 158.1363375835545, 152.17013810101602], [146.50670794009332, 146.36119450492143, 156.04331242268123, 141.81778707262765, 133.12223760839427, 137.81951296462265, 160.40996079749883, 160.54005786888794, 170.3559001058529, 150.6535877057802]]</t>
         </is>
       </c>
     </row>
@@ -1191,14 +1191,14 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E15" t="b">
         <v>1</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>13.080000000000002</t>
+          <t>11.600000000000001</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>149.74603725750146</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1218,12 +1218,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>[[15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 13.0, 12.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 10.0, 12.0, 14.0, 13.0, 12.0, 12.0, 13.0, 10.0, 12.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 12.0, 12.0, 13.0, 12.0, 12.0, 12.0, 13.0, 12.0, 10.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0], [14.0, 14.0, 14.0, 16.0, 13.0, 14.0, 14.0, 14.0, 15.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 15.0, 10.0, 16.0], [13.0, 13.0, 12.0, 12.0, 12.0, 10.0, 12.0, 12.0, 12.0, 12.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0], [14.0, 14.0, 14.0, 15.0, 15.0, 15.0, 15.0, 14.0, 14.0, 10.0], [14.0, 12.0, 14.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [13.0, 10.0, 10.0, 13.0, 13.0, 12.0, 13.0, 13.0, 10.0, 13.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 16.0, 12.0, 12.0], [13.0, 13.0, 12.0, 12.0, 12.0, 10.0, 12.0, 12.0, 12.0, 12.0], [12.0, 14.0, 14.0, 16.0, 15.0, 14.0, 14.0, 16.0, 12.0, 13.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [10.0, 14.0, 12.0, 10.0, 12.0, 13.0, 13.0, 11.0, 12.0, 13.0], [14.0, 14.0, 12.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 14.0, 15.0, 12.0], [10.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 13.0, 10.0, 13.0], [10.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 13.0, 10.0, 13.0], [13.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0], [15.0, 15.0, 16.0, 13.0, 12.0, 14.0, 12.0, 14.0, 15.0, 14.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 13.0, 12.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 13.0, 13.0, 10.0], [16.0, 15.0, 12.0, 15.0, 14.0, 12.0, 14.0, 15.0, 15.0, 12.0], [16.0, 17.0, 17.0, 12.0, 14.0, 12.0, 12.0, 12.0, 14.0, 14.0]]</t>
+          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [15.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 12.0, 12.0, 15.0], [12.0, 13.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 13.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [13.0, 12.0, 13.0, 12.0, 12.0, 13.0, 13.0, 10.0, 12.0, 10.0]]</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>[[144.17921313809367, 166.35220031338423, 141.22171984560214, 145.3855231073463, 144.90639468917507, 147.27238158198946, 154.3238228233656, 157.98766645630056, 148.09405833559518, 153.9072787005084], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [144.30117409217885, 172.14729779439898, 142.40331771791733, 144.8190493875945, 163.38871241541744, 138.37602675777651, 145.19294131188033, 153.81985957820902, 145.16959966818743, 154.01228026780007], [138.5950961011988, 159.93270578904753, 145.68391375185405, 142.55305687560497, 151.24177471797898, 147.22991933251757, 155.39988729281495, 164.16938949754916, 152.11914188605147, 146.7053737467431], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.08136289158472, 160.49623667828618, 145.4987985222077, 141.43986050360445, 157.9292714840807, 150.70287516416076, 161.7472400092508, 153.70033433406178, 149.3168725093424, 131.7174068947811], [140.98959900595693, 162.99321023852437, 140.38278876177927, 149.78099912120337, 160.5570071317603, 144.82442509913304, 158.9031371435798, 149.6418701897537, 146.87052710478156, 148.68669519488822], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [143.74044209255126, 161.8910669627725, 140.14184098297, 143.18716101161152, 164.7169006038425, 143.71132625069296, 157.7794211144888, 151.17537657648876, 142.12314403742783, 155.16357935851443], [138.30012114995344, 155.1088900607881, 133.72029570587694, 158.18967098930176, 157.62917959053266, 151.43673509842776, 151.9013337518322, 150.7223156274309, 150.6337752637292, 155.98794175348755], [141.69795868289765, 160.13482094842018, 142.09099875306856, 156.48707979343624, 164.16136161273224, 140.3901466759431, 151.0647504374702, 156.86462005597053, 146.45522413259854, 144.28329789882335], [148.2009552205627, 165.08780994485082, 152.3765345193727, 138.4276094077305, 150.13832991527178, 141.69081770545236, 158.60760144277467, 154.45947443059003, 140.62344799303048, 154.01767841172455], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [118.5901570276999, 164.29670634824816, 134.45811446512846, 143.58298645856215, 160.18352050060176, 149.6417928032472, 160.83886619545365, 172.6790173465758, 142.53701433592758, 156.82208350991596], [150.03780013362507, 157.96129209120093, 130.14080628606516, 146.83174460066198, 152.76236912074017, 152.49716682824345, 165.95665916466442, 146.33538452449912, 151.00434467421977, 150.10269156744056], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [142.3175565041156, 157.07966095880727, 140.65243589292643, 146.39006015317656, 158.84130944106187, 143.41892367687444, 144.7012664163339, 170.44697427144183, 140.0615524164133, 159.72051926020941], [143.1609562614084, 152.080137850226, 146.5439872986877, 148.60330294578583, 159.51872916684874, 126.47997850559219, 147.3184981101908, 171.5368382288596, 156.186595413062, 152.20123521069925], [129.19861613587076, 165.00393668186683, 146.03750532321607, 138.08157977216175, 164.05997105719132, 159.2035061403781, 158.91703991686694, 160.55240623428136, 133.36065538477132, 149.21504234475606], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [138.64000650561, 151.86873674340978, 138.32456021370763, 161.7335877936576, 151.6848443573904, 136.28496273135173, 151.04700607126532, 160.00284567116378, 150.87959157390125, 163.1641173299031], [143.48850037839307, 155.4933055473404, 140.58853020416862, 159.85835524368773, 164.78432821434643, 126.41020852112312, 151.1747917241475, 163.2933719101649, 149.21610263858187, 149.32276460940685], [139.87991413377017, 161.49924507831477, 140.27796357727996, 154.66410937869347, 144.83977940148063, 142.96223798876127, 159.0317739406516, 158.2554937467503, 147.191755098787, 155.02798664687145], [148.3011917158448, 152.24135327016148, 138.24322771433754, 159.91265087419478, 157.75302017067696, 158.5786808938281, 147.92743000516273, 133.41406355031097, 153.4502590576199, 153.80838173922336], [142.47324381977754, 159.75391385863625, 139.89686476919496, 145.92151539200015, 165.15378792221145, 141.8884481702422, 147.56315632618478, 157.37789100557123, 152.37492819700643, 151.2265095305356], [151.77483014045058, 157.36992639649077, 145.1618572256677, 158.0463074247516, 156.45693331800123, 120.78821544824784, 148.9198164926133, 152.63719450795264, 157.35176560591893, 155.12341243126613], [122.56086781889486, 153.33018154775155, 138.73316026639344, 162.8616151383083, 160.47717131128687, 144.43501925639598, 153.8554606392985, 160.9905612202666, 141.2595350303938, 165.12668676237058], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [137.71140916636776, 159.04502682053018, 146.36776204231367, 137.6717594479347, 149.78346457725695, 149.8343764514719, 156.96511399072568, 165.1925738690632, 151.00844474590428, 150.0503278797923], [138.69691740865682, 161.36899676610903, 141.0319809300706, 142.05497300143577, 151.9853314935421, 150.1777877692477, 158.95250888203665, 158.09076104019178, 150.52377473544067, 150.74722696462945], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [148.2009552205627, 165.08780994485082, 152.3765345193727, 138.4276094077305, 150.13832991527178, 141.69081770545236, 158.60760144277467, 154.45947443059003, 140.62344799303048, 154.01767841172455], [138.68858555784465, 155.72401439258195, 130.9195634604849, 164.28562240424654, 170.29051638672433, 139.7351254814477, 149.6251369865507, 161.88719987536257, 156.7102103479174, 135.7642840981997], [146.96819049514585, 166.07135480306746, 149.9806344602439, 143.10317688672225, 153.82144256053363, 123.85796945663141, 162.44295163751056, 164.80514965374246, 141.46778093293213, 151.111608104831], [142.3175565041156, 157.07966095880727, 140.65243589292643, 146.39006015317656, 158.84130944106187, 143.41892367687444, 144.7012664163339, 170.44697427144183, 140.0615524164133, 159.72051926020941], [142.3175565041156, 157.07966095880727, 140.65243589292643, 146.39006015317656, 158.84130944106187, 143.41892367687444, 144.7012664163339, 170.44697427144183, 140.0615524164133, 159.72051926020941], [128.2589192837509, 166.08527098056226, 140.48593481787083, 156.75657747977493, 158.97455500840914, 150.1259112681928, 157.30358706207375, 160.5979410069489, 132.26593227072797, 152.77562981304905], [138.68858555784465, 155.72401439258195, 130.9195634604849, 164.28562240424654, 170.29051638672433, 139.7351254814477, 149.6251369865507, 161.88719987536257, 156.7102103479174, 135.7642840981997], [142.38507405557888, 171.73493977404362, 161.8371470067761, 131.83151517339343, 154.04495693839516, 147.54839841766926, 156.1370755170307, 147.74563929610653, 138.91488040381208, 151.45063240855475], [156.98103532867623, 161.0264333281865, 143.49649357216288, 147.7500803719328, 152.9105891271033, 143.27139593548364, 150.18685756618822, 161.52706406322142, 146.73054433794155, 139.74976536046415], [148.2009552205627, 165.08780994485082, 152.3765345193727, 138.4276094077305, 150.13832991527178, 141.69081770545236, 158.60760144277467, 154.45947443059003, 140.62344799303048, 154.01767841172455], [146.43558153704748, 170.88428268338927, 143.80721878884884, 141.2368943978099, 150.8486682203332, 138.096656740119, 165.18505563067094, 149.13284922728405, 146.27819900576614, 151.7248527600918], [143.43336569884465, 162.27639083571958, 151.8097645753834, 136.64783823820326, 147.15900502194785, 139.29224338683775, 141.99632632747594, 159.98622905009674, 158.28108176744016, 162.74801408941113]]</t>
+          <t>[[158.43510730480543, 161.38625728895036, 139.50799914532448, 150.15171674843418, 155.5768701800851, 152.2636517151059, 138.41402410546937, 155.4206183225901, 150.88778422094938, 140.60765864697333], [124.03285480088802, 156.9706535996761, 156.49802068276634, 153.90884126563586, 156.35365303592954, 159.8132886282515, 148.4062601526134, 153.21868756893195, 139.0379984681402, 155.39000078852774], [162.34384290121412, 152.48682424876634, 162.68878633168222, 159.22627277360777, 154.24170531510774, 145.43098874909305, 159.24123923268274, 125.31911611926084, 150.8650079433483, 122.7938685756444], [157.09933005828364, 156.50913162196633, 158.05549053938137, 156.92696380390694, 154.41738160021566, 153.05020722875776, 164.9966471362981, 125.5256103484539, 131.0160675479705, 145.6167611162228], [163.15071866102272, 172.63229004339323, 132.57925151358444, 124.9527099090768, 159.50885294667876, 156.5971657522344, 165.71505299527303, 129.938085366239, 123.4633807224316, 154.6311651032274]]</t>
         </is>
       </c>
     </row>
@@ -1244,14 +1244,14 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>13.127272727272729</t>
+          <t>14.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>149.95562622743154</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>[[15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 13.0, 12.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [16.0, 16.0, 15.0, 13.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [12.0, 10.0, 12.0, 14.0, 13.0, 12.0, 12.0, 13.0, 10.0, 12.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 12.0, 12.0, 13.0, 12.0, 12.0, 12.0, 13.0, 12.0, 10.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0], [14.0, 14.0, 14.0, 16.0, 13.0, 14.0, 14.0, 14.0, 15.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 15.0, 10.0, 16.0], [13.0, 13.0, 12.0, 12.0, 12.0, 10.0, 12.0, 12.0, 12.0, 12.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0], [14.0, 14.0, 14.0, 15.0, 15.0, 15.0, 15.0, 14.0, 14.0, 10.0], [14.0, 12.0, 14.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [13.0, 10.0, 10.0, 13.0, 13.0, 12.0, 13.0, 13.0, 10.0, 13.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 16.0, 12.0, 12.0], [13.0, 13.0, 12.0, 12.0, 12.0, 10.0, 12.0, 12.0, 12.0, 12.0], [12.0, 14.0, 14.0, 16.0, 15.0, 14.0, 14.0, 16.0, 12.0, 13.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0], [14.0, 12.0, 14.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [10.0, 14.0, 12.0, 10.0, 12.0, 13.0, 13.0, 11.0, 12.0, 13.0], [14.0, 14.0, 12.0, 16.0, 16.0, 14.0, 14.0, 15.0, 12.0, 13.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 14.0, 15.0, 12.0], [10.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 13.0, 10.0, 13.0], [10.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 13.0, 10.0, 13.0], [13.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [12.0, 12.0, 12.0, 13.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0], [15.0, 15.0, 16.0, 13.0, 12.0, 14.0, 12.0, 14.0, 15.0, 14.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 13.0, 12.0], [12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 13.0, 13.0, 10.0], [16.0, 15.0, 12.0, 15.0, 14.0, 12.0, 14.0, 15.0, 15.0, 12.0], [16.0, 17.0, 17.0, 12.0, 14.0, 12.0, 12.0, 12.0, 14.0, 14.0], [14.0, 14.0, 14.0, 15.0, 12.0, 14.0, 14.0, 14.0, 15.0, 14.0], [15.0, 16.0, 15.0, 14.0, 15.0, 10.0, 14.0, 12.0, 15.0, 14.0], [10.0, 15.0, 11.0, 10.0, 12.0, 13.0, 13.0, 11.0, 12.0, 13.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0]]</t>
+          <t>[[14.0, 12.0, 16.0, 13.0, 14.0, 14.0, 14.0, 15.0, 14.0, 14.0], [16.0, 15.0, 10.0, 15.0, 16.0, 15.0, 10.0, 10.0, 16.0, 17.0], [14.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0, 15.0, 14.0, 12.0], [14.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [14.0, 14.0, 15.0, 15.0, 14.0, 12.0, 14.0, 15.0, 15.0, 12.0]]</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>[[144.17921313809367, 166.35220031338423, 141.22171984560214, 145.3855231073463, 144.90639468917507, 147.27238158198946, 154.3238228233656, 157.98766645630056, 148.09405833559518, 153.9072787005084], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [144.30117409217885, 172.14729779439898, 142.40331771791733, 144.8190493875945, 163.38871241541744, 138.37602675777651, 145.19294131188033, 153.81985957820902, 145.16959966818743, 154.01228026780007], [138.5950961011988, 159.93270578904753, 145.68391375185405, 142.55305687560497, 151.24177471797898, 147.22991933251757, 155.39988729281495, 164.16938949754916, 152.11914188605147, 146.7053737467431], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.08136289158472, 160.49623667828618, 145.4987985222077, 141.43986050360445, 157.9292714840807, 150.70287516416076, 161.7472400092508, 153.70033433406178, 149.3168725093424, 131.7174068947811], [140.98959900595693, 162.99321023852437, 140.38278876177927, 149.78099912120337, 160.5570071317603, 144.82442509913304, 158.9031371435798, 149.6418701897537, 146.87052710478156, 148.68669519488822], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [143.74044209255126, 161.8910669627725, 140.14184098297, 143.18716101161152, 164.7169006038425, 143.71132625069296, 157.7794211144888, 151.17537657648876, 142.12314403742783, 155.16357935851443], [138.30012114995344, 155.1088900607881, 133.72029570587694, 158.18967098930176, 157.62917959053266, 151.43673509842776, 151.9013337518322, 150.7223156274309, 150.6337752637292, 155.98794175348755], [141.69795868289765, 160.13482094842018, 142.09099875306856, 156.48707979343624, 164.16136161273224, 140.3901466759431, 151.0647504374702, 156.86462005597053, 146.45522413259854, 144.28329789882335], [148.2009552205627, 165.08780994485082, 152.3765345193727, 138.4276094077305, 150.13832991527178, 141.69081770545236, 158.60760144277467, 154.45947443059003, 140.62344799303048, 154.01767841172455], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [118.5901570276999, 164.29670634824816, 134.45811446512846, 143.58298645856215, 160.18352050060176, 149.6417928032472, 160.83886619545365, 172.6790173465758, 142.53701433592758, 156.82208350991596], [150.03780013362507, 157.96129209120093, 130.14080628606516, 146.83174460066198, 152.76236912074017, 152.49716682824345, 165.95665916466442, 146.33538452449912, 151.00434467421977, 150.10269156744056], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [142.3175565041156, 157.07966095880727, 140.65243589292643, 146.39006015317656, 158.84130944106187, 143.41892367687444, 144.7012664163339, 170.44697427144183, 140.0615524164133, 159.72051926020941], [143.1609562614084, 152.080137850226, 146.5439872986877, 148.60330294578583, 159.51872916684874, 126.47997850559219, 147.3184981101908, 171.5368382288596, 156.186595413062, 152.20123521069925], [129.19861613587076, 165.00393668186683, 146.03750532321607, 138.08157977216175, 164.05997105719132, 159.2035061403781, 158.91703991686694, 160.55240623428136, 133.36065538477132, 149.21504234475606], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [138.64000650561, 151.86873674340978, 138.32456021370763, 161.7335877936576, 151.6848443573904, 136.28496273135173, 151.04700607126532, 160.00284567116378, 150.87959157390125, 163.1641173299031], [143.48850037839307, 155.4933055473404, 140.58853020416862, 159.85835524368773, 164.78432821434643, 126.41020852112312, 151.1747917241475, 163.2933719101649, 149.21610263858187, 149.32276460940685], [139.87991413377017, 161.49924507831477, 140.27796357727996, 154.66410937869347, 144.83977940148063, 142.96223798876127, 159.0317739406516, 158.2554937467503, 147.191755098787, 155.02798664687145], [148.3011917158448, 152.24135327016148, 138.24322771433754, 159.91265087419478, 157.75302017067696, 158.5786808938281, 147.92743000516273, 133.41406355031097, 153.4502590576199, 153.80838173922336], [142.47324381977754, 159.75391385863625, 139.89686476919496, 145.92151539200015, 165.15378792221145, 141.8884481702422, 147.56315632618478, 157.37789100557123, 152.37492819700643, 151.2265095305356], [151.77483014045058, 157.36992639649077, 145.1618572256677, 158.0463074247516, 156.45693331800123, 120.78821544824784, 148.9198164926133, 152.63719450795264, 157.35176560591893, 155.12341243126613], [122.56086781889486, 153.33018154775155, 138.73316026639344, 162.8616151383083, 160.47717131128687, 144.43501925639598, 153.8554606392985, 160.9905612202666, 141.2595350303938, 165.12668676237058], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [137.71140916636776, 159.04502682053018, 146.36776204231367, 137.6717594479347, 149.78346457725695, 149.8343764514719, 156.96511399072568, 165.1925738690632, 151.00844474590428, 150.0503278797923], [138.69691740865682, 161.36899676610903, 141.0319809300706, 142.05497300143577, 151.9853314935421, 150.1777877692477, 158.95250888203665, 158.09076104019178, 150.52377473544067, 150.74722696462945], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [148.2009552205627, 165.08780994485082, 152.3765345193727, 138.4276094077305, 150.13832991527178, 141.69081770545236, 158.60760144277467, 154.45947443059003, 140.62344799303048, 154.01767841172455], [138.68858555784465, 155.72401439258195, 130.9195634604849, 164.28562240424654, 170.29051638672433, 139.7351254814477, 149.6251369865507, 161.88719987536257, 156.7102103479174, 135.7642840981997], [146.96819049514585, 166.07135480306746, 149.9806344602439, 143.10317688672225, 153.82144256053363, 123.85796945663141, 162.44295163751056, 164.80514965374246, 141.46778093293213, 151.111608104831], [142.3175565041156, 157.07966095880727, 140.65243589292643, 146.39006015317656, 158.84130944106187, 143.41892367687444, 144.7012664163339, 170.44697427144183, 140.0615524164133, 159.72051926020941], [142.3175565041156, 157.07966095880727, 140.65243589292643, 146.39006015317656, 158.84130944106187, 143.41892367687444, 144.7012664163339, 170.44697427144183, 140.0615524164133, 159.72051926020941], [128.2589192837509, 166.08527098056226, 140.48593481787083, 156.75657747977493, 158.97455500840914, 150.1259112681928, 157.30358706207375, 160.5979410069489, 132.26593227072797, 152.77562981304905], [138.68858555784465, 155.72401439258195, 130.9195634604849, 164.28562240424654, 170.29051638672433, 139.7351254814477, 149.6251369865507, 161.88719987536257, 156.7102103479174, 135.7642840981997], [142.38507405557888, 171.73493977404362, 161.8371470067761, 131.83151517339343, 154.04495693839516, 147.54839841766926, 156.1370755170307, 147.74563929610653, 138.91488040381208, 151.45063240855475], [156.98103532867623, 161.0264333281865, 143.49649357216288, 147.7500803719328, 152.9105891271033, 143.27139593548364, 150.18685756618822, 161.52706406322142, 146.73054433794155, 139.74976536046415], [148.2009552205627, 165.08780994485082, 152.3765345193727, 138.4276094077305, 150.13832991527178, 141.69081770545236, 158.60760144277467, 154.45947443059003, 140.62344799303048, 154.01767841172455], [146.43558153704748, 170.88428268338927, 143.80721878884884, 141.2368943978099, 150.8486682203332, 138.096656740119, 165.18505563067094, 149.13284922728405, 146.27819900576614, 151.7248527600918], [143.43336569884465, 162.27639083571958, 151.8097645753834, 136.64783823820326, 147.15900502194785, 139.29224338683775, 141.99632632747594, 159.98622905009674, 158.28108176744016, 162.74801408941113], [145.6772690691106, 164.27136625986887, 153.71626124086856, 137.13760166479236, 151.62770040675156, 145.58189509907913, 160.80599310876534, 154.05614239996504, 138.32703673170516, 152.4289930104539], [142.7236736728817, 156.9369792484378, 142.75213877779524, 160.7502118309055, 146.89126560551605, 124.13712593698982, 150.90524604800063, 159.65501389770097, 154.8575994045452, 164.0210045685877], [146.99208349831986, 163.47125118861828, 145.20099684320311, 143.3285990297801, 162.2660310184385, 144.787374535079, 150.6060944633506, 144.6167930901506, 141.55571092379174, 160.8053244006288], [142.25652363847527, 159.5999057865361, 142.0543137300079, 146.48341002427597, 145.1374968505289, 144.9938790373216, 159.7528243366441, 155.84183321006986, 146.98291684943885, 160.52715552806197], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305]]</t>
+          <t>[[159.40360895365404, 144.42461818313467, 124.88124889389034, 145.7654979137987, 167.02188397806336, 152.360518357847, 149.7985670877622, 147.26331499078864, 152.53527624607312, 160.17572438634843], [155.55456881290942, 164.98160871229425, 129.56532718885603, 148.98448840946094, 147.02698374004967, 137.59828571129245, 137.72245481968702, 122.73065091058733, 205.00902413704915, 138.30855247537534], [157.76077548995116, 163.00469626095935, 142.28604525965213, 154.86060913895065, 145.24182156151693, 150.34992075658903, 162.88617810891878, 120.59422087590971, 157.8333905830988, 148.81260095581408], [164.50956148543244, 132.32382269012965, 160.46237736337616, 155.28027964354507, 151.79789895648543, 149.84605226027494, 172.8838264724944, 147.0447265902426, 138.6665852443041, 130.8151282850758], [145.1221187891643, 152.32628933243933, 143.02814906065353, 190.12339368308255, 136.20547666526505, 135.41539996065055, 129.70388698605478, 185.1162081239367, 137.6837180679096, 144.68394881077697]]</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1297,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>150.33535470194857</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1324,12 +1324,12 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>[[14.0, 12.0, 18.0, 13.0, 13.0, 16.0, 16.0, 13.0, 12.0, 13.0], [12.0, 14.0, 12.0, 15.0, 16.0, 15.0, 14.0, 17.0, 10.0, 15.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0]]</t>
+          <t>[[14.0, 14.0, 14.0, 14.0, 12.0, 14.0, 15.0, 15.0, 14.0, 14.0], [14.0, 14.0, 17.0, 16.0, 10.0, 14.0, 16.0, 12.0, 12.0, 15.0], [15.0, 14.0, 14.0, 16.0, 14.0, 12.0, 14.0, 14.0, 15.0, 12.0], [14.0, 14.0, 14.0, 15.0, 14.0, 12.0, 15.0, 14.0, 14.0, 14.0], [12.0, 15.0, 14.0, 13.0, 13.0, 17.0, 15.0, 12.0, 15.0, 14.0]]</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>[[122.90298383034093, 149.63155516998935, 134.46993810727835, 159.89335728696, 162.28086250482588, 148.98161651322775, 144.39738543509063, 159.40687339475582, 154.6699089950017, 166.99577775389028], [136.92673690300782, 152.41426340791796, 140.4650185749978, 158.73754740136758, 161.1705390839441, 139.46890032685872, 141.96264035510453, 162.68144119531928, 140.7078970655398, 169.0952746773031], [117.93802893800317, 156.66439786563146, 146.332446464142, 168.3638152630262, 161.42586482933453, 134.35863585847466, 144.36672865750734, 166.05241837220228, 139.2906934914242, 168.8372292516147], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959]]</t>
+          <t>[[159.99971389618864, 160.75315617355483, 137.75912252698865, 156.9842108120697, 156.75555432997143, 155.0551206681865, 154.79116482651253, 132.68298781914478, 141.32959736419767, 147.51963057454583], [159.54978113777545, 161.05791372335813, 150.29189694539204, 149.93017225400837, 118.19888786835756, 147.1876872630155, 158.69906087606293, 160.35776618037693, 141.81287313967928, 156.54421960333437], [155.26433137099596, 158.42279768662107, 141.90914720711876, 168.93105425128073, 157.29961167631816, 154.50031759859516, 164.8764495234053, 151.4199059203876, 109.64570693484389, 141.36093682179393], [154.0666100215715, 140.44220943861188, 153.19450942875136, 156.2157861318265, 151.0520237884125, 155.16416103198387, 158.74526966114337, 130.2245051745408, 150.7663301250524, 152.37529433009138], [126.12550005587862, 149.18625378573154, 148.9922809824132, 176.90499317056035, 174.68060114237954, 122.21291291784863, 137.44483336814739, 149.27798776146727, 135.73141122274205, 183.0734845841919]]</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>149.93583680327097</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1377,12 +1377,12 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>[[14.0, 12.0, 18.0, 13.0, 13.0, 16.0, 16.0, 13.0, 12.0, 13.0], [12.0, 14.0, 12.0, 15.0, 16.0, 15.0, 14.0, 17.0, 10.0, 15.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [12.0, 16.0, 13.0, 15.0, 15.0, 15.0, 15.0, 13.0, 14.0, 12.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 16.0, 12.0, 13.0], [15.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 12.0, 14.0, 12.0]]</t>
+          <t>[[15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 15.0, 14.0, 14.0, 12.0], [13.0, 12.0, 17.0, 12.0, 15.0, 12.0, 15.0, 15.0, 15.0, 14.0], [12.0, 14.0, 13.0, 14.0, 15.0, 14.0, 16.0, 15.0, 15.0, 12.0], [15.0, 15.0, 12.0, 14.0, 15.0, 13.0, 13.0, 15.0, 13.0, 15.0], [16.0, 15.0, 13.0, 16.0, 16.0, 10.0, 16.0, 10.0, 14.0, 14.0]]</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>[[122.90298383034093, 149.63155516998935, 134.46993810727835, 159.89335728696, 162.28086250482588, 148.98161651322775, 144.39738543509063, 159.40687339475582, 154.6699089950017, 166.99577775389028], [136.92673690300782, 152.41426340791796, 140.4650185749978, 158.73754740136758, 161.1705390839441, 139.46890032685872, 141.96264035510453, 162.68144119531928, 140.7078970655398, 169.0952746773031], [117.93802893800317, 156.66439786563146, 146.332446464142, 168.3638152630262, 161.42586482933453, 134.35863585847466, 144.36672865750734, 166.05241837220228, 139.2906934914242, 168.8372292516147], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [129.59691839843916, 166.45888525354428, 140.36119416175188, 155.77566134571126, 159.81438745202777, 151.08984582163438, 160.21527752707183, 160.53100384067415, 127.06364327592814, 152.72344191457776], [140.85063617275654, 153.2559596735747, 136.06232207532406, 159.15343723764363, 161.01009057633348, 149.28651253052465, 148.76925868477986, 156.50256025655176, 154.6754203974782, 144.06406138639366]]</t>
+          <t>[[152.86845308542559, 163.29745969019888, 158.15503468515845, 156.44220260522877, 156.35549360868438, 151.29816430367157, 148.9176016301535, 144.3211771739991, 150.99249869776298, 120.98217351107724], [154.1322262336486, 131.97655437050827, 142.0523596202264, 162.4374445914525, 158.34246860905415, 140.99789073606982, 160.22693903269777, 148.82082568760848, 149.62386248813533, 155.01968762195938], [140.70462554045372, 163.3879781111989, 142.87615749043414, 154.1301480715288, 153.48615497297533, 137.99391678582455, 142.62334537516057, 170.26306818086115, 155.54590874661156, 142.61895571631183], [130.8792537145822, 154.79970574332276, 132.88184317268195, 153.08251291076604, 149.4613601463185, 138.54880799821876, 147.75251145669202, 157.5079332551853, 150.48695371319064, 166.8699220871489], [164.9430652588061, 157.91305858571502, 164.33419702410342, 130.69668715602046, 169.85116540344833, 108.98976178379793, 143.20656282888146, 141.2382813093852, 158.42033341255924, 164.0371462286435]]</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>150.36302589913603</t>
+          <t>149.9263602914859</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1430,12 +1430,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>[[14.0, 12.0, 18.0, 13.0, 13.0, 16.0, 16.0, 13.0, 12.0, 13.0], [12.0, 14.0, 12.0, 15.0, 16.0, 15.0, 14.0, 17.0, 10.0, 15.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [12.0, 16.0, 13.0, 15.0, 15.0, 15.0, 15.0, 13.0, 14.0, 12.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 16.0, 12.0, 13.0], [15.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 12.0, 14.0, 12.0], [13.0, 12.0, 14.0, 16.0, 13.0, 14.0, 14.0, 16.0, 12.0, 16.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [12.0, 17.0, 12.0, 13.0, 14.0, 16.0, 15.0, 13.0, 14.0, 14.0], [16.0, 15.0, 15.0, 14.0, 14.0, 10.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0]]</t>
+          <t>[[16.0, 12.0, 14.0, 14.0, 14.0, 12.0, 14.0, 16.0, 13.0, 15.0], [14.0, 16.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0, 15.0, 12.0], [14.0, 15.0, 15.0, 14.0, 12.0, 12.0, 14.0, 15.0, 15.0, 14.0], [15.0, 14.0, 15.0, 12.0, 15.0, 14.0, 16.0, 14.0, 14.0, 11.0], [12.0, 15.0, 12.0, 15.0, 13.0, 15.0, 16.0, 12.0, 15.0, 15.0]]</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>[[122.90298383034093, 149.63155516998935, 134.46993810727835, 159.89335728696, 162.28086250482588, 148.98161651322775, 144.39738543509063, 159.40687339475582, 154.6699089950017, 166.99577775389028], [136.92673690300782, 152.41426340791796, 140.4650185749978, 158.73754740136758, 161.1705390839441, 139.46890032685872, 141.96264035510453, 162.68144119531928, 140.7078970655398, 169.0952746773031], [117.93802893800317, 156.66439786563146, 146.332446464142, 168.3638152630262, 161.42586482933453, 134.35863585847466, 144.36672865750734, 166.05241837220228, 139.2906934914242, 168.8372292516147], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [129.59691839843916, 166.45888525354428, 140.36119416175188, 155.77566134571126, 159.81438745202777, 151.08984582163438, 160.21527752707183, 160.53100384067415, 127.06364327592814, 152.72344191457776], [140.85063617275654, 153.2559596735747, 136.06232207532406, 159.15343723764363, 161.01009057633348, 149.28651253052465, 148.76925868477986, 156.50256025655176, 154.6754203974782, 144.06406138639366], [138.8652855740076, 163.2310172648969, 142.93884492251513, 150.66586196154768, 163.94517654724618, 141.69508828309387, 152.25723789162132, 159.69885558580114, 131.19476810822135, 159.13812285240948], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [151.18591401869966, 164.53591801468053, 146.12620232042943, 146.49236792115607, 145.01180344561874, 142.18838554532982, 165.64714172032012, 154.4700576636602, 138.958999413653, 149.01346892781294], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992]]</t>
+          <t>[[162.33109553876815, 146.05482325564716, 139.63209781817153, 154.68189381970416, 152.75896921478483, 125.27910542132304, 157.8034315571765, 159.21159631290712, 148.81376161877304, 157.06348443410508], [140.86259861033358, 139.29482106848008, 146.50226340061687, 173.74165210353866, 130.22319640639512, 152.717439974957, 160.1900167234797, 148.64104876567077, 166.51525499178393, 144.4601384829558], [158.30448913267475, 171.3857064761569, 144.75531116506176, 155.29702408261812, 151.9767880768871, 141.0328493636183, 158.27487596948154, 158.1572216519934, 136.3649951962508, 128.08099787661783], [159.22625077966165, 136.4643136157053, 143.88243210166726, 158.15752760159276, 153.16788469203823, 161.5136071668001, 148.9793961969441, 148.75736585033488, 141.54794958018076, 150.4730792981909], [122.02930591272015, 152.30745296911851, 132.30710366258188, 153.7872751572102, 157.40663779171396, 157.59429319796095, 149.49613719467462, 149.311627472209, 155.68282991148348, 153.81659591057567]]</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>150.36302589913603</t>
+          <t>150.06180365970653</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>[[14.0, 12.0, 18.0, 13.0, 13.0, 16.0, 16.0, 13.0, 12.0, 13.0], [12.0, 14.0, 12.0, 15.0, 16.0, 15.0, 14.0, 17.0, 10.0, 15.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [12.0, 16.0, 13.0, 15.0, 15.0, 15.0, 15.0, 13.0, 14.0, 12.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 16.0, 12.0, 13.0], [15.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 12.0, 14.0, 12.0], [13.0, 12.0, 14.0, 16.0, 13.0, 14.0, 14.0, 16.0, 12.0, 16.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [12.0, 17.0, 12.0, 13.0, 14.0, 16.0, 15.0, 13.0, 14.0, 14.0], [16.0, 15.0, 15.0, 14.0, 14.0, 10.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [13.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 15.0, 10.0, 15.0], [16.0, 17.0, 17.0, 12.0, 14.0, 12.0, 12.0, 12.0, 14.0, 14.0]]</t>
+          <t>[[15.0, 14.0, 15.0, 12.0, 14.0, 12.0, 14.0, 14.0, 15.0, 15.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 13.0, 12.0, 15.0, 15.0], [14.0, 15.0, 13.0, 16.0, 14.0, 14.0, 15.0, 15.0, 12.0, 12.0], [15.0, 16.0, 14.0, 15.0, 14.0, 12.0, 12.0, 12.0, 15.0, 15.0], [15.0, 13.0, 12.0, 12.0, 15.0, 15.0, 15.0, 15.0, 14.0, 14.0]]</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>[[122.90298383034093, 149.63155516998935, 134.46993810727835, 159.89335728696, 162.28086250482588, 148.98161651322775, 144.39738543509063, 159.40687339475582, 154.6699089950017, 166.99577775389028], [136.92673690300782, 152.41426340791796, 140.4650185749978, 158.73754740136758, 161.1705390839441, 139.46890032685872, 141.96264035510453, 162.68144119531928, 140.7078970655398, 169.0952746773031], [117.93802893800317, 156.66439786563146, 146.332446464142, 168.3638152630262, 161.42586482933453, 134.35863585847466, 144.36672865750734, 166.05241837220228, 139.2906934914242, 168.8372292516147], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [129.59691839843916, 166.45888525354428, 140.36119416175188, 155.77566134571126, 159.81438745202777, 151.08984582163438, 160.21527752707183, 160.53100384067415, 127.06364327592814, 152.72344191457776], [140.85063617275654, 153.2559596735747, 136.06232207532406, 159.15343723764363, 161.01009057633348, 149.28651253052465, 148.76925868477986, 156.50256025655176, 154.6754203974782, 144.06406138639366], [138.8652855740076, 163.2310172648969, 142.93884492251513, 150.66586196154768, 163.94517654724618, 141.69508828309387, 152.25723789162132, 159.69885558580114, 131.19476810822135, 159.13812285240948], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [151.18591401869966, 164.53591801468053, 146.12620232042943, 146.49236792115607, 145.01180344561874, 142.18838554532982, 165.64714172032012, 154.4700576636602, 138.958999413653, 149.01346892781294], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [145.00861869199673, 169.89012625702654, 150.94648190822008, 137.26531493208992, 151.4261003442735, 144.4535191089386, 150.1355639301699, 168.3443923167847, 136.80169785106128, 149.35844365079936], [144.48174753407125, 165.77100154921015, 143.67007428618058, 145.2365234213503, 144.72697193361753, 144.42898813900806, 154.28443888591346, 157.72899676382707, 145.36920682695333, 157.93230965122885], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.35159055962103, 166.8891315058427, 146.3623987630658, 150.69813365332797, 165.13197419074965, 136.91583982012213, 149.22514550882286, 157.90954418769113, 130.1827751692454, 157.96372563287196], [143.43336569884465, 162.27639083571958, 151.8097645753834, 136.64783823820326, 147.15900502194785, 139.29224338683775, 141.99632632747594, 159.98622905009674, 158.28108176744016, 162.74801408941113]]</t>
+          <t>[[167.68898385150007, 154.88203908272732, 160.03013597977494, 145.0780308423056, 123.7744764519587, 156.2807797119117, 153.58905492092882, 137.14160922906194, 156.7034770782459, 148.4616718429456], [155.49111940298724, 149.60532505114048, 161.39742223299243, 151.69572218016077, 153.93351576690034, 113.75039834161552, 162.87068040883696, 141.7952638347083, 159.87787384241767, 153.2129379296009], [152.6502324321323, 169.96059450949133, 142.6202121141058, 163.71655098622807, 137.20322234260587, 149.2214817613624, 149.96569957825514, 125.77652146409866, 151.7087631223402, 160.8069806807408], [163.25934543650604, 141.22329066462729, 164.29039808449335, 141.15525043213052, 145.28033450099133, 135.44451245122826, 137.9151754995478, 137.19138917330918, 167.58281341200848, 157.91619273862477], [146.78827167639955, 158.7074647354423, 146.21032312657914, 142.59194592530181, 154.1124383279714, 135.23867317202462, 151.5945641849898, 146.3135757131728, 154.24049537744833, 165.14295137844707]]</t>
         </is>
       </c>
     </row>
@@ -1509,7 +1509,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -1536,12 +1536,12 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>[[14.0, 12.0, 18.0, 13.0, 13.0, 16.0, 16.0, 13.0, 12.0, 13.0], [12.0, 14.0, 12.0, 15.0, 16.0, 15.0, 14.0, 17.0, 10.0, 15.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [12.0, 16.0, 13.0, 15.0, 15.0, 15.0, 15.0, 13.0, 14.0, 12.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 16.0, 12.0, 13.0], [15.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 12.0, 14.0, 12.0], [13.0, 12.0, 14.0, 16.0, 13.0, 14.0, 14.0, 16.0, 12.0, 16.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [12.0, 17.0, 12.0, 13.0, 14.0, 16.0, 15.0, 13.0, 14.0, 14.0], [16.0, 15.0, 15.0, 14.0, 14.0, 10.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [13.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 15.0, 10.0, 15.0], [16.0, 17.0, 17.0, 12.0, 14.0, 12.0, 12.0, 12.0, 14.0, 14.0], [14.0, 15.0, 15.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 17.0, 13.0, 14.0, 14.0, 12.0, 12.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 14.0, 14.0, 15.0]]</t>
+          <t>[[14.0, 16.0, 16.0, 14.0, 14.0, 10.0, 14.0, 14.0, 14.0, 14.0], [13.0, 11.0, 12.0, 14.0, 15.0, 14.0, 16.0, 15.0, 14.0, 16.0], [14.0, 15.0, 14.0, 14.0, 15.0, 13.0, 15.0, 12.0, 16.0, 12.0], [13.0, 11.0, 12.0, 17.0, 15.0, 16.0, 12.0, 15.0, 15.0, 14.0], [14.0, 14.0, 17.0, 14.0, 14.0, 15.0, 16.0, 12.0, 12.0, 12.0]]</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>[[122.90298383034093, 149.63155516998935, 134.46993810727835, 159.89335728696, 162.28086250482588, 148.98161651322775, 144.39738543509063, 159.40687339475582, 154.6699089950017, 166.99577775389028], [136.92673690300782, 152.41426340791796, 140.4650185749978, 158.73754740136758, 161.1705390839441, 139.46890032685872, 141.96264035510453, 162.68144119531928, 140.7078970655398, 169.0952746773031], [117.93802893800317, 156.66439786563146, 146.332446464142, 168.3638152630262, 161.42586482933453, 134.35863585847466, 144.36672865750734, 166.05241837220228, 139.2906934914242, 168.8372292516147], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [129.59691839843916, 166.45888525354428, 140.36119416175188, 155.77566134571126, 159.81438745202777, 151.08984582163438, 160.21527752707183, 160.53100384067415, 127.06364327592814, 152.72344191457776], [140.85063617275654, 153.2559596735747, 136.06232207532406, 159.15343723764363, 161.01009057633348, 149.28651253052465, 148.76925868477986, 156.50256025655176, 154.6754203974782, 144.06406138639366], [138.8652855740076, 163.2310172648969, 142.93884492251513, 150.66586196154768, 163.94517654724618, 141.69508828309387, 152.25723789162132, 159.69885558580114, 131.19476810822135, 159.13812285240948], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [151.18591401869966, 164.53591801468053, 146.12620232042943, 146.49236792115607, 145.01180344561874, 142.18838554532982, 165.64714172032012, 154.4700576636602, 138.958999413653, 149.01346892781294], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [145.00861869199673, 169.89012625702654, 150.94648190822008, 137.26531493208992, 151.4261003442735, 144.4535191089386, 150.1355639301699, 168.3443923167847, 136.80169785106128, 149.35844365079936], [144.48174753407125, 165.77100154921015, 143.67007428618058, 145.2365234213503, 144.72697193361753, 144.42898813900806, 154.28443888591346, 157.72899676382707, 145.36920682695333, 157.93230965122885], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.35159055962103, 166.8891315058427, 146.3623987630658, 150.69813365332797, 165.13197419074965, 136.91583982012213, 149.22514550882286, 157.90954418769113, 130.1827751692454, 157.96372563287196], [143.43336569884465, 162.27639083571958, 151.8097645753834, 136.64783823820326, 147.15900502194785, 139.29224338683775, 141.99632632747594, 159.98622905009674, 158.28108176744016, 162.74801408941113], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [142.25652363847527, 159.5999057865361, 142.0543137300079, 146.48341002427597, 145.1374968505289, 144.9938790373216, 159.7528243366441, 155.84183321006986, 146.98291684943885, 160.52715552806197], [141.26685426640162, 155.80429527279927, 143.88566867940946, 149.04282074550076, 158.49796293787327, 152.6871646979185, 138.616325116148, 165.64384663639626, 151.5560792244251, 146.62924141448818], [137.39806057977424, 148.58966617518814, 140.67400125052686, 159.98720654102195, 151.20648545278075, 134.57334417065363, 151.30659911431914, 162.4738491702741, 157.48089409974844, 159.94015243707338], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763]]</t>
+          <t>[[160.1778983785378, 151.4183244115257, 142.70812509179228, 161.51453299098574, 153.39128397050135, 150.2226064844456, 155.9314633823827, 167.0985785394233, 108.08729072716325, 153.0801550146028], [156.78565252884374, 163.9318641765121, 115.71047262589198, 156.60298733736067, 158.50908572842368, 154.94303520928003, 158.64495350608826, 134.91078900495359, 142.95876323954988, 160.6326556344565], [146.94506264509042, 152.17714935745082, 160.56735828106397, 159.84043135781906, 163.15183410180265, 160.71607870761434, 160.70304273439328, 137.77427899014188, 153.78615816638813, 107.968864649596], [138.61989630543692, 139.1622519292897, 155.08584823487246, 150.35401212786326, 158.5138646274837, 164.14344727274695, 144.95140864559744, 142.26177631122673, 155.06296653478933, 155.474787002054], [152.93750445084882, 170.74822021683195, 109.83282387028503, 161.2201030840335, 158.297522601774, 148.86319250836857, 168.39520021657222, 136.59633238695125, 164.75286958198748, 131.98649007370773]]</t>
         </is>
       </c>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>150.10811715617712</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1589,12 +1589,12 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>[[14.0, 12.0, 18.0, 13.0, 13.0, 16.0, 16.0, 13.0, 12.0, 13.0], [12.0, 14.0, 12.0, 15.0, 16.0, 15.0, 14.0, 17.0, 10.0, 15.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [12.0, 16.0, 13.0, 15.0, 15.0, 15.0, 15.0, 13.0, 14.0, 12.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 16.0, 12.0, 13.0], [15.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 12.0, 14.0, 12.0], [13.0, 12.0, 14.0, 16.0, 13.0, 14.0, 14.0, 16.0, 12.0, 16.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [12.0, 17.0, 12.0, 13.0, 14.0, 16.0, 15.0, 13.0, 14.0, 14.0], [16.0, 15.0, 15.0, 14.0, 14.0, 10.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [13.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 15.0, 10.0, 15.0], [16.0, 17.0, 17.0, 12.0, 14.0, 12.0, 12.0, 12.0, 14.0, 14.0], [14.0, 15.0, 15.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 17.0, 13.0, 14.0, 14.0, 12.0, 12.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 14.0, 14.0, 15.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [16.0, 15.0, 12.0, 15.0, 14.0, 12.0, 14.0, 15.0, 15.0, 12.0], [10.0, 12.0, 12.0, 13.0, 17.0, 15.0, 12.0, 19.0, 13.0, 17.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0]]</t>
+          <t>[[14.0, 14.0, 15.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0, 14.0], [13.0, 15.0, 15.0, 15.0, 14.0, 12.0, 12.0, 15.0, 15.0, 14.0], [14.0, 14.0, 15.0, 15.0, 12.0, 12.0, 15.0, 14.0, 14.0, 15.0], [16.0, 12.0, 15.0, 14.0, 13.0, 14.0, 15.0, 13.0, 14.0, 14.0], [13.0, 13.0, 14.0, 13.0, 15.0, 14.0, 14.0, 18.0, 14.0, 12.0]]</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>[[122.90298383034093, 149.63155516998935, 134.46993810727835, 159.89335728696, 162.28086250482588, 148.98161651322775, 144.39738543509063, 159.40687339475582, 154.6699089950017, 166.99577775389028], [136.92673690300782, 152.41426340791796, 140.4650185749978, 158.73754740136758, 161.1705390839441, 139.46890032685872, 141.96264035510453, 162.68144119531928, 140.7078970655398, 169.0952746773031], [117.93802893800317, 156.66439786563146, 146.332446464142, 168.3638152630262, 161.42586482933453, 134.35863585847466, 144.36672865750734, 166.05241837220228, 139.2906934914242, 168.8372292516147], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [129.59691839843916, 166.45888525354428, 140.36119416175188, 155.77566134571126, 159.81438745202777, 151.08984582163438, 160.21527752707183, 160.53100384067415, 127.06364327592814, 152.72344191457776], [140.85063617275654, 153.2559596735747, 136.06232207532406, 159.15343723764363, 161.01009057633348, 149.28651253052465, 148.76925868477986, 156.50256025655176, 154.6754203974782, 144.06406138639366], [138.8652855740076, 163.2310172648969, 142.93884492251513, 150.66586196154768, 163.94517654724618, 141.69508828309387, 152.25723789162132, 159.69885558580114, 131.19476810822135, 159.13812285240948], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [151.18591401869966, 164.53591801468053, 146.12620232042943, 146.49236792115607, 145.01180344561874, 142.18838554532982, 165.64714172032012, 154.4700576636602, 138.958999413653, 149.01346892781294], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [145.00861869199673, 169.89012625702654, 150.94648190822008, 137.26531493208992, 151.4261003442735, 144.4535191089386, 150.1355639301699, 168.3443923167847, 136.80169785106128, 149.35844365079936], [144.48174753407125, 165.77100154921015, 143.67007428618058, 145.2365234213503, 144.72697193361753, 144.42898813900806, 154.28443888591346, 157.72899676382707, 145.36920682695333, 157.93230965122885], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.35159055962103, 166.8891315058427, 146.3623987630658, 150.69813365332797, 165.13197419074965, 136.91583982012213, 149.22514550882286, 157.90954418769113, 130.1827751692454, 157.96372563287196], [143.43336569884465, 162.27639083571958, 151.8097645753834, 136.64783823820326, 147.15900502194785, 139.29224338683775, 141.99632632747594, 159.98622905009674, 158.28108176744016, 162.74801408941113], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [142.25652363847527, 159.5999057865361, 142.0543137300079, 146.48341002427597, 145.1374968505289, 144.9938790373216, 159.7528243366441, 155.84183321006986, 146.98291684943885, 160.52715552806197], [141.26685426640162, 155.80429527279927, 143.88566867940946, 149.04282074550076, 158.49796293787327, 152.6871646979185, 138.616325116148, 165.64384663639626, 151.5560792244251, 146.62924141448818], [137.39806057977424, 148.58966617518814, 140.67400125052686, 159.98720654102195, 151.20648545278075, 134.57334417065363, 151.30659911431914, 162.4738491702741, 157.48089409974844, 159.94015243707338], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [145.53652095954817, 163.32896093363726, 145.83922379407923, 139.59257291067934, 157.5803745697041, 142.30329659241025, 149.5140693517617, 150.27860689867248, 152.76200183233587, 156.89463114853217], [141.14757650090718, 159.77000143923615, 140.87122760860075, 159.86621289459802, 148.49973773854714, 118.46152402005815, 154.26502009369028, 160.0846209339392, 157.96858191571968, 162.69575584606412], [128.37183100025948, 168.31303965328658, 145.3544291690687, 160.20901607844743, 161.69201884997244, 140.06227788360673, 155.67390226891183, 162.61713237672632, 116.65156785148072, 164.6850438596003], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277]]</t>
+          <t>[[160.14239107124408, 154.38706245944343, 148.12313494644872, 152.16370615419964, 137.43442151841032, 152.39650803179393, 152.60927202595482, 142.70211477367985, 152.6563242120576, 151.01532379812826], [106.78546737722492, 161.06274135682443, 160.05566076143225, 155.14164951005668, 151.8889842656339, 161.6284197298115, 133.50074722763452, 157.26604711611537, 155.9277519393983, 160.37278970722863], [160.6588200755327, 120.50585352420602, 163.26276396983346, 151.19981685422897, 147.00422448393553, 139.14600415456985, 166.12190868934977, 160.15425832676812, 147.18804560194266, 148.38856331099342], [154.35090829109132, 119.37311071714852, 151.5859062420438, 143.23421113650295, 156.14079340801428, 155.52163430835105, 167.62456914580764, 144.90242064241568, 151.0367900068507, 159.85991509313465], [146.28737660302676, 142.21940403446814, 146.98595714612264, 133.34398363572438, 163.43692596559794, 129.3197749664453, 136.43302605569383, 176.2723699670176, 171.2943203803414, 145.29168308897576]]</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1615,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -1632,7 +1632,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>150.27550488640708</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1642,12 +1642,12 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>[[14.0, 12.0, 18.0, 13.0, 13.0, 16.0, 16.0, 13.0, 12.0, 13.0], [12.0, 14.0, 12.0, 15.0, 16.0, 15.0, 14.0, 17.0, 10.0, 15.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [12.0, 16.0, 13.0, 15.0, 15.0, 15.0, 15.0, 13.0, 14.0, 12.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 16.0, 12.0, 13.0], [15.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 12.0, 14.0, 12.0], [13.0, 12.0, 14.0, 16.0, 13.0, 14.0, 14.0, 16.0, 12.0, 16.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [12.0, 17.0, 12.0, 13.0, 14.0, 16.0, 15.0, 13.0, 14.0, 14.0], [16.0, 15.0, 15.0, 14.0, 14.0, 10.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [13.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 15.0, 10.0, 15.0], [16.0, 17.0, 17.0, 12.0, 14.0, 12.0, 12.0, 12.0, 14.0, 14.0], [14.0, 15.0, 15.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 17.0, 13.0, 14.0, 14.0, 12.0, 12.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 14.0, 14.0, 15.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [16.0, 15.0, 12.0, 15.0, 14.0, 12.0, 14.0, 15.0, 15.0, 12.0], [10.0, 12.0, 12.0, 13.0, 17.0, 15.0, 12.0, 19.0, 13.0, 17.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 12.0, 15.0, 15.0, 12.0, 14.0, 15.0, 15.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [12.0, 14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 16.0, 12.0, 15.0]]</t>
+          <t>[[15.0, 14.0, 15.0, 12.0, 15.0, 15.0, 13.0, 12.0, 14.0, 15.0], [15.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 14.0, 14.0, 12.0], [15.0, 16.0, 10.0, 16.0, 15.0, 16.0, 15.0, 10.0, 15.0, 12.0], [15.0, 15.0, 14.0, 14.0, 12.0, 12.0, 14.0, 16.0, 14.0, 14.0], [12.0, 15.0, 13.0, 15.0, 14.0, 15.0, 15.0, 15.0, 14.0, 12.0]]</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>[[122.90298383034093, 149.63155516998935, 134.46993810727835, 159.89335728696, 162.28086250482588, 148.98161651322775, 144.39738543509063, 159.40687339475582, 154.6699089950017, 166.99577775389028], [136.92673690300782, 152.41426340791796, 140.4650185749978, 158.73754740136758, 161.1705390839441, 139.46890032685872, 141.96264035510453, 162.68144119531928, 140.7078970655398, 169.0952746773031], [117.93802893800317, 156.66439786563146, 146.332446464142, 168.3638152630262, 161.42586482933453, 134.35863585847466, 144.36672865750734, 166.05241837220228, 139.2906934914242, 168.8372292516147], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [129.59691839843916, 166.45888525354428, 140.36119416175188, 155.77566134571126, 159.81438745202777, 151.08984582163438, 160.21527752707183, 160.53100384067415, 127.06364327592814, 152.72344191457776], [140.85063617275654, 153.2559596735747, 136.06232207532406, 159.15343723764363, 161.01009057633348, 149.28651253052465, 148.76925868477986, 156.50256025655176, 154.6754203974782, 144.06406138639366], [138.8652855740076, 163.2310172648969, 142.93884492251513, 150.66586196154768, 163.94517654724618, 141.69508828309387, 152.25723789162132, 159.69885558580114, 131.19476810822135, 159.13812285240948], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [151.18591401869966, 164.53591801468053, 146.12620232042943, 146.49236792115607, 145.01180344561874, 142.18838554532982, 165.64714172032012, 154.4700576636602, 138.958999413653, 149.01346892781294], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [145.00861869199673, 169.89012625702654, 150.94648190822008, 137.26531493208992, 151.4261003442735, 144.4535191089386, 150.1355639301699, 168.3443923167847, 136.80169785106128, 149.35844365079936], [144.48174753407125, 165.77100154921015, 143.67007428618058, 145.2365234213503, 144.72697193361753, 144.42898813900806, 154.28443888591346, 157.72899676382707, 145.36920682695333, 157.93230965122885], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.35159055962103, 166.8891315058427, 146.3623987630658, 150.69813365332797, 165.13197419074965, 136.91583982012213, 149.22514550882286, 157.90954418769113, 130.1827751692454, 157.96372563287196], [143.43336569884465, 162.27639083571958, 151.8097645753834, 136.64783823820326, 147.15900502194785, 139.29224338683775, 141.99632632747594, 159.98622905009674, 158.28108176744016, 162.74801408941113], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [142.25652363847527, 159.5999057865361, 142.0543137300079, 146.48341002427597, 145.1374968505289, 144.9938790373216, 159.7528243366441, 155.84183321006986, 146.98291684943885, 160.52715552806197], [141.26685426640162, 155.80429527279927, 143.88566867940946, 149.04282074550076, 158.49796293787327, 152.6871646979185, 138.616325116148, 165.64384663639626, 151.5560792244251, 146.62924141448818], [137.39806057977424, 148.58966617518814, 140.67400125052686, 159.98720654102195, 151.20648545278075, 134.57334417065363, 151.30659911431914, 162.4738491702741, 157.48089409974844, 159.94015243707338], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [145.53652095954817, 163.32896093363726, 145.83922379407923, 139.59257291067934, 157.5803745697041, 142.30329659241025, 149.5140693517617, 150.27860689867248, 152.76200183233587, 156.89463114853217], [141.14757650090718, 159.77000143923615, 140.87122760860075, 159.86621289459802, 148.49973773854714, 118.46152402005815, 154.26502009369028, 160.0846209339392, 157.96858191571968, 162.69575584606412], [128.37183100025948, 168.31303965328658, 145.3544291690687, 160.20901607844743, 161.69201884997244, 140.06227788360673, 155.67390226891183, 162.61713237672632, 116.65156785148072, 164.6850438596003], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [143.35893609363842, 162.52970249105087, 138.28225415037392, 145.2731801238887, 144.05906475069207, 148.0718842215696, 160.35204226743426, 158.20843931707492, 149.47815340911865, 154.0166021665192], [142.47324381977754, 159.75391385863625, 139.89686476919496, 145.92151539200015, 165.15378792221145, 141.8884481702422, 147.56315632618478, 157.37789100557123, 152.37492819700643, 151.2265095305356], [151.18591401869966, 164.53591801468053, 146.12620232042943, 146.49236792115607, 145.01180344561874, 142.18838554532982, 165.64714172032012, 154.4700576636602, 138.958999413653, 149.01346892781294], [145.97241670858784, 159.4535781753873, 142.4068495408466, 159.75930928992415, 147.97068820255, 126.87563086386061, 141.54999018159674, 159.32003925937462, 156.24548341981966, 164.07627334941307], [138.69691740865682, 161.36899676610903, 141.0319809300706, 142.05497300143577, 151.9853314935421, 150.1777877692477, 158.95250888203665, 158.09076104019178, 150.52377473544067, 150.74722696462945]]</t>
+          <t>[[161.30410962317063, 155.97036679426316, 156.34203247589267, 116.8864952589919, 156.27568380324183, 164.2533870818885, 148.24206534173618, 132.24906150903905, 165.49745989024356, 146.60959721289325], [157.5629142090821, 152.335032159214, 156.70414137249546, 153.78893594069984, 155.32412747742117, 133.64971673788034, 156.9614991178213, 160.57828993444346, 128.21277724439997, 148.51282479790308], [160.59221808323773, 147.63060115605873, 123.81006043253102, 157.41970645884658, 159.0454514861273, 173.0060342851978, 155.11881942366884, 129.97412109965313, 144.93497243006925, 152.09827413597037], [158.34350746275575, 149.6582030727827, 137.7532646210309, 150.49131986354968, 156.0531895301201, 137.98342742686083, 156.92171834576092, 150.22452445949182, 151.70536639264085, 151.89900505891234], [143.44111136867232, 160.3786547471762, 135.49465706888628, 154.75878902955705, 157.69110898814918, 166.04993740950974, 150.00885918228795, 137.13729552888594, 150.72734696074107, 146.16318082849952]]</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1668,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -1685,7 +1685,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>149.90775767046713</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1695,12 +1695,12 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>[[14.0, 12.0, 18.0, 13.0, 13.0, 16.0, 16.0, 13.0, 12.0, 13.0], [12.0, 14.0, 12.0, 15.0, 16.0, 15.0, 14.0, 17.0, 10.0, 15.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [12.0, 16.0, 13.0, 15.0, 15.0, 15.0, 15.0, 13.0, 14.0, 12.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 16.0, 12.0, 13.0], [15.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 12.0, 14.0, 12.0], [13.0, 12.0, 14.0, 16.0, 13.0, 14.0, 14.0, 16.0, 12.0, 16.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [12.0, 17.0, 12.0, 13.0, 14.0, 16.0, 15.0, 13.0, 14.0, 14.0], [16.0, 15.0, 15.0, 14.0, 14.0, 10.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [13.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 15.0, 10.0, 15.0], [16.0, 17.0, 17.0, 12.0, 14.0, 12.0, 12.0, 12.0, 14.0, 14.0], [14.0, 15.0, 15.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 17.0, 13.0, 14.0, 14.0, 12.0, 12.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 14.0, 14.0, 15.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [16.0, 15.0, 12.0, 15.0, 14.0, 12.0, 14.0, 15.0, 15.0, 12.0], [10.0, 12.0, 12.0, 13.0, 17.0, 15.0, 12.0, 19.0, 13.0, 17.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 12.0, 15.0, 15.0, 12.0, 14.0, 15.0, 15.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [12.0, 14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 16.0, 12.0, 15.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0]]</t>
+          <t>[[12.0, 14.0, 15.0, 15.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0], [14.0, 14.0, 16.0, 16.0, 14.0, 10.0, 14.0, 14.0, 14.0, 14.0], [15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0, 15.0], [12.0, 12.0, 18.0, 16.0, 14.0, 12.0, 15.0, 11.0, 16.0, 14.0], [12.0, 16.0, 16.0, 12.0, 16.0, 16.0, 16.0, 10.0, 10.0, 16.0]]</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>[[122.90298383034093, 149.63155516998935, 134.46993810727835, 159.89335728696, 162.28086250482588, 148.98161651322775, 144.39738543509063, 159.40687339475582, 154.6699089950017, 166.99577775389028], [136.92673690300782, 152.41426340791796, 140.4650185749978, 158.73754740136758, 161.1705390839441, 139.46890032685872, 141.96264035510453, 162.68144119531928, 140.7078970655398, 169.0952746773031], [117.93802893800317, 156.66439786563146, 146.332446464142, 168.3638152630262, 161.42586482933453, 134.35863585847466, 144.36672865750734, 166.05241837220228, 139.2906934914242, 168.8372292516147], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [129.59691839843916, 166.45888525354428, 140.36119416175188, 155.77566134571126, 159.81438745202777, 151.08984582163438, 160.21527752707183, 160.53100384067415, 127.06364327592814, 152.72344191457776], [140.85063617275654, 153.2559596735747, 136.06232207532406, 159.15343723764363, 161.01009057633348, 149.28651253052465, 148.76925868477986, 156.50256025655176, 154.6754203974782, 144.06406138639366], [138.8652855740076, 163.2310172648969, 142.93884492251513, 150.66586196154768, 163.94517654724618, 141.69508828309387, 152.25723789162132, 159.69885558580114, 131.19476810822135, 159.13812285240948], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [151.18591401869966, 164.53591801468053, 146.12620232042943, 146.49236792115607, 145.01180344561874, 142.18838554532982, 165.64714172032012, 154.4700576636602, 138.958999413653, 149.01346892781294], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [145.00861869199673, 169.89012625702654, 150.94648190822008, 137.26531493208992, 151.4261003442735, 144.4535191089386, 150.1355639301699, 168.3443923167847, 136.80169785106128, 149.35844365079936], [144.48174753407125, 165.77100154921015, 143.67007428618058, 145.2365234213503, 144.72697193361753, 144.42898813900806, 154.28443888591346, 157.72899676382707, 145.36920682695333, 157.93230965122885], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.35159055962103, 166.8891315058427, 146.3623987630658, 150.69813365332797, 165.13197419074965, 136.91583982012213, 149.22514550882286, 157.90954418769113, 130.1827751692454, 157.96372563287196], [143.43336569884465, 162.27639083571958, 151.8097645753834, 136.64783823820326, 147.15900502194785, 139.29224338683775, 141.99632632747594, 159.98622905009674, 158.28108176744016, 162.74801408941113], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [142.25652363847527, 159.5999057865361, 142.0543137300079, 146.48341002427597, 145.1374968505289, 144.9938790373216, 159.7528243366441, 155.84183321006986, 146.98291684943885, 160.52715552806197], [141.26685426640162, 155.80429527279927, 143.88566867940946, 149.04282074550076, 158.49796293787327, 152.6871646979185, 138.616325116148, 165.64384663639626, 151.5560792244251, 146.62924141448818], [137.39806057977424, 148.58966617518814, 140.67400125052686, 159.98720654102195, 151.20648545278075, 134.57334417065363, 151.30659911431914, 162.4738491702741, 157.48089409974844, 159.94015243707338], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [145.53652095954817, 163.32896093363726, 145.83922379407923, 139.59257291067934, 157.5803745697041, 142.30329659241025, 149.5140693517617, 150.27860689867248, 152.76200183233587, 156.89463114853217], [141.14757650090718, 159.77000143923615, 140.87122760860075, 159.86621289459802, 148.49973773854714, 118.46152402005815, 154.26502009369028, 160.0846209339392, 157.96858191571968, 162.69575584606412], [128.37183100025948, 168.31303965328658, 145.3544291690687, 160.20901607844743, 161.69201884997244, 140.06227788360673, 155.67390226891183, 162.61713237672632, 116.65156785148072, 164.6850438596003], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [143.35893609363842, 162.52970249105087, 138.28225415037392, 145.2731801238887, 144.05906475069207, 148.0718842215696, 160.35204226743426, 158.20843931707492, 149.47815340911865, 154.0166021665192], [142.47324381977754, 159.75391385863625, 139.89686476919496, 145.92151539200015, 165.15378792221145, 141.8884481702422, 147.56315632618478, 157.37789100557123, 152.37492819700643, 151.2265095305356], [151.18591401869966, 164.53591801468053, 146.12620232042943, 146.49236792115607, 145.01180344561874, 142.18838554532982, 165.64714172032012, 154.4700576636602, 138.958999413653, 149.01346892781294], [145.97241670858784, 159.4535781753873, 142.4068495408466, 159.75930928992415, 147.97068820255, 126.87563086386061, 141.54999018159674, 159.32003925937462, 156.24548341981966, 164.07627334941307], [138.69691740865682, 161.36899676610903, 141.0319809300706, 142.05497300143577, 151.9853314935421, 150.1777877692477, 158.95250888203665, 158.09076104019178, 150.52377473544067, 150.74722696462945], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [145.18619098277483, 158.099399886659, 141.65275875946995, 145.5376776347957, 160.17451813795222, 141.11272369244492, 158.52271796849632, 154.17722545010116, 153.2253082891169, 145.9417381895496], [143.0805372769047, 161.28337645928195, 141.75098649846507, 142.3715891042668, 162.97239903736323, 141.34306445929676, 156.9939742245395, 152.34450483926946, 149.82029047723458, 151.66953661473852], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959]]</t>
+          <t>[[143.47492532070575, 122.9146395062597, 155.7969086440705, 159.93301237172955, 150.0651258816084, 162.54346493209871, 159.49009167787227, 161.20061210581025, 140.1209633563099, 147.2012456743762], [153.8495328757091, 121.478931296217, 155.82556223164866, 151.73628448134022, 162.22266417391745, 150.2374051148492, 152.46516639785622, 154.40919837113393, 151.33449529403794, 150.0710187546509], [122.65163039380616, 153.27833209968594, 155.71054244761686, 157.43320504921707, 145.02013205617766, 156.98870118646337, 159.01547484194126, 153.6360516257647, 154.22132227725575, 145.6748670134318], [145.11474504898953, 150.6302074646412, 149.47288970296168, 148.5559647762762, 178.23829731579409, 144.80856121660648, 158.59207668272785, 126.51514184556495, 136.8948584597004, 164.80751647809822], [140.01014301585633, 168.79633000971674, 163.1363572469868, 134.55184155200163, 140.76873950956295, 166.17107534589158, 140.73000710868718, 130.00255002361064, 147.57308075225393, 150.0159925138667]]</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>149.80567235745792</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1748,12 +1748,12 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>[[14.0, 12.0, 18.0, 13.0, 13.0, 16.0, 16.0, 13.0, 12.0, 13.0], [12.0, 14.0, 12.0, 15.0, 16.0, 15.0, 14.0, 17.0, 10.0, 15.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [12.0, 16.0, 13.0, 15.0, 15.0, 15.0, 15.0, 13.0, 14.0, 12.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 16.0, 12.0, 13.0], [15.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 12.0, 14.0, 12.0], [13.0, 12.0, 14.0, 16.0, 13.0, 14.0, 14.0, 16.0, 12.0, 16.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [12.0, 17.0, 12.0, 13.0, 14.0, 16.0, 15.0, 13.0, 14.0, 14.0], [16.0, 15.0, 15.0, 14.0, 14.0, 10.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [13.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 15.0, 10.0, 15.0], [16.0, 17.0, 17.0, 12.0, 14.0, 12.0, 12.0, 12.0, 14.0, 14.0], [14.0, 15.0, 15.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 17.0, 13.0, 14.0, 14.0, 12.0, 12.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 14.0, 14.0, 15.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [16.0, 15.0, 12.0, 15.0, 14.0, 12.0, 14.0, 15.0, 15.0, 12.0], [10.0, 12.0, 12.0, 13.0, 17.0, 15.0, 12.0, 19.0, 13.0, 17.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 12.0, 15.0, 15.0, 12.0, 14.0, 15.0, 15.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [12.0, 14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 16.0, 12.0, 15.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [14.0, 14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 12.0], [13.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [12.0, 16.0, 10.0, 15.0, 15.0, 16.0, 16.0, 13.0, 15.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [17.0, 16.0, 17.0, 12.0, 14.0, 12.0, 12.0, 12.0, 14.0, 14.0]]</t>
+          <t>[[14.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0, 14.0, 14.0, 13.0], [12.0, 13.0, 15.0, 15.0, 14.0, 14.0, 15.0, 15.0, 15.0, 12.0], [14.0, 13.0, 16.0, 13.0, 14.0, 10.0, 15.0, 14.0, 16.0, 15.0], [14.0, 14.0, 14.0, 14.0, 14.0, 14.0, 15.0, 14.0, 15.0, 12.0], [15.0, 17.0, 13.0, 15.0, 16.0, 14.0, 12.0, 11.0, 15.0, 12.0]]</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>[[122.90298383034093, 149.63155516998935, 134.46993810727835, 159.89335728696, 162.28086250482588, 148.98161651322775, 144.39738543509063, 159.40687339475582, 154.6699089950017, 166.99577775389028], [136.92673690300782, 152.41426340791796, 140.4650185749978, 158.73754740136758, 161.1705390839441, 139.46890032685872, 141.96264035510453, 162.68144119531928, 140.7078970655398, 169.0952746773031], [117.93802893800317, 156.66439786563146, 146.332446464142, 168.3638152630262, 161.42586482933453, 134.35863585847466, 144.36672865750734, 166.05241837220228, 139.2906934914242, 168.8372292516147], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [129.59691839843916, 166.45888525354428, 140.36119416175188, 155.77566134571126, 159.81438745202777, 151.08984582163438, 160.21527752707183, 160.53100384067415, 127.06364327592814, 152.72344191457776], [140.85063617275654, 153.2559596735747, 136.06232207532406, 159.15343723764363, 161.01009057633348, 149.28651253052465, 148.76925868477986, 156.50256025655176, 154.6754203974782, 144.06406138639366], [138.8652855740076, 163.2310172648969, 142.93884492251513, 150.66586196154768, 163.94517654724618, 141.69508828309387, 152.25723789162132, 159.69885558580114, 131.19476810822135, 159.13812285240948], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [151.18591401869966, 164.53591801468053, 146.12620232042943, 146.49236792115607, 145.01180344561874, 142.18838554532982, 165.64714172032012, 154.4700576636602, 138.958999413653, 149.01346892781294], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [145.00861869199673, 169.89012625702654, 150.94648190822008, 137.26531493208992, 151.4261003442735, 144.4535191089386, 150.1355639301699, 168.3443923167847, 136.80169785106128, 149.35844365079936], [144.48174753407125, 165.77100154921015, 143.67007428618058, 145.2365234213503, 144.72697193361753, 144.42898813900806, 154.28443888591346, 157.72899676382707, 145.36920682695333, 157.93230965122885], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.35159055962103, 166.8891315058427, 146.3623987630658, 150.69813365332797, 165.13197419074965, 136.91583982012213, 149.22514550882286, 157.90954418769113, 130.1827751692454, 157.96372563287196], [143.43336569884465, 162.27639083571958, 151.8097645753834, 136.64783823820326, 147.15900502194785, 139.29224338683775, 141.99632632747594, 159.98622905009674, 158.28108176744016, 162.74801408941113], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [142.25652363847527, 159.5999057865361, 142.0543137300079, 146.48341002427597, 145.1374968505289, 144.9938790373216, 159.7528243366441, 155.84183321006986, 146.98291684943885, 160.52715552806197], [141.26685426640162, 155.80429527279927, 143.88566867940946, 149.04282074550076, 158.49796293787327, 152.6871646979185, 138.616325116148, 165.64384663639626, 151.5560792244251, 146.62924141448818], [137.39806057977424, 148.58966617518814, 140.67400125052686, 159.98720654102195, 151.20648545278075, 134.57334417065363, 151.30659911431914, 162.4738491702741, 157.48089409974844, 159.94015243707338], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [145.53652095954817, 163.32896093363726, 145.83922379407923, 139.59257291067934, 157.5803745697041, 142.30329659241025, 149.5140693517617, 150.27860689867248, 152.76200183233587, 156.89463114853217], [141.14757650090718, 159.77000143923615, 140.87122760860075, 159.86621289459802, 148.49973773854714, 118.46152402005815, 154.26502009369028, 160.0846209339392, 157.96858191571968, 162.69575584606412], [128.37183100025948, 168.31303965328658, 145.3544291690687, 160.20901607844743, 161.69201884997244, 140.06227788360673, 155.67390226891183, 162.61713237672632, 116.65156785148072, 164.6850438596003], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [143.35893609363842, 162.52970249105087, 138.28225415037392, 145.2731801238887, 144.05906475069207, 148.0718842215696, 160.35204226743426, 158.20843931707492, 149.47815340911865, 154.0166021665192], [142.47324381977754, 159.75391385863625, 139.89686476919496, 145.92151539200015, 165.15378792221145, 141.8884481702422, 147.56315632618478, 157.37789100557123, 152.37492819700643, 151.2265095305356], [151.18591401869966, 164.53591801468053, 146.12620232042943, 146.49236792115607, 145.01180344561874, 142.18838554532982, 165.64714172032012, 154.4700576636602, 138.958999413653, 149.01346892781294], [145.97241670858784, 159.4535781753873, 142.4068495408466, 159.75930928992415, 147.97068820255, 126.87563086386061, 141.54999018159674, 159.32003925937462, 156.24548341981966, 164.07627334941307], [138.69691740865682, 161.36899676610903, 141.0319809300706, 142.05497300143577, 151.9853314935421, 150.1777877692477, 158.95250888203665, 158.09076104019178, 150.52377473544067, 150.74722696462945], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [145.18619098277483, 158.099399886659, 141.65275875946995, 145.5376776347957, 160.17451813795222, 141.11272369244492, 158.52271796849632, 154.17722545010116, 153.2253082891169, 145.9417381895496], [143.0805372769047, 161.28337645928195, 141.75098649846507, 142.3715891042668, 162.97239903736323, 141.34306445929676, 156.9939742245395, 152.34450483926946, 149.82029047723458, 151.66953661473852], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [146.64317479735988, 161.5337112728855, 150.47215491636206, 145.53368330088531, 154.55868909231992, 141.1877137989166, 163.56305914137073, 153.07863709074726, 141.11139776641875, 145.94803781409468], [144.60010629456147, 169.43951929689237, 142.4570306270456, 145.33699899674997, 161.25303423071955, 145.5055759990721, 151.06696141231535, 155.54480781204182, 132.65222904761524, 155.77399527434713], [123.4791607988294, 161.33603491669362, 131.02644054355991, 144.7481620312516, 149.7863160951474, 161.6152063451183, 173.48438400022587, 153.54428119663942, 149.78389164114128, 154.82638142275377], [151.77483014045058, 157.36992639649077, 145.1618572256677, 158.0463074247516, 156.45693331800123, 120.78821544824784, 148.9198164926133, 152.63719450795264, 157.35176560591893, 155.12341243126613], [143.74384306196606, 164.1252770443115, 151.80434598827767, 136.06238542529633, 148.60885914109565, 136.33344822627134, 148.02587785777536, 158.63036197759527, 153.8425704067714, 162.4532898619999]]</t>
+          <t>[[142.8827387225483, 157.07730219285753, 166.52475596297967, 158.50922368191732, 161.7443112201323, 132.57554480836663, 156.69246160007722, 163.36966790559944, 139.25766437336162, 124.99658852352063], [162.4431997514302, 134.88741924402595, 166.09968246600016, 153.16439730270778, 150.15696600045658, 151.4380756572095, 158.85041642702933, 142.37726840156674, 159.25940889247084, 124.95342484846341], [154.3505094436592, 163.19920181102208, 150.16930923563066, 146.73061995061323, 157.8675978328568, 113.36841971500351, 153.56476726298393, 157.75586470007323, 150.82168206364213, 155.80228697587572], [148.04738704766402, 163.31017866599385, 150.2392865261676, 160.123871579108, 157.0686784872406, 153.51742173736503, 144.96989432150085, 113.8362059066002, 158.217221830998, 154.30011288872248], [149.0921496392564, 133.02233215227207, 157.79094306017956, 198.7938297064862, 135.27936341463726, 175.0029447619666, 139.74464021847604, 114.94203930889667, 135.17819892420863, 136.91614072107464]]</t>
         </is>
       </c>
     </row>
@@ -1774,7 +1774,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1801,24 +1801,24 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>[[14.0, 12.0, 18.0, 13.0, 13.0, 16.0, 16.0, 13.0, 12.0, 13.0], [12.0, 14.0, 12.0, 15.0, 16.0, 15.0, 14.0, 17.0, 10.0, 15.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [12.0, 16.0, 13.0, 15.0, 15.0, 15.0, 15.0, 13.0, 14.0, 12.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 16.0, 12.0, 13.0], [15.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 12.0, 14.0, 12.0], [13.0, 12.0, 14.0, 16.0, 13.0, 14.0, 14.0, 16.0, 12.0, 16.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [12.0, 17.0, 12.0, 13.0, 14.0, 16.0, 15.0, 13.0, 14.0, 14.0], [16.0, 15.0, 15.0, 14.0, 14.0, 10.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [13.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 15.0, 10.0, 15.0], [16.0, 17.0, 17.0, 12.0, 14.0, 12.0, 12.0, 12.0, 14.0, 14.0], [14.0, 15.0, 15.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 17.0, 13.0, 14.0, 14.0, 12.0, 12.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 14.0, 14.0, 15.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [16.0, 15.0, 12.0, 15.0, 14.0, 12.0, 14.0, 15.0, 15.0, 12.0], [10.0, 12.0, 12.0, 13.0, 17.0, 15.0, 12.0, 19.0, 13.0, 17.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 12.0, 15.0, 15.0, 12.0, 14.0, 15.0, 15.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [12.0, 14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 16.0, 12.0, 15.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [14.0, 14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 12.0], [13.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [12.0, 16.0, 10.0, 15.0, 15.0, 16.0, 16.0, 13.0, 15.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [17.0, 16.0, 17.0, 12.0, 14.0, 12.0, 12.0, 12.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 14.0, 15.0, 12.0], [15.0, 13.0, 16.0, 13.0, 15.0, 14.0, 12.0, 15.0, 15.0, 12.0], [14.0, 15.0, 15.0, 14.0, 15.0, 12.0, 14.0, 12.0, 15.0, 14.0]]</t>
+          <t>[[12.0, 15.0, 15.0, 14.0, 14.0, 14.0, 14.0, 14.0, 12.0, 16.0], [14.0, 14.0, 13.0, 16.0, 15.0, 14.0, 13.0, 12.0, 14.0, 15.0], [15.0, 14.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [12.0, 13.0, 16.0, 14.0, 14.0, 14.0, 14.0, 15.0, 14.0, 14.0], [14.0, 12.0, 15.0, 12.0, 15.0, 14.0, 14.0, 15.0, 15.0, 14.0]]</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>[[122.90298383034093, 149.63155516998935, 134.46993810727835, 159.89335728696, 162.28086250482588, 148.98161651322775, 144.39738543509063, 159.40687339475582, 154.6699089950017, 166.99577775389028], [136.92673690300782, 152.41426340791796, 140.4650185749978, 158.73754740136758, 161.1705390839441, 139.46890032685872, 141.96264035510453, 162.68144119531928, 140.7078970655398, 169.0952746773031], [117.93802893800317, 156.66439786563146, 146.332446464142, 168.3638152630262, 161.42586482933453, 134.35863585847466, 144.36672865750734, 166.05241837220228, 139.2906934914242, 168.8372292516147], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [129.59691839843916, 166.45888525354428, 140.36119416175188, 155.77566134571126, 159.81438745202777, 151.08984582163438, 160.21527752707183, 160.53100384067415, 127.06364327592814, 152.72344191457776], [140.85063617275654, 153.2559596735747, 136.06232207532406, 159.15343723764363, 161.01009057633348, 149.28651253052465, 148.76925868477986, 156.50256025655176, 154.6754203974782, 144.06406138639366], [138.8652855740076, 163.2310172648969, 142.93884492251513, 150.66586196154768, 163.94517654724618, 141.69508828309387, 152.25723789162132, 159.69885558580114, 131.19476810822135, 159.13812285240948], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [151.18591401869966, 164.53591801468053, 146.12620232042943, 146.49236792115607, 145.01180344561874, 142.18838554532982, 165.64714172032012, 154.4700576636602, 138.958999413653, 149.01346892781294], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [145.00861869199673, 169.89012625702654, 150.94648190822008, 137.26531493208992, 151.4261003442735, 144.4535191089386, 150.1355639301699, 168.3443923167847, 136.80169785106128, 149.35844365079936], [144.48174753407125, 165.77100154921015, 143.67007428618058, 145.2365234213503, 144.72697193361753, 144.42898813900806, 154.28443888591346, 157.72899676382707, 145.36920682695333, 157.93230965122885], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.35159055962103, 166.8891315058427, 146.3623987630658, 150.69813365332797, 165.13197419074965, 136.91583982012213, 149.22514550882286, 157.90954418769113, 130.1827751692454, 157.96372563287196], [143.43336569884465, 162.27639083571958, 151.8097645753834, 136.64783823820326, 147.15900502194785, 139.29224338683775, 141.99632632747594, 159.98622905009674, 158.28108176744016, 162.74801408941113], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [142.25652363847527, 159.5999057865361, 142.0543137300079, 146.48341002427597, 145.1374968505289, 144.9938790373216, 159.7528243366441, 155.84183321006986, 146.98291684943885, 160.52715552806197], [141.26685426640162, 155.80429527279927, 143.88566867940946, 149.04282074550076, 158.49796293787327, 152.6871646979185, 138.616325116148, 165.64384663639626, 151.5560792244251, 146.62924141448818], [137.39806057977424, 148.58966617518814, 140.67400125052686, 159.98720654102195, 151.20648545278075, 134.57334417065363, 151.30659911431914, 162.4738491702741, 157.48089409974844, 159.94015243707338], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [145.53652095954817, 163.32896093363726, 145.83922379407923, 139.59257291067934, 157.5803745697041, 142.30329659241025, 149.5140693517617, 150.27860689867248, 152.76200183233587, 156.89463114853217], [141.14757650090718, 159.77000143923615, 140.87122760860075, 159.86621289459802, 148.49973773854714, 118.46152402005815, 154.26502009369028, 160.0846209339392, 157.96858191571968, 162.69575584606412], [128.37183100025948, 168.31303965328658, 145.3544291690687, 160.20901607844743, 161.69201884997244, 140.06227788360673, 155.67390226891183, 162.61713237672632, 116.65156785148072, 164.6850438596003], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [143.35893609363842, 162.52970249105087, 138.28225415037392, 145.2731801238887, 144.05906475069207, 148.0718842215696, 160.35204226743426, 158.20843931707492, 149.47815340911865, 154.0166021665192], [142.47324381977754, 159.75391385863625, 139.89686476919496, 145.92151539200015, 165.15378792221145, 141.8884481702422, 147.56315632618478, 157.37789100557123, 152.37492819700643, 151.2265095305356], [151.18591401869966, 164.53591801468053, 146.12620232042943, 146.49236792115607, 145.01180344561874, 142.18838554532982, 165.64714172032012, 154.4700576636602, 138.958999413653, 149.01346892781294], [145.97241670858784, 159.4535781753873, 142.4068495408466, 159.75930928992415, 147.97068820255, 126.87563086386061, 141.54999018159674, 159.32003925937462, 156.24548341981966, 164.07627334941307], [138.69691740865682, 161.36899676610903, 141.0319809300706, 142.05497300143577, 151.9853314935421, 150.1777877692477, 158.95250888203665, 158.09076104019178, 150.52377473544067, 150.74722696462945], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [145.18619098277483, 158.099399886659, 141.65275875946995, 145.5376776347957, 160.17451813795222, 141.11272369244492, 158.52271796849632, 154.17722545010116, 153.2253082891169, 145.9417381895496], [143.0805372769047, 161.28337645928195, 141.75098649846507, 142.3715891042668, 162.97239903736323, 141.34306445929676, 156.9939742245395, 152.34450483926946, 149.82029047723458, 151.66953661473852], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [146.64317479735988, 161.5337112728855, 150.47215491636206, 145.53368330088531, 154.55868909231992, 141.1877137989166, 163.56305914137073, 153.07863709074726, 141.11139776641875, 145.94803781409468], [144.60010629456147, 169.43951929689237, 142.4570306270456, 145.33699899674997, 161.25303423071955, 145.5055759990721, 151.06696141231535, 155.54480781204182, 132.65222904761524, 155.77399527434713], [123.4791607988294, 161.33603491669362, 131.02644054355991, 144.7481620312516, 149.7863160951474, 161.6152063451183, 173.48438400022587, 153.54428119663942, 149.78389164114128, 154.82638142275377], [151.77483014045058, 157.36992639649077, 145.1618572256677, 158.0463074247516, 156.45693331800123, 120.78821544824784, 148.9198164926133, 152.63719450795264, 157.35176560591893, 155.12341243126613], [143.74384306196606, 164.1252770443115, 151.80434598827767, 136.06238542529633, 148.60885914109565, 136.33344822627134, 148.02587785777536, 158.63036197759527, 153.8425704067714, 162.4532898619999], [140.9692473082241, 158.83708354814627, 142.50648445339854, 150.6469290609464, 159.43914344419983, 143.88423257680765, 151.95366940862746, 162.83914933877537, 153.26970678446094, 139.28461306777402], [143.35893609363842, 162.52970249105087, 138.28225415037392, 145.2731801238887, 144.05906475069207, 148.0718842215696, 160.35204226743426, 158.20843931707492, 149.47815340911865, 154.0166021665192], [138.5950961011988, 159.93270578904753, 145.68391375185405, 142.55305687560497, 151.24177471797898, 147.22991933251757, 155.39988729281495, 164.16938949754916, 152.11914188605147, 146.7053737467431], [140.43119284335623, 164.15110042573548, 136.54600560664568, 136.53489502042416, 156.16264309799706, 145.90220196994045, 146.3435165551005, 162.685726080723, 156.44291786101934, 158.43005953041867], [142.93905828606603, 156.17886135868338, 140.83900194594102, 159.81222040273823, 150.47350943243492, 126.48838000412711, 152.21387729630555, 159.85812911026164, 152.13961889080628, 162.68760226399635]]</t>
+          <t>[[150.99980972164937, 161.22756029964512, 158.6667277143557, 159.50803187551162, 158.77322556767473, 160.8989908161002, 152.15103177048587, 140.4416898022828, 105.22708918554834, 155.73610223810695], [148.61568661936766, 135.4047954355038, 151.36733886069584, 158.57748587647265, 164.66655313788578, 140.72110355655286, 155.3758178187173, 139.5520459884772, 151.44698555427112, 157.9024461434163], [161.07726040708732, 151.92559526792633, 114.70953781399258, 152.1336810374921, 164.64091287448065, 155.05908270602697, 159.1668898322144, 149.0320796621414, 140.45486140067882, 155.43035798931993], [156.81940624046706, 149.04009660787463, 154.85558024619397, 147.8086093601166, 153.36963681120872, 157.87887081256824, 152.71009419031589, 157.35810546508117, 121.48780108750273, 152.3020581700316], [156.32786561990198, 154.31190076693127, 143.84342175950397, 103.0550447689633, 160.79457902678493, 152.9381494150279, 144.90230707087252, 163.1537049924905, 164.5172921389378, 159.7859934319463]]</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>homoSelfPlay.csv</t>
+          <t>mixedSelfPlay.csv</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>[4, 3]</t>
+          <t>['J', 3]</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1830,11 +1830,11 @@
         <v>1</v>
       </c>
       <c r="E27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>14.000000000000004</t>
+          <t>NAN</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>150.36302589913606</t>
+          <t>118.01748834382616</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1854,12 +1854,12 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>[[14.0, 12.0, 18.0, 13.0, 13.0, 16.0, 16.0, 13.0, 12.0, 13.0], [12.0, 14.0, 12.0, 15.0, 16.0, 15.0, 14.0, 17.0, 10.0, 15.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [12.0, 16.0, 13.0, 15.0, 15.0, 15.0, 15.0, 13.0, 14.0, 12.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 15.0, 15.0, 16.0, 12.0, 14.0, 12.0, 14.0, 12.0], [12.0, 14.0, 12.0, 17.0, 16.0, 14.0, 14.0, 16.0, 12.0, 13.0], [15.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 12.0, 14.0, 12.0], [13.0, 12.0, 14.0, 16.0, 13.0, 14.0, 14.0, 16.0, 12.0, 16.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [12.0, 17.0, 12.0, 13.0, 14.0, 16.0, 15.0, 13.0, 14.0, 14.0], [16.0, 15.0, 15.0, 14.0, 14.0, 10.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 15.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [13.0, 15.0, 17.0, 14.0, 15.0, 14.0, 12.0, 15.0, 10.0, 15.0], [16.0, 17.0, 17.0, 12.0, 14.0, 12.0, 12.0, 12.0, 14.0, 14.0], [14.0, 15.0, 15.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0, 14.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 17.0, 13.0, 14.0, 14.0, 12.0, 12.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 12.0, 12.0, 14.0, 14.0, 14.0, 15.0], [16.0, 11.0, 15.0, 15.0, 17.0, 13.0, 14.0, 10.0, 17.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [16.0, 15.0, 12.0, 15.0, 14.0, 12.0, 14.0, 15.0, 15.0, 12.0], [10.0, 12.0, 12.0, 13.0, 17.0, 15.0, 12.0, 19.0, 13.0, 17.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 14.0, 12.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 12.0, 15.0, 15.0, 12.0, 14.0, 15.0, 15.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [12.0, 14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 16.0, 12.0, 15.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [15.0, 15.0, 16.0, 12.0, 14.0, 14.0, 12.0, 14.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [14.0, 14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 15.0, 12.0], [13.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [12.0, 16.0, 10.0, 15.0, 15.0, 16.0, 16.0, 13.0, 15.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 15.0, 14.0, 12.0], [17.0, 16.0, 17.0, 12.0, 14.0, 12.0, 12.0, 12.0, 14.0, 14.0], [15.0, 15.0, 14.0, 15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 12.0], [14.0, 14.0, 12.0, 15.0, 15.0, 14.0, 14.0, 15.0, 12.0, 15.0], [14.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0, 14.0, 15.0, 12.0], [15.0, 13.0, 16.0, 13.0, 15.0, 14.0, 12.0, 15.0, 15.0, 12.0], [14.0, 15.0, 15.0, 14.0, 15.0, 12.0, 14.0, 12.0, 15.0, 14.0], [15.0, 16.0, 19.0, 10.0, 14.0, 14.0, 10.0, 14.0, 14.0, 14.0], [11.0, 13.0, 21.0, 16.0, 15.0, 13.0, 10.0, 10.0, 16.0, 15.0], [12.0, 15.0, 15.0, 15.0, 15.0, 12.0, 14.0, 15.0, 12.0, 15.0], [15.0, 14.0, 14.0, 14.0, 14.0, 14.0, 14.0, 14.0, 15.0, 12.0], [15.0, 15.0, 14.0, 15.0, 14.0, 12.0, 14.0, 14.0, 15.0, 12.0]]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>[[122.90298383034093, 149.63155516998935, 134.46993810727835, 159.89335728696, 162.28086250482588, 148.98161651322775, 144.39738543509063, 159.40687339475582, 154.6699089950017, 166.99577775389028], [136.92673690300782, 152.41426340791796, 140.4650185749978, 158.73754740136758, 161.1705390839441, 139.46890032685872, 141.96264035510453, 162.68144119531928, 140.7078970655398, 169.0952746773031], [117.93802893800317, 156.66439786563146, 146.332446464142, 168.3638152630262, 161.42586482933453, 134.35863585847466, 144.36672865750734, 166.05241837220228, 139.2906934914242, 168.8372292516147], [139.05348361397182, 153.0353630212329, 134.6451628890464, 167.1464893490191, 169.42438131443626, 136.07777621399072, 147.6848803775167, 167.75631124355988, 150.7889562734787, 138.01745469510809], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [151.5766827987286, 160.89247202945913, 158.49720917823913, 141.79221891691344, 156.80336063699386, 147.23868565932864, 155.844039006083, 151.69107425534176, 146.68518045128104, 132.60933605899186], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [134.18785570876, 147.85124910190177, 135.53065679465996, 164.17728395666614, 170.78268551478783, 136.81694356997872, 147.71332527947666, 167.16943946663048, 150.72744357413927, 148.67337602435964], [129.59691839843916, 166.45888525354428, 140.36119416175188, 155.77566134571126, 159.81438745202777, 151.08984582163438, 160.21527752707183, 160.53100384067415, 127.06364327592814, 152.72344191457776], [140.85063617275654, 153.2559596735747, 136.06232207532406, 159.15343723764363, 161.01009057633348, 149.28651253052465, 148.76925868477986, 156.50256025655176, 154.6754203974782, 144.06406138639366], [138.8652855740076, 163.2310172648969, 142.93884492251513, 150.66586196154768, 163.94517654724618, 141.69508828309387, 152.25723789162132, 159.69885558580114, 131.19476810822135, 159.13812285240948], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [151.18591401869966, 164.53591801468053, 146.12620232042943, 146.49236792115607, 145.01180344561874, 142.18838554532982, 165.64714172032012, 154.4700576636602, 138.958999413653, 149.01346892781294], [143.9349213959267, 162.05816996185024, 146.3655167640061, 143.25790112607598, 151.71457518331667, 146.85372952983502, 157.71149439282328, 155.1102287473242, 143.76338737380317, 152.8603345163992], [145.00861869199673, 169.89012625702654, 150.94648190822008, 137.26531493208992, 151.4261003442735, 144.4535191089386, 150.1355639301699, 168.3443923167847, 136.80169785106128, 149.35844365079936], [144.48174753407125, 165.77100154921015, 143.67007428618058, 145.2365234213503, 144.72697193361753, 144.42898813900806, 154.28443888591346, 157.72899676382707, 145.36920682695333, 157.93230965122885], [144.9903215329925, 159.06180259754143, 141.49870466288425, 141.8177823134863, 151.00551670424565, 140.37499991466723, 156.97135988708263, 160.47276208205406, 152.03388651988894, 155.4031227765176], [142.35159055962103, 166.8891315058427, 146.3623987630658, 150.69813365332797, 165.13197419074965, 136.91583982012213, 149.22514550882286, 157.90954418769113, 130.1827751692454, 157.96372563287196], [143.43336569884465, 162.27639083571958, 151.8097645753834, 136.64783823820326, 147.15900502194785, 139.29224338683775, 141.99632632747594, 159.98622905009674, 158.28108176744016, 162.74801408941113], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [142.25652363847527, 159.5999057865361, 142.0543137300079, 146.48341002427597, 145.1374968505289, 144.9938790373216, 159.7528243366441, 155.84183321006986, 146.98291684943885, 160.52715552806197], [141.26685426640162, 155.80429527279927, 143.88566867940946, 149.04282074550076, 158.49796293787327, 152.6871646979185, 138.616325116148, 165.64384663639626, 151.5560792244251, 146.62924141448818], [137.39806057977424, 148.58966617518814, 140.67400125052686, 159.98720654102195, 151.20648545278075, 134.57334417065363, 151.30659911431914, 162.4738491702741, 157.48089409974844, 159.94015243707338], [149.32058635056538, 157.63423688632014, 146.03466042029427, 158.29505074437785, 157.13716494150168, 114.1485851534252, 149.72902839123503, 160.75893793890506, 151.6115237359382, 158.96048442879763], [140.27965468686358, 150.0499170094252, 132.17261217851004, 163.7737470087345, 159.91712491334698, 154.9198971312533, 149.42348182272832, 143.72980228972474, 153.57246354785806, 155.79155840291588], [145.53652095954817, 163.32896093363726, 145.83922379407923, 139.59257291067934, 157.5803745697041, 142.30329659241025, 149.5140693517617, 150.27860689867248, 152.76200183233587, 156.89463114853217], [141.14757650090718, 159.77000143923615, 140.87122760860075, 159.86621289459802, 148.49973773854714, 118.46152402005815, 154.26502009369028, 160.0846209339392, 157.96858191571968, 162.69575584606412], [128.37183100025948, 168.31303965328658, 145.3544291690687, 160.20901607844743, 161.69201884997244, 140.06227788360673, 155.67390226891183, 162.61713237672632, 116.65156785148072, 164.6850438596003], [140.89029956579077, 162.79560262398593, 140.04512113866295, 149.23634161953396, 150.1315836138893, 123.17832467701236, 154.01558943006262, 171.11158833983797, 160.12163717255703, 152.1041708100277], [143.35893609363842, 162.52970249105087, 138.28225415037392, 145.2731801238887, 144.05906475069207, 148.0718842215696, 160.35204226743426, 158.20843931707492, 149.47815340911865, 154.0166021665192], [142.47324381977754, 159.75391385863625, 139.89686476919496, 145.92151539200015, 165.15378792221145, 141.8884481702422, 147.56315632618478, 157.37789100557123, 152.37492819700643, 151.2265095305356], [151.18591401869966, 164.53591801468053, 146.12620232042943, 146.49236792115607, 145.01180344561874, 142.18838554532982, 165.64714172032012, 154.4700576636602, 138.958999413653, 149.01346892781294], [145.97241670858784, 159.4535781753873, 142.4068495408466, 159.75930928992415, 147.97068820255, 126.87563086386061, 141.54999018159674, 159.32003925937462, 156.24548341981966, 164.07627334941307], [138.69691740865682, 161.36899676610903, 141.0319809300706, 142.05497300143577, 151.9853314935421, 150.1777877692477, 158.95250888203665, 158.09076104019178, 150.52377473544067, 150.74722696462945], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [142.2658121296411, 160.38961981911044, 144.1672194187174, 146.02217881828875, 150.95892872813042, 146.28621665894028, 145.71725887590006, 163.4473520811939, 156.69328216630524, 147.68239029513305], [145.18619098277483, 158.099399886659, 141.65275875946995, 145.5376776347957, 160.17451813795222, 141.11272369244492, 158.52271796849632, 154.17722545010116, 153.2253082891169, 145.9417381895496], [143.0805372769047, 161.28337645928195, 141.75098649846507, 142.3715891042668, 162.97239903736323, 141.34306445929676, 156.9939742245395, 152.34450483926946, 149.82029047723458, 151.66953661473852], [138.66076706253511, 157.9357235364792, 139.25396125449473, 161.02983880635668, 150.70856742682898, 126.93022278239751, 154.6225264200445, 159.46434923593975, 153.42513888248823, 161.5991635837959], [146.64317479735988, 161.5337112728855, 150.47215491636206, 145.53368330088531, 154.55868909231992, 141.1877137989166, 163.56305914137073, 153.07863709074726, 141.11139776641875, 145.94803781409468], [144.60010629456147, 169.43951929689237, 142.4570306270456, 145.33699899674997, 161.25303423071955, 145.5055759990721, 151.06696141231535, 155.54480781204182, 132.65222904761524, 155.77399527434713], [123.4791607988294, 161.33603491669362, 131.02644054355991, 144.7481620312516, 149.7863160951474, 161.6152063451183, 173.48438400022587, 153.54428119663942, 149.78389164114128, 154.82638142275377], [151.77483014045058, 157.36992639649077, 145.1618572256677, 158.0463074247516, 156.45693331800123, 120.78821544824784, 148.9198164926133, 152.63719450795264, 157.35176560591893, 155.12341243126613], [143.74384306196606, 164.1252770443115, 151.80434598827767, 136.06238542529633, 148.60885914109565, 136.33344822627134, 148.02587785777536, 158.63036197759527, 153.8425704067714, 162.4532898619999], [140.9692473082241, 158.83708354814627, 142.50648445339854, 150.6469290609464, 159.43914344419983, 143.88423257680765, 151.95366940862746, 162.83914933877537, 153.26970678446094, 139.28461306777402], [143.35893609363842, 162.52970249105087, 138.28225415037392, 145.2731801238887, 144.05906475069207, 148.0718842215696, 160.35204226743426, 158.20843931707492, 149.47815340911865, 154.0166021665192], [138.5950961011988, 159.93270578904753, 145.68391375185405, 142.55305687560497, 151.24177471797898, 147.22991933251757, 155.39988729281495, 164.16938949754916, 152.11914188605147, 146.7053737467431], [140.43119284335623, 164.15110042573548, 136.54600560664568, 136.53489502042416, 156.16264309799706, 145.90220196994045, 146.3435165551005, 162.685726080723, 156.44291786101934, 158.43005953041867], [142.93905828606603, 156.17886135868338, 140.83900194594102, 159.81222040273823, 150.47350943243492, 126.48838000412711, 152.21387729630555, 159.85812911026164, 152.13961889080628, 162.68760226399635], [148.52011380851286, 169.08039622624645, 151.36598427676907, 128.46548911131615, 148.03588501992917, 149.58935401608588, 151.15202592734116, 162.57793407903947, 144.22395238289582, 150.61912414322452], [148.2954193196735, 152.24427197966386, 138.2287898368027, 159.317863919773, 157.61598652265508, 158.62815209128155, 147.91205987985015, 135.39050732987238, 154.9251591488199, 151.0720489629685], [128.37183100025948, 168.31303965328658, 145.3544291690687, 160.20901607844743, 161.69201884997244, 140.06227788360673, 155.67390226891183, 162.61713237672632, 116.65156785148072, 164.6850438596003], [146.20671553242394, 168.4914372357847, 150.66503756070438, 142.91002004209219, 151.74386525948898, 146.2479686509097, 149.46673232274205, 154.12028522527538, 146.43635281851195, 147.34184434342723], [152.1650596290336, 172.7346441851432, 149.51134947937075, 130.71145715645213, 145.1106205053203, 148.80357162328332, 168.1370380014965, 159.87646251775178, 137.6534471253657, 138.92660876814332]]</t>
+          <t>[[128.27953388521115, 130.07609800230134, 115.78714566717395, 132.3775869716199, 111.68065528487813, 117.96055178639185, 123.61943761494285, 95.26495295287239, 109.53808433863523, 118.79376194408553], [121.63875209521336, 110.39859515388954, 121.37986977584023, 131.31156348114973, 115.33772045646188, 107.16234987306811, 125.64098595967806, 115.93048755533184, 115.6395764550268, 116.5324927174425], [112.94310209399319, 115.64467207659158, 116.58660591960145, 120.12510909159207, 128.36262358806923, 125.99226461262177, 118.5348304020664, 102.54439531411163, 122.59074902608828, 117.28700320999988], [128.76600893140687, 113.82690644861597, 110.69854043048886, 128.66241151581585, 113.86481827509704, 115.97682708056954, 129.2000408481944, 125.81919896204528, 92.28224477271954, 118.09729344322648], [114.01336406019885, 123.99338474017804, 118.84899835028762, 114.76003518453246, 114.71921400101306, 125.61343493155562, 124.86124222254566, 93.9204166871229, 125.35911331195993, 122.62936568778417]]</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>["S", 3]</t>
+          <t>['S', 3]</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1880,14 +1880,14 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E28" t="b">
         <v>1</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>12.4</t>
+          <t>11.200000000000001</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>[[15.0, 12.0, 16.0, 15.0, 13.0, 14.0, 12.0, 15.0, 15.0, 13.0], [16.0, 16.0, 10.0, 15.0, 16.0, 14.0, 14.0, 10.0, 13.0, 16.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [15.0, 16.0, 12.0, 14.0, 16.0, 13.0, 14.0, 12.0, 15.0, 13.0]]</t>
+          <t>[[13.0, 12.0, 12.0, 19.0, 15.0, 13.0, 10.0, 15.0, 14.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [14.0, 12.0, 12.0, 10.0, 10.0, 13.0, 10.0, 14.0, 12.0, 13.0]]</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>["S", 3]</t>
+          <t>['S', 3]</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1933,7 +1933,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>[[17.0, 14.0, 18.0, 17.0, 13.0, 16.0, 14.0, 19.0, 17.0, 15.0], [18.0, 14.0, 15.0, 17.0, 15.0, 16.0, 12.0, 17.0, 19.0, 17.0], [18.0, 15.0, 16.0, 18.0, 14.0, 14.0, 15.0, 16.0, 16.0, 18.0], [18.0, 18.0, 15.0, 14.0, 18.0, 14.0, 19.0, 12.0, 15.0, 17.0], [19.0, 16.0, 13.0, 18.0, 16.0, 16.0, 17.0, 10.0, 18.0, 17.0]]</t>
+          <t>[[13.0, 18.0, 13.0, 19.0, 15.0, 16.0, 15.0, 19.0, 16.0, 16.0], [14.0, 19.0, 14.0, 14.0, 19.0, 14.0, 14.0, 16.0, 20.0, 16.0], [15.0, 17.0, 16.0, 15.0, 20.0, 18.0, 16.0, 14.0, 14.0, 15.0], [20.0, 22.0, 15.0, 17.0, 10.0, 13.0, 15.0, 19.0, 13.0, 16.0], [16.0, 15.0, 14.0, 15.0, 11.0, 14.0, 17.0, 24.0, 20.0, 14.0]]</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>["J", 3]</t>
+          <t>[4, 3]</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1986,14 +1986,14 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E30" t="b">
         <v>1</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>NAN</t>
+          <t>10.8</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>117.971439013186</t>
+          <t>146.19195559749386</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2013,12 +2013,12 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[[12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 13.0, 12.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 16.0, 10.0, 13.0, 13.0, 10.0, 13.0, 12.0, 10.0, 13.0]]</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>[[120.63388375216417, 111.40675460023704, 130.4025033919097, 119.04598225071695, 123.7427249344768, 110.18512818275588, 107.70961596250459, 122.19558525796495, 117.0260236450421, 117.36618815408781], [120.63388375216417, 111.40675460023704, 130.4025033919097, 119.04598225071695, 123.7427249344768, 110.18512818275588, 107.70961596250459, 122.19558525796495, 117.0260236450421, 117.36618815408781], [120.63388375216417, 111.40675460023704, 130.4025033919097, 119.04598225071695, 123.7427249344768, 110.18512818275588, 107.70961596250459, 122.19558525796495, 117.0260236450421, 117.36618815408781], [120.63388375216417, 111.40675460023704, 130.4025033919097, 119.04598225071695, 123.7427249344768, 110.18512818275588, 107.70961596250459, 122.19558525796495, 117.0260236450421, 117.36618815408781], [120.63388375216417, 111.40675460023704, 130.4025033919097, 119.04598225071695, 123.7427249344768, 110.18512818275588, 107.70961596250459, 122.19558525796495, 117.0260236450421, 117.36618815408781]]</t>
+          <t>[[146.23059123078906, 148.79925088929974, 140.43978721216746, 159.5644857451664, 159.4405700016616, 154.42563871315122, 153.0308171637937, 138.8733659357018, 138.34377678010426, 147.9631496181988], [127.79766562978502, 163.97214672074955, 157.6495378050816, 133.73689187396675, 147.86640348890023, 168.42100164517598, 155.5624442478229, 112.0605314953164, 176.8352429388917, 146.56222477349235], [151.33653114377427, 142.87579955428012, 145.37014146096828, 128.43487080227436, 160.31190748344477, 150.12429019101253, 146.73680867790208, 79.96916544073163, 173.8939194864584, 141.45228899754798], [185.73901548318233, 142.22321382053934, 146.38517451927382, 104.88640660422055, 174.47422745532646, 142.0605830315376, 126.63956795747089, 114.094072647251, 127.31641557955146, 182.44787001786548], [153.6767908871729, 172.81348471820095, 110.35855142876746, 170.42271541048942, 149.36522265525508, 118.78857111032708, 146.7141806682058, 161.26949314627657, 133.9897081183551, 147.85126746781256]]</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>["J", 3]</t>
+          <t>[4, 3]</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2039,14 +2039,14 @@
         </is>
       </c>
       <c r="D31" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E31" t="b">
         <v>1</v>
       </c>
-      <c r="E31" t="b">
-        <v>0</v>
-      </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>NAN</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>117.971439013186</t>
+          <t>149.14736821453283</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2066,12 +2066,12 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[[12.0, 11.0, 12.0, 13.0, 12.0, 11.0, 12.0, 12.0, 13.0, 12.0], [13.0, 12.0, 12.0, 12.0, 12.0, 11.0, 14.0, 11.0, 12.0, 11.0], [12.0, 12.0, 12.0, 13.0, 10.0, 12.0, 13.0, 12.0, 12.0, 12.0], [12.0, 10.0, 12.0, 11.0, 13.0, 11.0, 13.0, 14.0, 11.0, 13.0], [12.0, 13.0, 12.0, 11.0, 12.0, 12.0, 13.0, 13.0, 12.0, 10.0]]</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>[[120.63388375216417, 111.40675460023704, 130.4025033919097, 119.04598225071695, 123.7427249344768, 110.18512818275588, 107.70961596250459, 122.19558525796495, 117.0260236450421, 117.36618815408781], [120.63388375216417, 111.40675460023704, 130.4025033919097, 119.04598225071695, 123.7427249344768, 110.18512818275588, 107.70961596250459, 122.19558525796495, 117.0260236450421, 117.36618815408781], [120.63388375216417, 111.40675460023704, 130.4025033919097, 119.04598225071695, 123.7427249344768, 110.18512818275588, 107.70961596250459, 122.19558525796495, 117.0260236450421, 117.36618815408781], [120.63388375216417, 111.40675460023704, 130.4025033919097, 119.04598225071695, 123.7427249344768, 110.18512818275588, 107.70961596250459, 122.19558525796495, 117.0260236450421, 117.36618815408781], [120.63388375216417, 111.40675460023704, 130.4025033919097, 119.04598225071695, 123.7427249344768, 110.18512818275588, 107.70961596250459, 122.19558525796495, 117.0260236450421, 117.36618815408781]]</t>
+          <t>[[159.11414144957013, 142.91299253305849, 140.05763197773456, 162.6184971197973, 148.78229280943734, 130.71717204232044, 157.3248147700463, 130.79166015409868, 164.87647549706276, 156.52470814729978], [151.55337695271137, 166.70056705833161, 145.1753415877048, 156.46164978422945, 158.81079935308287, 137.7758965237918, 151.97771319458153, 134.88627739056443, 141.98012995886506, 147.93030414837781], [153.56270009496382, 147.2862035722315, 151.52749771314424, 137.20499187890496, 131.29327866972315, 158.11906171726062, 171.50118274158342, 129.15348999220907, 154.18563812605686, 160.03379363827756], [158.31810498837683, 122.91995390029523, 163.0623893714786, 147.61944394053936, 150.61018596137134, 138.40811883097146, 161.21729282872076, 129.60712824957804, 144.61954134628775, 172.28837990850352], [142.5007763393659, 160.7182970763203, 162.85408550783853, 144.59885820712196, 152.8391027209713, 158.4152221303833, 159.43529126602985, 122.60635893916222, 145.9713942595898, 137.91820435671303]]</t>
         </is>
       </c>
     </row>
@@ -2092,14 +2092,14 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="E32" t="b">
         <v>1</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>10.8</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>144.0694592507186</t>
+          <t>149.0067919076293</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2119,12 +2119,12 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 11.0, 13.0, 10.0, 14.0, 10.0, 10.0, 14.0, 14.0, 14.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0]]</t>
+          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 13.0, 12.0, 12.0, 12.0, 12.0, 13.0, 12.0, 12.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 11.0, 12.0, 13.0, 13.0, 11.0, 13.0, 12.0, 11.0, 12.0], [16.0, 15.0, 15.0, 13.0, 14.0, 13.0, 12.0, 15.0, 13.0, 14.0]]</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>[[171.67381543698417, 121.91060904702671, 145.6585137824614, 153.21305931525632, 131.79351506261247, 101.79753146907926, 144.20434380538205, 145.15285429284592, 169.02822720398967, 171.57082143390124], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [117.0671524124359, 86.84846978023653, 144.158379868197, 171.42811144601143, 199.67258146354172, 65.9627966957149, 144.85734474176556, 154.18804164564273, 160.2731231682561, 188.3833856349], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [169.16533358350605, 125.2512122003425, 124.36982905582596, 152.3431774421878, 164.55270315503893, 99.58614228205624, 138.9677058715599, 154.38699831564628, 167.33125598678217, 152.1864118047564]]</t>
+          <t>[[128.17407962248393, 150.6713190595997, 147.77686044990935, 155.42354837976694, 155.1518561168611, 163.4849657450738, 151.4881468361689, 135.48760441389305, 156.90462834689848, 149.8034661229313], [158.07257500815376, 149.42150277173343, 159.91586053467765, 164.17924146962326, 154.1224511761639, 158.45897751561657, 151.337747840098, 133.68864268378707, 134.80809267523554, 129.82497636597296], [117.73621954196513, 159.32425848233808, 115.09770021295435, 108.64424579438034, 174.30753576777835, 161.8550342373769, 166.6235788330783, 135.00163097610917, 161.36236518055298, 192.1347175271378], [148.8544951284401, 151.40602154120006, 165.37557737056235, 156.73548065874104, 161.04863177124207, 151.337641336202, 144.41001934522308, 115.29392968699467, 130.55864746528303, 161.4608324810581], [161.52742157081613, 158.7498696429248, 163.93614824552407, 133.28153004535383, 150.6115411136571, 148.0801728676479, 147.3800272020566, 128.2492932383538, 142.8272687084802, 148.93121627338377]]</t>
         </is>
       </c>
     </row>
@@ -2145,14 +2145,14 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="E33" t="b">
         <v>1</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.200000000000001</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>144.49807636431558</t>
+          <t>147.0019746451607</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2172,12 +2172,12 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 11.0, 13.0, 10.0, 14.0, 10.0, 10.0, 14.0, 14.0, 14.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 13.0, 13.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 14.0, 10.0, 10.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0]]</t>
+          <t>[[15.0, 12.0, 14.0, 14.0, 14.0, 14.0, 13.0, 15.0, 13.0, 16.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [14.0, 14.0, 10.0, 14.0, 10.0, 13.0, 13.0, 10.0, 12.0, 10.0]]</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>[[171.67381543698417, 121.91060904702671, 145.6585137824614, 153.21305931525632, 131.79351506261247, 101.79753146907926, 144.20434380538205, 145.15285429284592, 169.02822720398967, 171.57082143390124], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [117.0671524124359, 86.84846978023653, 144.158379868197, 171.42811144601143, 199.67258146354172, 65.9627966957149, 144.85734474176556, 154.18804164564273, 160.2731231682561, 188.3833856349], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [169.16533358350605, 125.2512122003425, 124.36982905582596, 152.3431774421878, 164.55270315503893, 99.58614228205624, 138.9677058715599, 154.38699831564628, 167.33125598678217, 152.1864118047564], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [158.91879250547223, 109.34905424813742, 151.8325536909609, 152.68116070222248, 146.07804621145328, 106.86655881456286, 136.88045179693185, 154.13992758038017, 160.99605161933857, 179.23554052829246], [147.69556523473256, 119.61709997950122, 160.24986339852572, 151.8924649007107, 162.39451480720385, 107.1137112904901, 120.95681944842299, 150.01966305951794, 154.40819491054984, 158.87312273925517], [151.75926646509785, 109.8886301535245, 151.53074398765813, 156.40416673372965, 134.9951394547665, 121.13166969142071, 149.92145423768537, 153.96707325127616, 160.15394794087257, 173.79465689965093], [149.73435649974806, 109.66089149608842, 155.06539360124026, 172.89423563219376, 171.21374507309983, 98.03539136506976, 123.97995851126295, 151.2177782733371, 158.14025310250054, 174.9784724380392]]</t>
+          <t>[[152.03127743495924, 131.26670686790283, 159.8490421036773, 135.86848756903362, 157.95629509709286, 150.1028699651616, 164.81293411936133, 127.85624458701675, 138.61092449650556, 173.616362921388], [139.12114064773328, 145.72937881484435, 156.20033633985406, 142.99311727269918, 138.80547384392406, 163.32945241330683, 154.95967816733656, 139.9668209019815, 154.84033456962823, 155.6901255374023], [154.44771596361446, 154.77516980055975, 170.16560900029444, 137.14975634114316, 148.3662676894486, 138.98320370700708, 132.5246189804189, 138.14586976040644, 153.70831507278874, 141.03408723605426], [174.2200869452611, 159.2943972186211, 163.3144277326722, 102.10440775625221, 162.01377810859188, 107.27670888878187, 144.82011201987459, 109.20862642243796, 163.75407556238778, 159.73653221889975], [155.66336328043957, 137.68724676017456, 151.09943304013282, 144.3950619538513, 157.49445593729854, 162.21449460723338, 130.71640283672272, 133.20706401399931, 135.1568463256065, 143.81359340625056]]</t>
         </is>
       </c>
     </row>
@@ -2198,14 +2198,14 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E34" t="b">
         <v>1</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>11.066666666666666</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2215,7 +2215,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>143.85387573298934</t>
+          <t>146.91538446482338</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2225,12 +2225,12 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 11.0, 13.0, 10.0, 14.0, 10.0, 10.0, 14.0, 14.0, 14.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 13.0, 13.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 14.0, 10.0, 10.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0]]</t>
+          <t>[[13.0, 12.0, 12.0, 13.0, 10.0, 12.0, 12.0, 12.0, 12.0, 12.0], [11.0, 13.0, 12.0, 12.0, 12.0, 11.0, 11.0, 13.0, 12.0, 13.0], [13.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 13.0, 12.0, 10.0], [10.0, 10.0, 12.0, 14.0, 10.0, 13.0, 14.0, 12.0, 13.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0]]</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>[[171.67381543698417, 121.91060904702671, 145.6585137824614, 153.21305931525632, 131.79351506261247, 101.79753146907926, 144.20434380538205, 145.15285429284592, 169.02822720398967, 171.57082143390124], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [117.0671524124359, 86.84846978023653, 144.158379868197, 171.42811144601143, 199.67258146354172, 65.9627966957149, 144.85734474176556, 154.18804164564273, 160.2731231682561, 188.3833856349], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [169.16533358350605, 125.2512122003425, 124.36982905582596, 152.3431774421878, 164.55270315503893, 99.58614228205624, 138.9677058715599, 154.38699831564628, 167.33125598678217, 152.1864118047564], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [158.91879250547223, 109.34905424813742, 151.8325536909609, 152.68116070222248, 146.07804621145328, 106.86655881456286, 136.88045179693185, 154.13992758038017, 160.99605161933857, 179.23554052829246], [147.69556523473256, 119.61709997950122, 160.24986339852572, 151.8924649007107, 162.39451480720385, 107.1137112904901, 120.95681944842299, 150.01966305951794, 154.40819491054984, 158.87312273925517], [151.75926646509785, 109.8886301535245, 151.53074398765813, 156.40416673372965, 134.9951394547665, 121.13166969142071, 149.92145423768537, 153.96707325127616, 160.15394794087257, 173.79465689965093], [149.73435649974806, 109.66089149608842, 155.06539360124026, 172.89423563219376, 171.21374507309983, 98.03539136506976, 123.97995851126295, 151.2177782733371, 158.14025310250054, 174.9784724380392], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [154.87670501106774, 124.45712875915734, 159.00186930720025, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 149.50901730168147, 153.1866101146596, 155.4404734500336], [148.57242003247117, 115.00137686241824, 127.42349700300535, 153.358448411623, 169.82162012787782, 102.0493683148124, 140.3944107616491, 157.57071101559134, 169.1542118150403, 169.08558067012228], [118.9573278499153, 87.27566948350537, 141.8942472343372, 156.0887845439302, 215.99334155094448, 63.60144531528303, 141.586417049037, 156.4440274161946, 157.31476582791896, 185.21953219907152], [155.63356434101732, 121.7037973314125, 141.61047245367973, 128.56412415865336, 136.09008626574686, 141.05775541519452, 134.93095555474864, 125.91983083232476, 131.26261056343623, 182.36619594400247]]</t>
+          <t>[[151.5685490056792, 144.4666159444, 154.24404120935523, 153.71141012768595, 136.09079868620188, 163.1257355569045, 145.52404551895583, 140.7613203547948, 150.83782811123078, 150.71426256045547], [110.39887649822099, 148.9418711753576, 159.16725337318633, 162.91418394253253, 160.25353249901715, 151.13866883284427, 129.16101084848788, 142.63509939798882, 171.48937537671148, 147.36174543690385], [162.65169068616527, 150.1474079019236, 134.87809915999514, 103.87675631102218, 171.1716395949866, 154.089214378227, 166.10073988198465, 128.96941884189857, 155.65314949788933, 156.38490498450807], [152.39149129061184, 98.36984845438856, 145.67368259689124, 177.48746555015126, 127.10419522040551, 149.56956087850878, 169.77080025105258, 139.0745897367991, 147.99088696923351, 144.9166808818338], [150.22491736423288, 152.05381263504862, 174.27705071453641, 161.4804216692513, 150.42671831669097, 156.7828367955221, 140.7336497710047, 126.90074883954217, 111.56281715803364, 110.54780245191581]]</t>
         </is>
       </c>
     </row>
@@ -2251,14 +2251,14 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="E35" t="b">
         <v>1</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>11.100000000000001</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>143.78707953071117</t>
+          <t>149.118668319664</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2278,12 +2278,12 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 11.0, 13.0, 10.0, 14.0, 10.0, 10.0, 14.0, 14.0, 14.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 13.0, 13.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 14.0, 10.0, 10.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [13.0, 10.0, 13.0, 16.0, 13.0, 10.0, 13.0, 17.0, 19.0, 16.0], [10.0, 11.0, 14.0, 14.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0]]</t>
+          <t>[[12.0, 10.0, 12.0, 13.0, 13.0, 12.0, 13.0, 10.0, 13.0, 12.0], [12.0, 12.0, 13.0, 10.0, 12.0, 14.0, 11.0, 11.0, 12.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 13.0, 12.0, 12.0, 12.0, 12.0, 10.0, 12.0, 13.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0]]</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>[[171.67381543698417, 121.91060904702671, 145.6585137824614, 153.21305931525632, 131.79351506261247, 101.79753146907926, 144.20434380538205, 145.15285429284592, 169.02822720398967, 171.57082143390124], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [117.0671524124359, 86.84846978023653, 144.158379868197, 171.42811144601143, 199.67258146354172, 65.9627966957149, 144.85734474176556, 154.18804164564273, 160.2731231682561, 188.3833856349], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [169.16533358350605, 125.2512122003425, 124.36982905582596, 152.3431774421878, 164.55270315503893, 99.58614228205624, 138.9677058715599, 154.38699831564628, 167.33125598678217, 152.1864118047564], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [158.91879250547223, 109.34905424813742, 151.8325536909609, 152.68116070222248, 146.07804621145328, 106.86655881456286, 136.88045179693185, 154.13992758038017, 160.99605161933857, 179.23554052829246], [147.69556523473256, 119.61709997950122, 160.24986339852572, 151.8924649007107, 162.39451480720385, 107.1137112904901, 120.95681944842299, 150.01966305951794, 154.40819491054984, 158.87312273925517], [151.75926646509785, 109.8886301535245, 151.53074398765813, 156.40416673372965, 134.9951394547665, 121.13166969142071, 149.92145423768537, 153.96707325127616, 160.15394794087257, 173.79465689965093], [149.73435649974806, 109.66089149608842, 155.06539360124026, 172.89423563219376, 171.21374507309983, 98.03539136506976, 123.97995851126295, 151.2177782733371, 158.14025310250054, 174.9784724380392], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [154.87670501106774, 124.45712875915734, 159.00186930720025, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 149.50901730168147, 153.1866101146596, 155.4404734500336], [148.57242003247117, 115.00137686241824, 127.42349700300535, 153.358448411623, 169.82162012787782, 102.0493683148124, 140.3944107616491, 157.57071101559134, 169.1542118150403, 169.08558067012228], [118.9573278499153, 87.27566948350537, 141.8942472343372, 156.0887845439302, 215.99334155094448, 63.60144531528303, 141.586417049037, 156.4440274161946, 157.31476582791896, 185.21953219907152], [155.63356434101732, 121.7037973314125, 141.61047245367973, 128.56412415865336, 136.09008626574686, 141.05775541519452, 134.93095555474864, 125.91983083232476, 131.26261056343623, 182.36619594400247], [151.0530785897105, 100.13685713420632, 161.3782749695759, 158.82492821063502, 156.23168163705236, 98.31033969951382, 146.06938513288128, 146.66128011680243, 160.50369887210744, 191.8184134047504], [169.84163444520755, 123.3416986713996, 154.83107455194718, 167.98929163470268, 140.7932798872149, 101.68952014718067, 141.77615836031643, 146.55188089601023, 156.74047339913525, 163.36485909573406], [122.27088733454492, 109.20997405555539, 165.61688938660893, 170.33382062522801, 182.70092984366494, 107.97616157403853, 103.39739396512512, 145.35031470925776, 163.65926547880437, 160.94583046901406], [116.35505577055113, 114.1192854646577, 123.7609397041828, 160.69814808763311, 178.38382498160877, 68.98150340340261, 133.86332008334244, 146.19438482366462, 176.35573400668068, 183.52554229325003], [115.76525255456991, 91.80230503030586, 149.46566000403075, 164.23826817920266, 199.34751449005594, 96.97113934572377, 125.65836770040076, 139.29213316594414, 166.70626408889285, 158.4806267178086]]</t>
+          <t>[[150.98064992027236, 135.86576076198904, 146.15378167233712, 162.28162462235056, 156.81105793396955, 150.8318334930873, 156.7461385267176, 142.79943411620894, 146.91577183831257, 144.7252143562382], [166.30042232517036, 164.62616632532476, 165.42103893891075, 139.53666401531544, 145.71962010595155, 159.71474995150868, 126.17523019305285, 131.26798918727118, 146.87929136377159, 148.33007096885055], [143.86849818074938, 152.9687229323682, 147.47646732755058, 149.98403830932304, 161.45472328379284, 165.38557739794302, 169.3551464528067, 128.05024658933655, 137.7875236745344, 136.83298648290176], [142.5635308585779, 145.59122558624318, 158.2964388625752, 173.4560994868657, 143.72727261347873, 146.7382279888007, 148.24995359730536, 130.04191641482734, 150.52729224946032, 154.6382066738736], [142.55662692724343, 180.51090949986093, 111.26941191434567, 173.0679859365572, 182.76298758992044, 159.3306008158138, 140.21355390157322, 101.92550355562457, 143.23482728222007, 145.9844029801145]]</t>
         </is>
       </c>
     </row>
@@ -2304,14 +2304,14 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="E36" t="b">
         <v>1</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>11.279999999999998</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>143.79998787685767</t>
+          <t>148.65912722149181</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2331,12 +2331,12 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 11.0, 13.0, 10.0, 14.0, 10.0, 10.0, 14.0, 14.0, 14.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 13.0, 13.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 14.0, 10.0, 10.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [13.0, 10.0, 13.0, 16.0, 13.0, 10.0, 13.0, 17.0, 19.0, 16.0], [10.0, 11.0, 14.0, 14.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 13.0, 17.0, 10.0, 14.0, 17.0, 19.0, 17.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 14.0, 14.0, 14.0, 10.0, 10.0, 14.0, 14.0, 10.0]]</t>
+          <t>[[12.0, 10.0, 12.0, 13.0, 13.0, 12.0, 12.0, 13.0, 11.0, 12.0], [13.0, 10.0, 12.0, 13.0, 13.0, 13.0, 14.0, 12.0, 10.0, 10.0], [12.0, 13.0, 12.0, 12.0, 12.0, 12.0, 12.0, 12.0, 13.0, 10.0], [12.0, 14.0, 12.0, 12.0, 12.0, 10.0, 12.0, 12.0, 12.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0]]</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>[[171.67381543698417, 121.91060904702671, 145.6585137824614, 153.21305931525632, 131.79351506261247, 101.79753146907926, 144.20434380538205, 145.15285429284592, 169.02822720398967, 171.57082143390124], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [117.0671524124359, 86.84846978023653, 144.158379868197, 171.42811144601143, 199.67258146354172, 65.9627966957149, 144.85734474176556, 154.18804164564273, 160.2731231682561, 188.3833856349], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [169.16533358350605, 125.2512122003425, 124.36982905582596, 152.3431774421878, 164.55270315503893, 99.58614228205624, 138.9677058715599, 154.38699831564628, 167.33125598678217, 152.1864118047564], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [158.91879250547223, 109.34905424813742, 151.8325536909609, 152.68116070222248, 146.07804621145328, 106.86655881456286, 136.88045179693185, 154.13992758038017, 160.99605161933857, 179.23554052829246], [147.69556523473256, 119.61709997950122, 160.24986339852572, 151.8924649007107, 162.39451480720385, 107.1137112904901, 120.95681944842299, 150.01966305951794, 154.40819491054984, 158.87312273925517], [151.75926646509785, 109.8886301535245, 151.53074398765813, 156.40416673372965, 134.9951394547665, 121.13166969142071, 149.92145423768537, 153.96707325127616, 160.15394794087257, 173.79465689965093], [149.73435649974806, 109.66089149608842, 155.06539360124026, 172.89423563219376, 171.21374507309983, 98.03539136506976, 123.97995851126295, 151.2177782733371, 158.14025310250054, 174.9784724380392], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [154.87670501106774, 124.45712875915734, 159.00186930720025, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 149.50901730168147, 153.1866101146596, 155.4404734500336], [148.57242003247117, 115.00137686241824, 127.42349700300535, 153.358448411623, 169.82162012787782, 102.0493683148124, 140.3944107616491, 157.57071101559134, 169.1542118150403, 169.08558067012228], [118.9573278499153, 87.27566948350537, 141.8942472343372, 156.0887845439302, 215.99334155094448, 63.60144531528303, 141.586417049037, 156.4440274161946, 157.31476582791896, 185.21953219907152], [155.63356434101732, 121.7037973314125, 141.61047245367973, 128.56412415865336, 136.09008626574686, 141.05775541519452, 134.93095555474864, 125.91983083232476, 131.26261056343623, 182.36619594400247], [151.0530785897105, 100.13685713420632, 161.3782749695759, 158.82492821063502, 156.23168163705236, 98.31033969951382, 146.06938513288128, 146.66128011680243, 160.50369887210744, 191.8184134047504], [169.84163444520755, 123.3416986713996, 154.83107455194718, 167.98929163470268, 140.7932798872149, 101.68952014718067, 141.77615836031643, 146.55188089601023, 156.74047339913525, 163.36485909573406], [122.27088733454492, 109.20997405555539, 165.61688938660893, 170.33382062522801, 182.70092984366494, 107.97616157403853, 103.39739396512512, 145.35031470925776, 163.65926547880437, 160.94583046901406], [116.35505577055113, 114.1192854646577, 123.7609397041828, 160.69814808763311, 178.38382498160877, 68.98150340340261, 133.86332008334244, 146.19438482366462, 176.35573400668068, 183.52554229325003], [115.76525255456991, 91.80230503030586, 149.46566000403075, 164.23826817920266, 199.34751449005594, 96.97113934572377, 125.65836770040076, 139.29213316594414, 166.70626408889285, 158.4806267178086], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [123.72400459693046, 101.31380805074481, 135.26798136474852, 145.08457880992663, 200.86161538572605, 89.75116450662642, 120.30558500298024, 158.45816233102877, 174.8894098741557, 177.71466936907032], [149.27816962680123, 108.37247732346466, 138.71329142679446, 152.99701822494, 183.85670983256415, 98.26543736382182, 127.5550170615973, 153.75067512774277, 157.57839871208935, 183.54169965397787], [124.60931392388997, 99.55757900064643, 161.99929959628253, 150.1285082839572, 186.11983693459018, 86.00430019489998, 119.13204577034072, 155.41436252761594, 169.16448238826908, 170.3493231523084], [163.82826724191202, 123.63300303116105, 162.8980670120787, 166.58612468713937, 158.67319842829247, 101.19007738890186, 123.85647903797361, 141.86796497619403, 159.9811243798996, 158.63953984939445]]</t>
+          <t>[[149.3520095076797, 131.2003734649116, 155.12253015438918, 165.97256935006672, 146.7804088048679, 160.543425160181, 150.90865006741842, 159.93614819855367, 130.05929372570847, 143.25821697062187], [148.69098117060324, 127.90438353101385, 162.08069096236432, 152.7642584510545, 164.0445326464666, 150.7142477585181, 167.55924928859804, 155.65442230619735, 130.70896676888762, 122.69850984120151], [150.64185262371987, 149.86987706263562, 161.6798397952058, 132.73720459337855, 141.0641618242042, 155.53535429386318, 162.59633813581874, 143.16800043423268, 145.00030010495482, 152.3278691351194], [164.15776696394883, 148.45657308977562, 157.19318208265736, 146.79743066095526, 163.761842216108, 152.12019605793708, 144.72792811891307, 129.39388419951285, 142.17662854419325, 143.8794992353713], [146.6722312573745, 145.01700711015621, 163.64514645931087, 114.04897422132902, 134.98206812656045, 165.67054597948555, 162.16539856979955, 153.0721944853858, 131.21919335209054, 153.22400421128827]]</t>
         </is>
       </c>
     </row>
@@ -2357,14 +2357,14 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="E37" t="b">
         <v>1</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>11.333333333333332</t>
+          <t>10.8</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>143.98310832939723</t>
+          <t>147.99111164856293</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2384,12 +2384,12 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 11.0, 13.0, 10.0, 14.0, 10.0, 10.0, 14.0, 14.0, 14.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 13.0, 13.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 14.0, 10.0, 10.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [13.0, 10.0, 13.0, 16.0, 13.0, 10.0, 13.0, 17.0, 19.0, 16.0], [10.0, 11.0, 14.0, 14.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 13.0, 17.0, 10.0, 14.0, 17.0, 19.0, 17.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 14.0, 14.0, 14.0, 10.0, 10.0, 14.0, 14.0, 10.0], [10.0, 10.0, 13.0, 19.0, 16.0, 10.0, 13.0, 13.0, 19.0, 17.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0]]</t>
+          <t>[[12.0, 12.0, 12.0, 12.0, 12.0, 13.0, 12.0, 12.0, 13.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [13.0, 11.0, 12.0, 13.0, 12.0, 11.0, 12.0, 12.0, 12.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0]]</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>[[171.67381543698417, 121.91060904702671, 145.6585137824614, 153.21305931525632, 131.79351506261247, 101.79753146907926, 144.20434380538205, 145.15285429284592, 169.02822720398967, 171.57082143390124], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [117.0671524124359, 86.84846978023653, 144.158379868197, 171.42811144601143, 199.67258146354172, 65.9627966957149, 144.85734474176556, 154.18804164564273, 160.2731231682561, 188.3833856349], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [169.16533358350605, 125.2512122003425, 124.36982905582596, 152.3431774421878, 164.55270315503893, 99.58614228205624, 138.9677058715599, 154.38699831564628, 167.33125598678217, 152.1864118047564], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [158.91879250547223, 109.34905424813742, 151.8325536909609, 152.68116070222248, 146.07804621145328, 106.86655881456286, 136.88045179693185, 154.13992758038017, 160.99605161933857, 179.23554052829246], [147.69556523473256, 119.61709997950122, 160.24986339852572, 151.8924649007107, 162.39451480720385, 107.1137112904901, 120.95681944842299, 150.01966305951794, 154.40819491054984, 158.87312273925517], [151.75926646509785, 109.8886301535245, 151.53074398765813, 156.40416673372965, 134.9951394547665, 121.13166969142071, 149.92145423768537, 153.96707325127616, 160.15394794087257, 173.79465689965093], [149.73435649974806, 109.66089149608842, 155.06539360124026, 172.89423563219376, 171.21374507309983, 98.03539136506976, 123.97995851126295, 151.2177782733371, 158.14025310250054, 174.9784724380392], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [154.87670501106774, 124.45712875915734, 159.00186930720025, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 149.50901730168147, 153.1866101146596, 155.4404734500336], [148.57242003247117, 115.00137686241824, 127.42349700300535, 153.358448411623, 169.82162012787782, 102.0493683148124, 140.3944107616491, 157.57071101559134, 169.1542118150403, 169.08558067012228], [118.9573278499153, 87.27566948350537, 141.8942472343372, 156.0887845439302, 215.99334155094448, 63.60144531528303, 141.586417049037, 156.4440274161946, 157.31476582791896, 185.21953219907152], [155.63356434101732, 121.7037973314125, 141.61047245367973, 128.56412415865336, 136.09008626574686, 141.05775541519452, 134.93095555474864, 125.91983083232476, 131.26261056343623, 182.36619594400247], [151.0530785897105, 100.13685713420632, 161.3782749695759, 158.82492821063502, 156.23168163705236, 98.31033969951382, 146.06938513288128, 146.66128011680243, 160.50369887210744, 191.8184134047504], [169.84163444520755, 123.3416986713996, 154.83107455194718, 167.98929163470268, 140.7932798872149, 101.68952014718067, 141.77615836031643, 146.55188089601023, 156.74047339913525, 163.36485909573406], [122.27088733454492, 109.20997405555539, 165.61688938660893, 170.33382062522801, 182.70092984366494, 107.97616157403853, 103.39739396512512, 145.35031470925776, 163.65926547880437, 160.94583046901406], [116.35505577055113, 114.1192854646577, 123.7609397041828, 160.69814808763311, 178.38382498160877, 68.98150340340261, 133.86332008334244, 146.19438482366462, 176.35573400668068, 183.52554229325003], [115.76525255456991, 91.80230503030586, 149.46566000403075, 164.23826817920266, 199.34751449005594, 96.97113934572377, 125.65836770040076, 139.29213316594414, 166.70626408889285, 158.4806267178086], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [123.72400459693046, 101.31380805074481, 135.26798136474852, 145.08457880992663, 200.86161538572605, 89.75116450662642, 120.30558500298024, 158.45816233102877, 174.8894098741557, 177.71466936907032], [149.27816962680123, 108.37247732346466, 138.71329142679446, 152.99701822494, 183.85670983256415, 98.26543736382182, 127.5550170615973, 153.75067512774277, 157.57839871208935, 183.54169965397787], [124.60931392388997, 99.55757900064643, 161.99929959628253, 150.1285082839572, 186.11983693459018, 86.00430019489998, 119.13204577034072, 155.41436252761594, 169.16448238826908, 170.3493231523084], [163.82826724191202, 123.63300303116105, 162.8980670120787, 166.58612468713937, 158.67319842829247, 101.19007738890186, 123.85647903797361, 141.86796497619403, 159.9811243798996, 158.63953984939445], [148.67533995564713, 108.42457729451831, 142.42838475310768, 157.76017755019018, 175.27052518344323, 98.69191696560306, 130.78580900589537, 150.57399766610484, 168.29287308414735, 176.59224756357847], [150.027945250437, 108.79702288668555, 146.15298522743862, 142.32196166402898, 181.20052992519373, 98.66945040809613, 133.44593232016487, 150.76253296723166, 155.14298179124637, 188.26268790756117], [148.67533995564713, 108.42457729451831, 142.42838475310768, 157.76017755019018, 175.27052518344323, 98.69191696560306, 130.78580900589537, 150.57399766610484, 168.29287308414735, 176.59224756357847], [117.75853219996374, 104.55487481547416, 145.71552532921476, 171.12163119570744, 154.03785309717847, 96.62628959763566, 143.01389905230988, 148.6565437698375, 165.84899302629753, 163.7556890865001], [168.85386525471753, 123.60444750594341, 137.40385276973333, 157.67445281251932, 156.92671983700316, 102.20671718726648, 137.71856360164185, 148.732299411782, 164.68903502507757, 166.26001663639278]]</t>
+          <t>[[143.21619887091217, 142.78166202391816, 155.6232838848781, 154.34080333205836, 137.56108536554407, 165.8993256716703, 165.09758144419533, 141.9934005720503, 137.7283623139118, 149.59126018489454], [162.58948838354567, 160.1226011636061, 139.82513626845264, 152.96758450801053, 135.12701938391612, 151.61013214277406, 150.493287248246, 134.85992711826094, 150.5984609100127, 150.12104645517394], [158.46583350604715, 143.94474980801536, 155.2264402096603, 148.59131176516215, 163.33510205433348, 143.13245211737618, 150.60010306170463, 128.1885347599593, 147.09184193162258, 156.2422810250139], [122.98992678619393, 139.24654249869775, 165.471693743431, 133.67393673571232, 176.97391216146974, 168.7508705311323, 166.71496501087327, 129.62898668843778, 134.0557936431074, 154.3350471696996], [107.13450481175435, 157.28556717351643, 133.74906034994123, 154.65666710454403, 133.88462131275145, 127.67422763197196, 149.3833883463211, 155.89581983178655, 137.70505024966664, 173.37870316221006]]</t>
         </is>
       </c>
     </row>
@@ -2410,14 +2410,14 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="E38" t="b">
         <v>1</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>11.37142857142857</t>
+          <t>12.000000000000002</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>144.1072860801123</t>
+          <t>149.02606457246125</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2437,12 +2437,12 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 11.0, 13.0, 10.0, 14.0, 10.0, 10.0, 14.0, 14.0, 14.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 13.0, 13.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 14.0, 10.0, 10.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [13.0, 10.0, 13.0, 16.0, 13.0, 10.0, 13.0, 17.0, 19.0, 16.0], [10.0, 11.0, 14.0, 14.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 13.0, 17.0, 10.0, 14.0, 17.0, 19.0, 17.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 14.0, 14.0, 14.0, 10.0, 10.0, 14.0, 14.0, 10.0], [10.0, 10.0, 13.0, 19.0, 16.0, 10.0, 13.0, 13.0, 19.0, 17.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 12.0, 13.0, 17.0, 10.0, 14.0, 18.0, 19.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 13.0, 18.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0]]</t>
+          <t>[[14.0, 14.0, 14.0, 15.0, 12.0, 13.0, 15.0, 15.0, 14.0, 14.0], [12.0, 12.0, 12.0, 12.0, 10.0, 12.0, 13.0, 12.0, 12.0, 13.0], [13.0, 12.0, 12.0, 13.0, 12.0, 12.0, 12.0, 12.0, 12.0, 10.0], [12.0, 13.0, 11.0, 10.0, 12.0, 12.0, 12.0, 12.0, 13.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0]]</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>[[171.67381543698417, 121.91060904702671, 145.6585137824614, 153.21305931525632, 131.79351506261247, 101.79753146907926, 144.20434380538205, 145.15285429284592, 169.02822720398967, 171.57082143390124], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [117.0671524124359, 86.84846978023653, 144.158379868197, 171.42811144601143, 199.67258146354172, 65.9627966957149, 144.85734474176556, 154.18804164564273, 160.2731231682561, 188.3833856349], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [169.16533358350605, 125.2512122003425, 124.36982905582596, 152.3431774421878, 164.55270315503893, 99.58614228205624, 138.9677058715599, 154.38699831564628, 167.33125598678217, 152.1864118047564], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [158.91879250547223, 109.34905424813742, 151.8325536909609, 152.68116070222248, 146.07804621145328, 106.86655881456286, 136.88045179693185, 154.13992758038017, 160.99605161933857, 179.23554052829246], [147.69556523473256, 119.61709997950122, 160.24986339852572, 151.8924649007107, 162.39451480720385, 107.1137112904901, 120.95681944842299, 150.01966305951794, 154.40819491054984, 158.87312273925517], [151.75926646509785, 109.8886301535245, 151.53074398765813, 156.40416673372965, 134.9951394547665, 121.13166969142071, 149.92145423768537, 153.96707325127616, 160.15394794087257, 173.79465689965093], [149.73435649974806, 109.66089149608842, 155.06539360124026, 172.89423563219376, 171.21374507309983, 98.03539136506976, 123.97995851126295, 151.2177782733371, 158.14025310250054, 174.9784724380392], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [154.87670501106774, 124.45712875915734, 159.00186930720025, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 149.50901730168147, 153.1866101146596, 155.4404734500336], [148.57242003247117, 115.00137686241824, 127.42349700300535, 153.358448411623, 169.82162012787782, 102.0493683148124, 140.3944107616491, 157.57071101559134, 169.1542118150403, 169.08558067012228], [118.9573278499153, 87.27566948350537, 141.8942472343372, 156.0887845439302, 215.99334155094448, 63.60144531528303, 141.586417049037, 156.4440274161946, 157.31476582791896, 185.21953219907152], [155.63356434101732, 121.7037973314125, 141.61047245367973, 128.56412415865336, 136.09008626574686, 141.05775541519452, 134.93095555474864, 125.91983083232476, 131.26261056343623, 182.36619594400247], [151.0530785897105, 100.13685713420632, 161.3782749695759, 158.82492821063502, 156.23168163705236, 98.31033969951382, 146.06938513288128, 146.66128011680243, 160.50369887210744, 191.8184134047504], [169.84163444520755, 123.3416986713996, 154.83107455194718, 167.98929163470268, 140.7932798872149, 101.68952014718067, 141.77615836031643, 146.55188089601023, 156.74047339913525, 163.36485909573406], [122.27088733454492, 109.20997405555539, 165.61688938660893, 170.33382062522801, 182.70092984366494, 107.97616157403853, 103.39739396512512, 145.35031470925776, 163.65926547880437, 160.94583046901406], [116.35505577055113, 114.1192854646577, 123.7609397041828, 160.69814808763311, 178.38382498160877, 68.98150340340261, 133.86332008334244, 146.19438482366462, 176.35573400668068, 183.52554229325003], [115.76525255456991, 91.80230503030586, 149.46566000403075, 164.23826817920266, 199.34751449005594, 96.97113934572377, 125.65836770040076, 139.29213316594414, 166.70626408889285, 158.4806267178086], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [123.72400459693046, 101.31380805074481, 135.26798136474852, 145.08457880992663, 200.86161538572605, 89.75116450662642, 120.30558500298024, 158.45816233102877, 174.8894098741557, 177.71466936907032], [149.27816962680123, 108.37247732346466, 138.71329142679446, 152.99701822494, 183.85670983256415, 98.26543736382182, 127.5550170615973, 153.75067512774277, 157.57839871208935, 183.54169965397787], [124.60931392388997, 99.55757900064643, 161.99929959628253, 150.1285082839572, 186.11983693459018, 86.00430019489998, 119.13204577034072, 155.41436252761594, 169.16448238826908, 170.3493231523084], [163.82826724191202, 123.63300303116105, 162.8980670120787, 166.58612468713937, 158.67319842829247, 101.19007738890186, 123.85647903797361, 141.86796497619403, 159.9811243798996, 158.63953984939445], [148.67533995564713, 108.42457729451831, 142.42838475310768, 157.76017755019018, 175.27052518344323, 98.69191696560306, 130.78580900589537, 150.57399766610484, 168.29287308414735, 176.59224756357847], [150.027945250437, 108.79702288668555, 146.15298522743862, 142.32196166402898, 181.20052992519373, 98.66945040809613, 133.44593232016487, 150.76253296723166, 155.14298179124637, 188.26268790756117], [148.67533995564713, 108.42457729451831, 142.42838475310768, 157.76017755019018, 175.27052518344323, 98.69191696560306, 130.78580900589537, 150.57399766610484, 168.29287308414735, 176.59224756357847], [117.75853219996374, 104.55487481547416, 145.71552532921476, 171.12163119570744, 154.03785309717847, 96.62628959763566, 143.01389905230988, 148.6565437698375, 165.84899302629753, 163.7556890865001], [168.85386525471753, 123.60444750594341, 137.40385276973333, 157.67445281251932, 156.92671983700316, 102.20671718726648, 137.71856360164185, 148.732299411782, 164.68903502507757, 166.26001663639278], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [124.60931392388997, 99.55757900064643, 161.99929959628253, 150.1285082839572, 186.11983693459018, 86.00430019489998, 119.13204577034072, 155.41436252761594, 169.16448238826908, 170.3493231523084], [149.27816962680123, 108.37247732346466, 138.71329142679446, 152.99701822494, 183.85670983256415, 98.26543736382182, 127.5550170615973, 153.75067512774277, 157.57839871208935, 183.54169965397787], [148.65858587031735, 117.5537430787448, 152.7370674658746, 155.0185002942349, 147.46163154928857, 129.97949714189932, 132.1733655775968, 150.43382549066143, 156.29210499732608, 168.29369368023086], [169.11123835390373, 122.6553643831684, 144.88497598512376, 148.40715049726467, 162.9523172779664, 100.41858968258288, 133.79930341502003, 156.57000045809946, 154.37301314092394, 169.3832824070351]]</t>
+          <t>[[111.44013158068762, 145.90763938850728, 152.33957542520798, 146.23861971647764, 166.80067170287577, 147.45211344017454, 155.98531315269585, 145.6350843638284, 148.0295776822259, 164.57394304434152], [155.56434747573292, 160.7363458106189, 154.4786615537434, 159.59151819951828, 146.71942863608987, 157.1102589336299, 142.28611883760388, 134.80546589070994, 130.7650224025433, 152.18210233735246], [147.0339283419166, 142.88191599871985, 158.41602937640417, 136.9536563764236, 164.48087375495342, 153.49877492649384, 148.9055033666255, 150.2021563933882, 152.8507122068979, 134.09848839339205], [157.24320556649093, 153.6784802874149, 134.40797648971326, 168.1112898888679, 151.86337330139474, 145.88038269247997, 154.20232347388614, 139.82673750098417, 133.4477556767396, 155.6757680395254], [117.10958822043081, 148.50043695935312, 161.18841530879132, 153.521240275286, 159.83849414822538, 162.876150016841, 141.1919618072483, 146.8612389453535, 138.16122468503178, 159.7532066292249]]</t>
         </is>
       </c>
     </row>
@@ -2463,14 +2463,14 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="E39" t="b">
         <v>1</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>11.25</t>
+          <t>11.200000000000001</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>143.95106242075457</t>
+          <t>148.6991087906081</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2490,12 +2490,12 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 11.0, 13.0, 10.0, 14.0, 10.0, 10.0, 14.0, 14.0, 14.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 13.0, 13.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 14.0, 10.0, 10.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [13.0, 10.0, 13.0, 16.0, 13.0, 10.0, 13.0, 17.0, 19.0, 16.0], [10.0, 11.0, 14.0, 14.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 13.0, 17.0, 10.0, 14.0, 17.0, 19.0, 17.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 14.0, 14.0, 14.0, 10.0, 10.0, 14.0, 14.0, 10.0], [10.0, 10.0, 13.0, 19.0, 16.0, 10.0, 13.0, 13.0, 19.0, 17.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 12.0, 13.0, 17.0, 10.0, 14.0, 18.0, 19.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 13.0, 18.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 14.0, 14.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0]]</t>
+          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [12.0, 15.0, 11.0, 16.0, 15.0, 13.0, 13.0, 15.0, 15.0, 15.0], [12.0, 12.0, 12.0, 12.0, 10.0, 13.0, 13.0, 12.0, 12.0, 12.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0]]</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>[[171.67381543698417, 121.91060904702671, 145.6585137824614, 153.21305931525632, 131.79351506261247, 101.79753146907926, 144.20434380538205, 145.15285429284592, 169.02822720398967, 171.57082143390124], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [117.0671524124359, 86.84846978023653, 144.158379868197, 171.42811144601143, 199.67258146354172, 65.9627966957149, 144.85734474176556, 154.18804164564273, 160.2731231682561, 188.3833856349], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [169.16533358350605, 125.2512122003425, 124.36982905582596, 152.3431774421878, 164.55270315503893, 99.58614228205624, 138.9677058715599, 154.38699831564628, 167.33125598678217, 152.1864118047564], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [158.91879250547223, 109.34905424813742, 151.8325536909609, 152.68116070222248, 146.07804621145328, 106.86655881456286, 136.88045179693185, 154.13992758038017, 160.99605161933857, 179.23554052829246], [147.69556523473256, 119.61709997950122, 160.24986339852572, 151.8924649007107, 162.39451480720385, 107.1137112904901, 120.95681944842299, 150.01966305951794, 154.40819491054984, 158.87312273925517], [151.75926646509785, 109.8886301535245, 151.53074398765813, 156.40416673372965, 134.9951394547665, 121.13166969142071, 149.92145423768537, 153.96707325127616, 160.15394794087257, 173.79465689965093], [149.73435649974806, 109.66089149608842, 155.06539360124026, 172.89423563219376, 171.21374507309983, 98.03539136506976, 123.97995851126295, 151.2177782733371, 158.14025310250054, 174.9784724380392], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [154.87670501106774, 124.45712875915734, 159.00186930720025, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 149.50901730168147, 153.1866101146596, 155.4404734500336], [148.57242003247117, 115.00137686241824, 127.42349700300535, 153.358448411623, 169.82162012787782, 102.0493683148124, 140.3944107616491, 157.57071101559134, 169.1542118150403, 169.08558067012228], [118.9573278499153, 87.27566948350537, 141.8942472343372, 156.0887845439302, 215.99334155094448, 63.60144531528303, 141.586417049037, 156.4440274161946, 157.31476582791896, 185.21953219907152], [155.63356434101732, 121.7037973314125, 141.61047245367973, 128.56412415865336, 136.09008626574686, 141.05775541519452, 134.93095555474864, 125.91983083232476, 131.26261056343623, 182.36619594400247], [151.0530785897105, 100.13685713420632, 161.3782749695759, 158.82492821063502, 156.23168163705236, 98.31033969951382, 146.06938513288128, 146.66128011680243, 160.50369887210744, 191.8184134047504], [169.84163444520755, 123.3416986713996, 154.83107455194718, 167.98929163470268, 140.7932798872149, 101.68952014718067, 141.77615836031643, 146.55188089601023, 156.74047339913525, 163.36485909573406], [122.27088733454492, 109.20997405555539, 165.61688938660893, 170.33382062522801, 182.70092984366494, 107.97616157403853, 103.39739396512512, 145.35031470925776, 163.65926547880437, 160.94583046901406], [116.35505577055113, 114.1192854646577, 123.7609397041828, 160.69814808763311, 178.38382498160877, 68.98150340340261, 133.86332008334244, 146.19438482366462, 176.35573400668068, 183.52554229325003], [115.76525255456991, 91.80230503030586, 149.46566000403075, 164.23826817920266, 199.34751449005594, 96.97113934572377, 125.65836770040076, 139.29213316594414, 166.70626408889285, 158.4806267178086], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [123.72400459693046, 101.31380805074481, 135.26798136474852, 145.08457880992663, 200.86161538572605, 89.75116450662642, 120.30558500298024, 158.45816233102877, 174.8894098741557, 177.71466936907032], [149.27816962680123, 108.37247732346466, 138.71329142679446, 152.99701822494, 183.85670983256415, 98.26543736382182, 127.5550170615973, 153.75067512774277, 157.57839871208935, 183.54169965397787], [124.60931392388997, 99.55757900064643, 161.99929959628253, 150.1285082839572, 186.11983693459018, 86.00430019489998, 119.13204577034072, 155.41436252761594, 169.16448238826908, 170.3493231523084], [163.82826724191202, 123.63300303116105, 162.8980670120787, 166.58612468713937, 158.67319842829247, 101.19007738890186, 123.85647903797361, 141.86796497619403, 159.9811243798996, 158.63953984939445], [148.67533995564713, 108.42457729451831, 142.42838475310768, 157.76017755019018, 175.27052518344323, 98.69191696560306, 130.78580900589537, 150.57399766610484, 168.29287308414735, 176.59224756357847], [150.027945250437, 108.79702288668555, 146.15298522743862, 142.32196166402898, 181.20052992519373, 98.66945040809613, 133.44593232016487, 150.76253296723166, 155.14298179124637, 188.26268790756117], [148.67533995564713, 108.42457729451831, 142.42838475310768, 157.76017755019018, 175.27052518344323, 98.69191696560306, 130.78580900589537, 150.57399766610484, 168.29287308414735, 176.59224756357847], [117.75853219996374, 104.55487481547416, 145.71552532921476, 171.12163119570744, 154.03785309717847, 96.62628959763566, 143.01389905230988, 148.6565437698375, 165.84899302629753, 163.7556890865001], [168.85386525471753, 123.60444750594341, 137.40385276973333, 157.67445281251932, 156.92671983700316, 102.20671718726648, 137.71856360164185, 148.732299411782, 164.68903502507757, 166.26001663639278], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [124.60931392388997, 99.55757900064643, 161.99929959628253, 150.1285082839572, 186.11983693459018, 86.00430019489998, 119.13204577034072, 155.41436252761594, 169.16448238826908, 170.3493231523084], [149.27816962680123, 108.37247732346466, 138.71329142679446, 152.99701822494, 183.85670983256415, 98.26543736382182, 127.5550170615973, 153.75067512774277, 157.57839871208935, 183.54169965397787], [148.65858587031735, 117.5537430787448, 152.7370674658746, 155.0185002942349, 147.46163154928857, 129.97949714189932, 132.1733655775968, 150.43382549066143, 156.29210499732608, 168.29369368023086], [169.11123835390373, 122.6553643831684, 144.88497598512376, 148.40715049726467, 162.9523172779664, 100.41858968258288, 133.79930341502003, 156.57000045809946, 154.37301314092394, 169.3832824070351], [122.27088733454492, 109.20997405555539, 165.61688938660893, 170.33382062522801, 182.70092984366494, 107.97616157403853, 103.39739396512512, 145.35031470925776, 163.65926547880437, 160.94583046901406], [173.98158099973762, 121.41401484854968, 155.2467272053208, 161.62490708015008, 139.23687798531955, 102.66460567234407, 139.44735831850167, 133.4012159187808, 173.97371251361338, 159.06106997603828], [119.41894344108162, 89.6361386782091, 144.86306350872732, 165.1607863571104, 211.6367393571435, 67.17495721088726, 127.51666835624646, 156.22666357481478, 168.0842230731582, 174.34523059533836], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [155.63356434101732, 121.7037973314125, 141.61047245367973, 128.56412415865336, 136.09008626574686, 141.05775541519452, 134.93095555474864, 125.91983083232476, 131.26261056343623, 182.36619594400247]]</t>
+          <t>[[153.99095802287687, 162.79185562240343, 157.84289886579248, 159.44203287324362, 132.21500709985602, 151.4488419777103, 147.43432541275112, 143.0962574468172, 144.47920002983372, 141.7500970510019], [135.20763106226153, 168.28130903161863, 146.7575476919731, 152.82421195914011, 151.86965831439346, 163.81824359943482, 144.87481342671188, 121.36687704291863, 139.02090446796865, 162.6257127631833], [141.04244203284907, 167.61386115453595, 131.04977561307172, 144.4305146749665, 154.3936525220863, 150.26576922358834, 149.09457610844646, 144.4518472357404, 159.34560224586585, 148.11166736061838], [144.28802916845027, 154.78839624546427, 165.7701148768861, 152.85001347852068, 119.02008846980081, 159.88141680936837, 143.56561119113078, 156.87635470323482, 145.24614813602102, 149.93350236424405], [138.42146213702762, 145.80988933370597, 165.94317476807996, 163.21851009861774, 127.929210490825, 149.45392294347724, 183.3923805433234, 117.92739903926497, 130.33493551620165, 149.36678728309977]]</t>
         </is>
       </c>
     </row>
@@ -2516,14 +2516,14 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E40" t="b">
         <v>1</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>11.288888888888888</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>143.98979747762107</t>
+          <t>148.10692086634887</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2543,12 +2543,12 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 11.0, 13.0, 10.0, 14.0, 10.0, 10.0, 14.0, 14.0, 14.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 13.0, 13.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 14.0, 10.0, 10.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [13.0, 10.0, 13.0, 16.0, 13.0, 10.0, 13.0, 17.0, 19.0, 16.0], [10.0, 11.0, 14.0, 14.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 13.0, 17.0, 10.0, 14.0, 17.0, 19.0, 17.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 14.0, 14.0, 14.0, 10.0, 10.0, 14.0, 14.0, 10.0], [10.0, 10.0, 13.0, 19.0, 16.0, 10.0, 13.0, 13.0, 19.0, 17.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 12.0, 13.0, 17.0, 10.0, 14.0, 18.0, 19.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 13.0, 18.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 14.0, 14.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 13.0, 14.0, 10.0, 10.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 14.0, 13.0, 14.0, 10.0, 10.0, 10.0, 15.0, 14.0]]</t>
+          <t>[[13.0, 11.0, 12.0, 12.0, 12.0, 11.0, 12.0, 12.0, 13.0, 12.0], [13.0, 13.0, 12.0, 11.0, 12.0, 11.0, 13.0, 11.0, 12.0, 12.0], [13.0, 10.0, 13.0, 11.0, 12.0, 12.0, 12.0, 13.0, 12.0, 12.0], [13.0, 13.0, 10.0, 12.0, 13.0, 12.0, 12.0, 12.0, 13.0, 10.0], [10.0, 15.0, 14.0, 14.0, 10.0, 14.0, 13.0, 10.0, 10.0, 10.0]]</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>[[171.67381543698417, 121.91060904702671, 145.6585137824614, 153.21305931525632, 131.79351506261247, 101.79753146907926, 144.20434380538205, 145.15285429284592, 169.02822720398967, 171.57082143390124], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [117.0671524124359, 86.84846978023653, 144.158379868197, 171.42811144601143, 199.67258146354172, 65.9627966957149, 144.85734474176556, 154.18804164564273, 160.2731231682561, 188.3833856349], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [169.16533358350605, 125.2512122003425, 124.36982905582596, 152.3431774421878, 164.55270315503893, 99.58614228205624, 138.9677058715599, 154.38699831564628, 167.33125598678217, 152.1864118047564], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [158.91879250547223, 109.34905424813742, 151.8325536909609, 152.68116070222248, 146.07804621145328, 106.86655881456286, 136.88045179693185, 154.13992758038017, 160.99605161933857, 179.23554052829246], [147.69556523473256, 119.61709997950122, 160.24986339852572, 151.8924649007107, 162.39451480720385, 107.1137112904901, 120.95681944842299, 150.01966305951794, 154.40819491054984, 158.87312273925517], [151.75926646509785, 109.8886301535245, 151.53074398765813, 156.40416673372965, 134.9951394547665, 121.13166969142071, 149.92145423768537, 153.96707325127616, 160.15394794087257, 173.79465689965093], [149.73435649974806, 109.66089149608842, 155.06539360124026, 172.89423563219376, 171.21374507309983, 98.03539136506976, 123.97995851126295, 151.2177782733371, 158.14025310250054, 174.9784724380392], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [154.87670501106774, 124.45712875915734, 159.00186930720025, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 149.50901730168147, 153.1866101146596, 155.4404734500336], [148.57242003247117, 115.00137686241824, 127.42349700300535, 153.358448411623, 169.82162012787782, 102.0493683148124, 140.3944107616491, 157.57071101559134, 169.1542118150403, 169.08558067012228], [118.9573278499153, 87.27566948350537, 141.8942472343372, 156.0887845439302, 215.99334155094448, 63.60144531528303, 141.586417049037, 156.4440274161946, 157.31476582791896, 185.21953219907152], [155.63356434101732, 121.7037973314125, 141.61047245367973, 128.56412415865336, 136.09008626574686, 141.05775541519452, 134.93095555474864, 125.91983083232476, 131.26261056343623, 182.36619594400247], [151.0530785897105, 100.13685713420632, 161.3782749695759, 158.82492821063502, 156.23168163705236, 98.31033969951382, 146.06938513288128, 146.66128011680243, 160.50369887210744, 191.8184134047504], [169.84163444520755, 123.3416986713996, 154.83107455194718, 167.98929163470268, 140.7932798872149, 101.68952014718067, 141.77615836031643, 146.55188089601023, 156.74047339913525, 163.36485909573406], [122.27088733454492, 109.20997405555539, 165.61688938660893, 170.33382062522801, 182.70092984366494, 107.97616157403853, 103.39739396512512, 145.35031470925776, 163.65926547880437, 160.94583046901406], [116.35505577055113, 114.1192854646577, 123.7609397041828, 160.69814808763311, 178.38382498160877, 68.98150340340261, 133.86332008334244, 146.19438482366462, 176.35573400668068, 183.52554229325003], [115.76525255456991, 91.80230503030586, 149.46566000403075, 164.23826817920266, 199.34751449005594, 96.97113934572377, 125.65836770040076, 139.29213316594414, 166.70626408889285, 158.4806267178086], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [123.72400459693046, 101.31380805074481, 135.26798136474852, 145.08457880992663, 200.86161538572605, 89.75116450662642, 120.30558500298024, 158.45816233102877, 174.8894098741557, 177.71466936907032], [149.27816962680123, 108.37247732346466, 138.71329142679446, 152.99701822494, 183.85670983256415, 98.26543736382182, 127.5550170615973, 153.75067512774277, 157.57839871208935, 183.54169965397787], [124.60931392388997, 99.55757900064643, 161.99929959628253, 150.1285082839572, 186.11983693459018, 86.00430019489998, 119.13204577034072, 155.41436252761594, 169.16448238826908, 170.3493231523084], [163.82826724191202, 123.63300303116105, 162.8980670120787, 166.58612468713937, 158.67319842829247, 101.19007738890186, 123.85647903797361, 141.86796497619403, 159.9811243798996, 158.63953984939445], [148.67533995564713, 108.42457729451831, 142.42838475310768, 157.76017755019018, 175.27052518344323, 98.69191696560306, 130.78580900589537, 150.57399766610484, 168.29287308414735, 176.59224756357847], [150.027945250437, 108.79702288668555, 146.15298522743862, 142.32196166402898, 181.20052992519373, 98.66945040809613, 133.44593232016487, 150.76253296723166, 155.14298179124637, 188.26268790756117], [148.67533995564713, 108.42457729451831, 142.42838475310768, 157.76017755019018, 175.27052518344323, 98.69191696560306, 130.78580900589537, 150.57399766610484, 168.29287308414735, 176.59224756357847], [117.75853219996374, 104.55487481547416, 145.71552532921476, 171.12163119570744, 154.03785309717847, 96.62628959763566, 143.01389905230988, 148.6565437698375, 165.84899302629753, 163.7556890865001], [168.85386525471753, 123.60444750594341, 137.40385276973333, 157.67445281251932, 156.92671983700316, 102.20671718726648, 137.71856360164185, 148.732299411782, 164.68903502507757, 166.26001663639278], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [124.60931392388997, 99.55757900064643, 161.99929959628253, 150.1285082839572, 186.11983693459018, 86.00430019489998, 119.13204577034072, 155.41436252761594, 169.16448238826908, 170.3493231523084], [149.27816962680123, 108.37247732346466, 138.71329142679446, 152.99701822494, 183.85670983256415, 98.26543736382182, 127.5550170615973, 153.75067512774277, 157.57839871208935, 183.54169965397787], [148.65858587031735, 117.5537430787448, 152.7370674658746, 155.0185002942349, 147.46163154928857, 129.97949714189932, 132.1733655775968, 150.43382549066143, 156.29210499732608, 168.29369368023086], [169.11123835390373, 122.6553643831684, 144.88497598512376, 148.40715049726467, 162.9523172779664, 100.41858968258288, 133.79930341502003, 156.57000045809946, 154.37301314092394, 169.3832824070351], [122.27088733454492, 109.20997405555539, 165.61688938660893, 170.33382062522801, 182.70092984366494, 107.97616157403853, 103.39739396512512, 145.35031470925776, 163.65926547880437, 160.94583046901406], [173.98158099973762, 121.41401484854968, 155.2467272053208, 161.62490708015008, 139.23687798531955, 102.66460567234407, 139.44735831850167, 133.4012159187808, 173.97371251361338, 159.06106997603828], [119.41894344108162, 89.6361386782091, 144.86306350872732, 165.1607863571104, 211.6367393571435, 67.17495721088726, 127.51666835624646, 156.22666357481478, 168.0842230731582, 174.34523059533836], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [155.63356434101732, 121.7037973314125, 141.61047245367973, 128.56412415865336, 136.09008626574686, 141.05775541519452, 134.93095555474864, 125.91983083232476, 131.26261056343623, 182.36619594400247], [146.18299237104432, 117.20105605174287, 126.9403685025021, 145.15044742546544, 168.3740185570338, 124.3244416636751, 128.32106677125984, 154.36131283034118, 170.5636407527166, 167.50903583812456], [181.393153961203, 136.65303694070522, 125.90506986307487, 151.23293415828567, 167.04522306488312, 103.96871006288565, 114.83430969632307, 159.04491127509579, 144.68189566301348, 131.87396315470303], [148.95420164834556, 102.41615587257776, 146.08091617104404, 143.6583501834782, 166.8856957427277, 104.25030634694905, 152.5036957947207, 149.91289442177094, 156.3036270071304, 191.01691397117983], [154.2340739641886, 120.83138478017217, 163.1793401868486, 160.31358068613486, 148.47839537340548, 117.1670246238789, 123.45996093277371, 154.16491696465175, 160.79963802966617, 156.97009997029812], [119.62309438448534, 90.435441749757, 143.33997457038888, 154.93751677485346, 225.34053642990904, 62.19288437268095, 128.31268015184958, 149.14552095531636, 162.8014528319032, 191.71203313048701]]</t>
+          <t>[[142.57613009339005, 147.20156844703385, 155.19336680362616, 161.21876753020504, 154.67046812860465, 138.47340573660483, 159.26429070874022, 122.65164891645928, 153.7070032455291, 155.8364535291869], [164.0985689239849, 160.05711658510708, 159.02345568208693, 132.1005211092795, 159.7958136379369, 144.3355278680992, 148.44240113818515, 112.57688911343298, 156.59256523794488, 154.09583511816817], [150.51147902246043, 150.90185220452213, 158.5042758106092, 124.55917177116149, 149.04914128703336, 170.04827664658572, 170.22235043124635, 136.0745386340964, 131.1700865318803, 147.00017378399613], [149.0912181205517, 162.00295320876677, 137.28401685610365, 160.39473467860086, 165.33208234822388, 157.81947336596826, 156.5212124788176, 142.0828142857634, 140.6249327519648, 121.05212479299784], [146.74048524902142, 158.2707010110014, 157.64151499983566, 156.81901403998555, 123.59583082961886, 167.42798877684157, 149.9232016812982, 108.15429389700161, 142.32134152798858, 132.29296473989444]]</t>
         </is>
       </c>
     </row>
@@ -2569,14 +2569,14 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="E41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>11.36</t>
+          <t>14.0</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>144.0548587481977</t>
+          <t>146.7455087620421</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2596,12 +2596,12 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 11.0, 13.0, 10.0, 14.0, 10.0, 10.0, 14.0, 14.0, 14.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 13.0, 13.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 14.0, 10.0, 10.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [13.0, 10.0, 13.0, 16.0, 13.0, 10.0, 13.0, 17.0, 19.0, 16.0], [10.0, 11.0, 14.0, 14.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 13.0, 17.0, 10.0, 14.0, 17.0, 19.0, 17.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 14.0, 14.0, 14.0, 10.0, 10.0, 14.0, 14.0, 10.0], [10.0, 10.0, 13.0, 19.0, 16.0, 10.0, 13.0, 13.0, 19.0, 17.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 12.0, 13.0, 17.0, 10.0, 14.0, 18.0, 19.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 13.0, 18.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 14.0, 14.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 13.0, 14.0, 10.0, 10.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 14.0, 13.0, 14.0, 10.0, 10.0, 10.0, 15.0, 14.0], [10.0, 13.0, 13.0, 13.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 13.0, 14.0, 10.0, 10.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 14.0, 15.0, 14.0, 10.0, 10.0, 10.0, 14.0, 13.0]]</t>
+          <t>[[15.0, 12.0, 14.0, 15.0, 16.0, 13.0, 15.0, 14.0, 14.0, 12.0], [13.0, 12.0, 17.0, 16.0, 14.0, 11.0, 15.0, 14.0, 14.0, 14.0], [15.0, 15.0, 12.0, 15.0, 12.0, 14.0, 14.0, 14.0, 15.0, 14.0], [19.0, 22.0, 10.0, 10.0, 10.0, 17.0, 14.0, 10.0, 10.0, 18.0], [16.0, 14.0, 10.0, 16.0, 14.0, 10.0, 10.0, 10.0, 20.0, 20.0]]</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>[[171.67381543698417, 121.91060904702671, 145.6585137824614, 153.21305931525632, 131.79351506261247, 101.79753146907926, 144.20434380538205, 145.15285429284592, 169.02822720398967, 171.57082143390124], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [117.0671524124359, 86.84846978023653, 144.158379868197, 171.42811144601143, 199.67258146354172, 65.9627966957149, 144.85734474176556, 154.18804164564273, 160.2731231682561, 188.3833856349], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [169.16533358350605, 125.2512122003425, 124.36982905582596, 152.3431774421878, 164.55270315503893, 99.58614228205624, 138.9677058715599, 154.38699831564628, 167.33125598678217, 152.1864118047564], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [158.91879250547223, 109.34905424813742, 151.8325536909609, 152.68116070222248, 146.07804621145328, 106.86655881456286, 136.88045179693185, 154.13992758038017, 160.99605161933857, 179.23554052829246], [147.69556523473256, 119.61709997950122, 160.24986339852572, 151.8924649007107, 162.39451480720385, 107.1137112904901, 120.95681944842299, 150.01966305951794, 154.40819491054984, 158.87312273925517], [151.75926646509785, 109.8886301535245, 151.53074398765813, 156.40416673372965, 134.9951394547665, 121.13166969142071, 149.92145423768537, 153.96707325127616, 160.15394794087257, 173.79465689965093], [149.73435649974806, 109.66089149608842, 155.06539360124026, 172.89423563219376, 171.21374507309983, 98.03539136506976, 123.97995851126295, 151.2177782733371, 158.14025310250054, 174.9784724380392], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [154.87670501106774, 124.45712875915734, 159.00186930720025, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 149.50901730168147, 153.1866101146596, 155.4404734500336], [148.57242003247117, 115.00137686241824, 127.42349700300535, 153.358448411623, 169.82162012787782, 102.0493683148124, 140.3944107616491, 157.57071101559134, 169.1542118150403, 169.08558067012228], [118.9573278499153, 87.27566948350537, 141.8942472343372, 156.0887845439302, 215.99334155094448, 63.60144531528303, 141.586417049037, 156.4440274161946, 157.31476582791896, 185.21953219907152], [155.63356434101732, 121.7037973314125, 141.61047245367973, 128.56412415865336, 136.09008626574686, 141.05775541519452, 134.93095555474864, 125.91983083232476, 131.26261056343623, 182.36619594400247], [151.0530785897105, 100.13685713420632, 161.3782749695759, 158.82492821063502, 156.23168163705236, 98.31033969951382, 146.06938513288128, 146.66128011680243, 160.50369887210744, 191.8184134047504], [169.84163444520755, 123.3416986713996, 154.83107455194718, 167.98929163470268, 140.7932798872149, 101.68952014718067, 141.77615836031643, 146.55188089601023, 156.74047339913525, 163.36485909573406], [122.27088733454492, 109.20997405555539, 165.61688938660893, 170.33382062522801, 182.70092984366494, 107.97616157403853, 103.39739396512512, 145.35031470925776, 163.65926547880437, 160.94583046901406], [116.35505577055113, 114.1192854646577, 123.7609397041828, 160.69814808763311, 178.38382498160877, 68.98150340340261, 133.86332008334244, 146.19438482366462, 176.35573400668068, 183.52554229325003], [115.76525255456991, 91.80230503030586, 149.46566000403075, 164.23826817920266, 199.34751449005594, 96.97113934572377, 125.65836770040076, 139.29213316594414, 166.70626408889285, 158.4806267178086], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [123.72400459693046, 101.31380805074481, 135.26798136474852, 145.08457880992663, 200.86161538572605, 89.75116450662642, 120.30558500298024, 158.45816233102877, 174.8894098741557, 177.71466936907032], [149.27816962680123, 108.37247732346466, 138.71329142679446, 152.99701822494, 183.85670983256415, 98.26543736382182, 127.5550170615973, 153.75067512774277, 157.57839871208935, 183.54169965397787], [124.60931392388997, 99.55757900064643, 161.99929959628253, 150.1285082839572, 186.11983693459018, 86.00430019489998, 119.13204577034072, 155.41436252761594, 169.16448238826908, 170.3493231523084], [163.82826724191202, 123.63300303116105, 162.8980670120787, 166.58612468713937, 158.67319842829247, 101.19007738890186, 123.85647903797361, 141.86796497619403, 159.9811243798996, 158.63953984939445], [148.67533995564713, 108.42457729451831, 142.42838475310768, 157.76017755019018, 175.27052518344323, 98.69191696560306, 130.78580900589537, 150.57399766610484, 168.29287308414735, 176.59224756357847], [150.027945250437, 108.79702288668555, 146.15298522743862, 142.32196166402898, 181.20052992519373, 98.66945040809613, 133.44593232016487, 150.76253296723166, 155.14298179124637, 188.26268790756117], [148.67533995564713, 108.42457729451831, 142.42838475310768, 157.76017755019018, 175.27052518344323, 98.69191696560306, 130.78580900589537, 150.57399766610484, 168.29287308414735, 176.59224756357847], [117.75853219996374, 104.55487481547416, 145.71552532921476, 171.12163119570744, 154.03785309717847, 96.62628959763566, 143.01389905230988, 148.6565437698375, 165.84899302629753, 163.7556890865001], [168.85386525471753, 123.60444750594341, 137.40385276973333, 157.67445281251932, 156.92671983700316, 102.20671718726648, 137.71856360164185, 148.732299411782, 164.68903502507757, 166.26001663639278], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [124.60931392388997, 99.55757900064643, 161.99929959628253, 150.1285082839572, 186.11983693459018, 86.00430019489998, 119.13204577034072, 155.41436252761594, 169.16448238826908, 170.3493231523084], [149.27816962680123, 108.37247732346466, 138.71329142679446, 152.99701822494, 183.85670983256415, 98.26543736382182, 127.5550170615973, 153.75067512774277, 157.57839871208935, 183.54169965397787], [148.65858587031735, 117.5537430787448, 152.7370674658746, 155.0185002942349, 147.46163154928857, 129.97949714189932, 132.1733655775968, 150.43382549066143, 156.29210499732608, 168.29369368023086], [169.11123835390373, 122.6553643831684, 144.88497598512376, 148.40715049726467, 162.9523172779664, 100.41858968258288, 133.79930341502003, 156.57000045809946, 154.37301314092394, 169.3832824070351], [122.27088733454492, 109.20997405555539, 165.61688938660893, 170.33382062522801, 182.70092984366494, 107.97616157403853, 103.39739396512512, 145.35031470925776, 163.65926547880437, 160.94583046901406], [173.98158099973762, 121.41401484854968, 155.2467272053208, 161.62490708015008, 139.23687798531955, 102.66460567234407, 139.44735831850167, 133.4012159187808, 173.97371251361338, 159.06106997603828], [119.41894344108162, 89.6361386782091, 144.86306350872732, 165.1607863571104, 211.6367393571435, 67.17495721088726, 127.51666835624646, 156.22666357481478, 168.0842230731582, 174.34523059533836], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [155.63356434101732, 121.7037973314125, 141.61047245367973, 128.56412415865336, 136.09008626574686, 141.05775541519452, 134.93095555474864, 125.91983083232476, 131.26261056343623, 182.36619594400247], [146.18299237104432, 117.20105605174287, 126.9403685025021, 145.15044742546544, 168.3740185570338, 124.3244416636751, 128.32106677125984, 154.36131283034118, 170.5636407527166, 167.50903583812456], [181.393153961203, 136.65303694070522, 125.90506986307487, 151.23293415828567, 167.04522306488312, 103.96871006288565, 114.83430969632307, 159.04491127509579, 144.68189566301348, 131.87396315470303], [148.95420164834556, 102.41615587257776, 146.08091617104404, 143.6583501834782, 166.8856957427277, 104.25030634694905, 152.5036957947207, 149.91289442177094, 156.3036270071304, 191.01691397117983], [154.2340739641886, 120.83138478017217, 163.1793401868486, 160.31358068613486, 148.47839537340548, 117.1670246238789, 123.45996093277371, 154.16491696465175, 160.79963802966617, 156.97009997029812], [119.62309438448534, 90.435441749757, 143.33997457038888, 154.93751677485346, 225.34053642990904, 62.19288437268095, 128.31268015184958, 149.14552095531636, 162.8014528319032, 191.71203313048701], [148.48479676441337, 126.21029578037393, 159.62527053798442, 150.8061319125178, 153.23293437543683, 119.63764321443003, 128.4032854786844, 149.37101807759663, 152.58048638924546, 152.88482163934412], [148.67533995564713, 108.42457729451831, 142.42838475310768, 157.76017755019018, 175.27052518344323, 98.69191696560306, 130.78580900589537, 150.57399766610484, 168.29287308414735, 176.59224756357847], [149.06216452946686, 106.48162668769525, 151.4162018926752, 152.32082662555626, 143.9027578301337, 123.58902848907663, 145.9721620405975, 153.7559937174116, 162.32183464471146, 171.55119884108467], [138.20605623854652, 107.42348781850717, 129.21584774205314, 142.2134787300486, 192.8664244086329, 96.20732846975696, 131.92385143024265, 156.3132038929684, 172.34092474542578, 184.7627903630174], [154.25124766900188, 130.41874324998875, 125.82420113609076, 156.97943007117505, 157.16274510072986, 126.51035377237639, 131.08744654012494, 159.55495885505314, 143.6280207101792, 136.0236397347833]]</t>
+          <t>[[141.3158430871751, 130.54228345970913, 164.39025357347245, 152.67593871446536, 153.62559550399877, 142.7404924911546, 162.13055969570385, 156.12770517112585, 139.01768007621587, 150.24445826717405], [134.82765317680915, 150.8901233740006, 164.9147229479346, 137.4487275759327, 173.31509591434605, 152.93245868186966, 157.88501014486346, 116.2274887452356, 135.73807411487795, 168.76191695031343], [153.71840673025517, 162.1002936953527, 141.7994967485494, 135.24455474175363, 142.88423190341095, 145.23056062122623, 158.86221378122488, 150.83550049185467, 133.7663624252267, 150.38555701131588], [190.1957446247918, 167.35036359251617, 135.86645534121476, 116.76151855957634, 153.0754578068192, 142.56842819744813, 122.0745877054018, 151.21718443446258, 116.99745441517337, 148.16110751369337], [154.72856407520013, 144.70585944630298, 83.9497176271272, 144.10411506456086, 144.69220014990339, 152.4102047857733, 144.75204042632956, 113.8160582630052, 169.61336084724786, 179.65575540900986]]</t>
         </is>
       </c>
     </row>
@@ -2622,14 +2622,14 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="E42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>11.309090909090909</t>
+          <t>14.0</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2639,7 +2639,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>143.90779359024936</t>
+          <t>147.19539265052668</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2649,12 +2649,12 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 11.0, 13.0, 10.0, 14.0, 10.0, 10.0, 14.0, 14.0, 14.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 13.0, 13.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 14.0, 10.0, 10.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [13.0, 10.0, 13.0, 16.0, 13.0, 10.0, 13.0, 17.0, 19.0, 16.0], [10.0, 11.0, 14.0, 14.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 13.0, 13.0, 17.0, 10.0, 14.0, 17.0, 19.0, 17.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 14.0, 14.0, 14.0, 10.0, 10.0, 14.0, 14.0, 10.0], [10.0, 10.0, 13.0, 19.0, 16.0, 10.0, 13.0, 13.0, 19.0, 17.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 12.0, 13.0, 17.0, 10.0, 14.0, 18.0, 19.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 13.0, 18.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 14.0, 14.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 13.0, 14.0, 10.0, 10.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 14.0, 13.0, 14.0, 10.0, 10.0, 10.0, 15.0, 14.0], [10.0, 13.0, 13.0, 13.0, 14.0, 10.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 13.0, 14.0, 10.0, 10.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 10.0, 13.0, 13.0, 10.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 14.0, 15.0, 14.0, 10.0, 10.0, 10.0, 14.0, 13.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0, 10.0], [10.0, 10.0, 12.0, 13.0, 16.0, 10.0, 14.0, 18.0, 20.0, 17.0]]</t>
+          <t>[[16.0, 13.0, 15.0, 12.0, 14.0, 15.0, 13.0, 15.0, 12.0, 15.0], [14.0, 16.0, 14.0, 12.0, 14.0, 14.0, 16.0, 14.0, 14.0, 12.0], [16.0, 16.0, 14.0, 14.0, 12.0, 14.0, 14.0, 12.0, 16.0, 12.0], [14.0, 16.0, 15.0, 13.0, 15.0, 14.0, 14.0, 13.0, 13.0, 13.0], [16.0, 22.0, 10.0, 15.0, 10.0, 11.0, 14.0, 12.0, 16.0, 14.0]]</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>[[171.67381543698417, 121.91060904702671, 145.6585137824614, 153.21305931525632, 131.79351506261247, 101.79753146907926, 144.20434380538205, 145.15285429284592, 169.02822720398967, 171.57082143390124], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [117.0671524124359, 86.84846978023653, 144.158379868197, 171.42811144601143, 199.67258146354172, 65.9627966957149, 144.85734474176556, 154.18804164564273, 160.2731231682561, 188.3833856349], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [169.16533358350605, 125.2512122003425, 124.36982905582596, 152.3431774421878, 164.55270315503893, 99.58614228205624, 138.9677058715599, 154.38699831564628, 167.33125598678217, 152.1864118047564], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [158.91879250547223, 109.34905424813742, 151.8325536909609, 152.68116070222248, 146.07804621145328, 106.86655881456286, 136.88045179693185, 154.13992758038017, 160.99605161933857, 179.23554052829246], [147.69556523473256, 119.61709997950122, 160.24986339852572, 151.8924649007107, 162.39451480720385, 107.1137112904901, 120.95681944842299, 150.01966305951794, 154.40819491054984, 158.87312273925517], [151.75926646509785, 109.8886301535245, 151.53074398765813, 156.40416673372965, 134.9951394547665, 121.13166969142071, 149.92145423768537, 153.96707325127616, 160.15394794087257, 173.79465689965093], [149.73435649974806, 109.66089149608842, 155.06539360124026, 172.89423563219376, 171.21374507309983, 98.03539136506976, 123.97995851126295, 151.2177782733371, 158.14025310250054, 174.9784724380392], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [154.87670501106774, 124.45712875915734, 159.00186930720025, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 149.50901730168147, 153.1866101146596, 155.4404734500336], [148.57242003247117, 115.00137686241824, 127.42349700300535, 153.358448411623, 169.82162012787782, 102.0493683148124, 140.3944107616491, 157.57071101559134, 169.1542118150403, 169.08558067012228], [118.9573278499153, 87.27566948350537, 141.8942472343372, 156.0887845439302, 215.99334155094448, 63.60144531528303, 141.586417049037, 156.4440274161946, 157.31476582791896, 185.21953219907152], [155.63356434101732, 121.7037973314125, 141.61047245367973, 128.56412415865336, 136.09008626574686, 141.05775541519452, 134.93095555474864, 125.91983083232476, 131.26261056343623, 182.36619594400247], [151.0530785897105, 100.13685713420632, 161.3782749695759, 158.82492821063502, 156.23168163705236, 98.31033969951382, 146.06938513288128, 146.66128011680243, 160.50369887210744, 191.8184134047504], [169.84163444520755, 123.3416986713996, 154.83107455194718, 167.98929163470268, 140.7932798872149, 101.68952014718067, 141.77615836031643, 146.55188089601023, 156.74047339913525, 163.36485909573406], [122.27088733454492, 109.20997405555539, 165.61688938660893, 170.33382062522801, 182.70092984366494, 107.97616157403853, 103.39739396512512, 145.35031470925776, 163.65926547880437, 160.94583046901406], [116.35505577055113, 114.1192854646577, 123.7609397041828, 160.69814808763311, 178.38382498160877, 68.98150340340261, 133.86332008334244, 146.19438482366462, 176.35573400668068, 183.52554229325003], [115.76525255456991, 91.80230503030586, 149.46566000403075, 164.23826817920266, 199.34751449005594, 96.97113934572377, 125.65836770040076, 139.29213316594414, 166.70626408889285, 158.4806267178086], [125.87152444376852, 112.25174296193403, 125.12493463520956, 161.91360363983492, 176.1976926865663, 95.84808145186982, 126.06153925617552, 148.35668741757596, 177.2675266637352, 178.77495846403392], [123.72400459693046, 101.31380805074481, 135.26798136474852, 145.08457880992663, 200.86161538572605, 89.75116450662642, 120.30558500298024, 158.45816233102877, 174.8894098741557, 177.71466936907032], [149.27816962680123, 108.37247732346466, 138.71329142679446, 152.99701822494, 183.85670983256415, 98.26543736382182, 127.5550170615973, 153.75067512774277, 157.57839871208935, 183.54169965397787], [124.60931392388997, 99.55757900064643, 161.99929959628253, 150.1285082839572, 186.11983693459018, 86.00430019489998, 119.13204577034072, 155.41436252761594, 169.16448238826908, 170.3493231523084], [163.82826724191202, 123.63300303116105, 162.8980670120787, 166.58612468713937, 158.67319842829247, 101.19007738890186, 123.85647903797361, 141.86796497619403, 159.9811243798996, 158.63953984939445], [148.67533995564713, 108.42457729451831, 142.42838475310768, 157.76017755019018, 175.27052518344323, 98.69191696560306, 130.78580900589537, 150.57399766610484, 168.29287308414735, 176.59224756357847], [150.027945250437, 108.79702288668555, 146.15298522743862, 142.32196166402898, 181.20052992519373, 98.66945040809613, 133.44593232016487, 150.76253296723166, 155.14298179124637, 188.26268790756117], [148.67533995564713, 108.42457729451831, 142.42838475310768, 157.76017755019018, 175.27052518344323, 98.69191696560306, 130.78580900589537, 150.57399766610484, 168.29287308414735, 176.59224756357847], [117.75853219996374, 104.55487481547416, 145.71552532921476, 171.12163119570744, 154.03785309717847, 96.62628959763566, 143.01389905230988, 148.6565437698375, 165.84899302629753, 163.7556890865001], [168.85386525471753, 123.60444750594341, 137.40385276973333, 157.67445281251932, 156.92671983700316, 102.20671718726648, 137.71856360164185, 148.732299411782, 164.68903502507757, 166.26001663639278], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [124.60931392388997, 99.55757900064643, 161.99929959628253, 150.1285082839572, 186.11983693459018, 86.00430019489998, 119.13204577034072, 155.41436252761594, 169.16448238826908, 170.3493231523084], [149.27816962680123, 108.37247732346466, 138.71329142679446, 152.99701822494, 183.85670983256415, 98.26543736382182, 127.5550170615973, 153.75067512774277, 157.57839871208935, 183.54169965397787], [148.65858587031735, 117.5537430787448, 152.7370674658746, 155.0185002942349, 147.46163154928857, 129.97949714189932, 132.1733655775968, 150.43382549066143, 156.29210499732608, 168.29369368023086], [169.11123835390373, 122.6553643831684, 144.88497598512376, 148.40715049726467, 162.9523172779664, 100.41858968258288, 133.79930341502003, 156.57000045809946, 154.37301314092394, 169.3832824070351], [122.27088733454492, 109.20997405555539, 165.61688938660893, 170.33382062522801, 182.70092984366494, 107.97616157403853, 103.39739396512512, 145.35031470925776, 163.65926547880437, 160.94583046901406], [173.98158099973762, 121.41401484854968, 155.2467272053208, 161.62490708015008, 139.23687798531955, 102.66460567234407, 139.44735831850167, 133.4012159187808, 173.97371251361338, 159.06106997603828], [119.41894344108162, 89.6361386782091, 144.86306350872732, 165.1607863571104, 211.6367393571435, 67.17495721088726, 127.51666835624646, 156.22666357481478, 168.0842230731582, 174.34523059533836], [109.83184940273217, 87.55118225280502, 173.27558964741314, 192.32819319963127, 202.6566054027225, 77.7955783209043, 110.7984266262011, 134.5099881875796, 171.96448643992636, 167.44659580947058], [155.63356434101732, 121.7037973314125, 141.61047245367973, 128.56412415865336, 136.09008626574686, 141.05775541519452, 134.93095555474864, 125.91983083232476, 131.26261056343623, 182.36619594400247], [146.18299237104432, 117.20105605174287, 126.9403685025021, 145.15044742546544, 168.3740185570338, 124.3244416636751, 128.32106677125984, 154.36131283034118, 170.5636407527166, 167.50903583812456], [181.393153961203, 136.65303694070522, 125.90506986307487, 151.23293415828567, 167.04522306488312, 103.96871006288565, 114.83430969632307, 159.04491127509579, 144.68189566301348, 131.87396315470303], [148.95420164834556, 102.41615587257776, 146.08091617104404, 143.6583501834782, 166.8856957427277, 104.25030634694905, 152.5036957947207, 149.91289442177094, 156.3036270071304, 191.01691397117983], [154.2340739641886, 120.83138478017217, 163.1793401868486, 160.31358068613486, 148.47839537340548, 117.1670246238789, 123.45996093277371, 154.16491696465175, 160.79963802966617, 156.97009997029812], [119.62309438448534, 90.435441749757, 143.33997457038888, 154.93751677485346, 225.34053642990904, 62.19288437268095, 128.31268015184958, 149.14552095531636, 162.8014528319032, 191.71203313048701], [148.48479676441337, 126.21029578037393, 159.62527053798442, 150.8061319125178, 153.23293437543683, 119.63764321443003, 128.4032854786844, 149.37101807759663, 152.58048638924546, 152.88482163934412], [148.67533995564713, 108.42457729451831, 142.42838475310768, 157.76017755019018, 175.27052518344323, 98.69191696560306, 130.78580900589537, 150.57399766610484, 168.29287308414735, 176.59224756357847], [149.06216452946686, 106.48162668769525, 151.4162018926752, 152.32082662555626, 143.9027578301337, 123.58902848907663, 145.9721620405975, 153.7559937174116, 162.32183464471146, 171.55119884108467], [138.20605623854652, 107.42348781850717, 129.21584774205314, 142.2134787300486, 192.8664244086329, 96.20732846975696, 131.92385143024265, 156.3132038929684, 172.34092474542578, 184.7627903630174], [154.25124766900188, 130.41874324998875, 125.82420113609076, 156.97943007117505, 157.16274510072986, 126.51035377237639, 131.08744654012494, 159.55495885505314, 143.6280207101792, 136.0236397347833], [175.45044868765953, 144.85557203619277, 97.35970782420642, 106.74860946813055, 116.99829105868903, 160.64925151872026, 161.94778876014928, 124.45884579721412, 120.36277491513589, 142.92708291981302], [142.63449826400614, 114.52912115848768, 162.5282288217732, 167.05112517426085, 186.8054381475563, 112.08697513982749, 104.78359141299305, 138.77711060508665, 161.08181121155621, 158.31794156050165], [122.74663386081352, 113.06323050057419, 146.57267726757388, 155.52207840429836, 190.72256075569607, 95.40417878586082, 127.13102346655903, 158.5148747504064, 157.40832002453945, 172.84554845016225], [181.393153961203, 136.65303694070522, 125.90506986307487, 151.23293415828567, 167.04522306488312, 103.96871006288565, 114.83430969632307, 159.04491127509579, 144.68189566301348, 131.87396315470303], [143.1069800873692, 100.82678189091465, 142.35190213646217, 156.72338410669272, 158.77990634245046, 104.02056322095221, 157.49620323294977, 149.72164263554606, 163.27352337203493, 188.63766492430616]]</t>
+          <t>[[143.9546414337465, 155.93661418823527, 156.02234767665738, 142.66876356279752, 145.84331399209412, 164.05292664928808, 155.05755548208455, 130.70002753637866, 138.07012673016678, 150.99195039312343], [168.93446178995708, 158.4459142284612, 139.58926818381008, 148.3953667606743, 164.45058717098613, 158.41641790210502, 156.86385093970057, 103.87830709669417, 152.84680937926137, 135.09349003435796], [157.82082867220757, 150.4994605626885, 147.69647029651756, 142.7958839373283, 139.4222617476472, 165.49719038635675, 141.31700237821124, 83.63997747362413, 188.77444200553944, 167.62875580255627], [139.64815413535186, 160.8459823325636, 153.9747611658381, 130.65715433812585, 155.84633625723637, 168.0598688232182, 178.55976522931985, 116.35827870255036, 142.82856643718986, 142.44339414986533], [169.1398940618324, 173.11916992147655, 107.54813382340834, 158.7073476797804, 149.19551634928246, 105.75811077754882, 138.37968359712116, 132.23524128046336, 162.53326205074183, 118.62599702016226]]</t>
         </is>
       </c>
     </row>
@@ -2675,7 +2675,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>142.71992395410652</t>
+          <t>144.46974555301207</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2702,12 +2702,12 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 12.0, 13.0, 16.0, 10.0, 14.0, 18.0, 20.0, 17.0], [10.0, 10.0, 17.0, 20.0, 18.0, 10.0, 10.0, 15.0, 14.0, 16.0], [12.0, 13.0, 17.0, 17.0, 17.0, 10.0, 10.0, 16.0, 18.0, 10.0], [10.0, 10.0, 12.0, 17.0, 17.0, 10.0, 13.0, 14.0, 20.0, 17.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0]]</t>
+          <t>[[14.0, 12.0, 15.0, 15.0, 15.0, 16.0, 14.0, 15.0, 12.0, 12.0], [16.0, 13.0, 15.0, 16.0, 13.0, 16.0, 13.0, 15.0, 10.0, 13.0], [10.0, 10.0, 21.0, 10.0, 20.0, 14.0, 14.0, 21.0, 10.0, 10.0], [13.0, 15.0, 17.0, 17.0, 10.0, 15.0, 17.0, 10.0, 10.0, 16.0], [10.0, 16.0, 10.0, 15.0, 13.0, 16.0, 16.0, 15.0, 16.0, 13.0]]</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>[[168.83996165156807, 123.59076141530063, 137.52389975446076, 156.56076627616952, 157.23945358979813, 102.19535536546157, 136.98234977747674, 148.11202772414816, 165.3966175086767, 168.1411905638944], [173.3778938221764, 121.08756093748445, 146.5913688266546, 154.40230569219315, 145.4947212627093, 103.72104361789681, 126.71084559796743, 151.73007906050145, 164.13194560985627, 156.0200638011278], [139.41539070961545, 114.54827561189082, 135.73475306205628, 140.81809021175053, 171.33152756667542, 119.20010596527693, 120.11723300749895, 148.21433184965375, 153.20138570473802, 156.95290611408822], [115.40154207344386, 89.81592503925985, 143.9484318186306, 167.27555292493275, 196.97953938222508, 68.16486543675677, 145.65137357476524, 149.6912349542489, 165.83173605452785, 185.4050771544179], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406]]</t>
+          <t>[[141.20123013658682, 127.22420910741194, 158.40996751036207, 139.29926279902793, 158.0029737625936, 163.29648752832074, 160.77686495954663, 128.49117422174027, 151.05113564614544, 158.71206748640083], [180.2174894768824, 134.7023277247296, 153.29419913157705, 178.11567394608116, 131.05687642371845, 160.2751775624008, 133.30799398874365, 156.9348759061682, 61.80588147458026, 163.9680774383658], [196.5429161620716, 118.20879323216276, 119.34273268874061, 131.52915034832716, 108.17245385819201, 146.39815980569793, 132.0525252620337, 154.6097077892856, 166.73461488818106, 125.80349266766493], [125.4511124759926, 178.91312086813988, 168.0124123592186, 159.63039637319574, 89.47917822015773, 183.84164431734894, 167.26652272339487, 117.21362094273546, 105.90444342946138, 151.08636760137773], [138.2763702451395, 165.72848049347246, 86.07488053789837, 133.2473294275904, 120.71849024901935, 132.7454376045337, 182.81070813522575, 157.6605484664594, 159.60469027051215, 160.28302997599008]]</t>
         </is>
       </c>
     </row>
@@ -2728,7 +2728,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>143.5218148073643</t>
+          <t>147.51689521748094</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2755,12 +2755,12 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 12.0, 13.0, 16.0, 10.0, 14.0, 18.0, 20.0, 17.0], [10.0, 10.0, 17.0, 20.0, 18.0, 10.0, 10.0, 15.0, 14.0, 16.0], [12.0, 13.0, 17.0, 17.0, 17.0, 10.0, 10.0, 16.0, 18.0, 10.0], [10.0, 10.0, 12.0, 17.0, 17.0, 10.0, 13.0, 14.0, 20.0, 17.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [10.0, 10.0, 20.0, 15.0, 14.0, 10.0, 12.0, 13.0, 17.0, 19.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 16.0, 13.0, 18.0, 10.0, 10.0, 18.0, 18.0, 14.0], [10.0, 10.0, 17.0, 16.0, 15.0, 10.0, 10.0, 16.0, 19.0, 17.0], [10.0, 10.0, 14.0, 19.0, 17.0, 10.0, 13.0, 13.0, 17.0, 17.0]]</t>
+          <t>[[16.0, 14.0, 14.0, 15.0, 13.0, 14.0, 15.0, 13.0, 14.0, 12.0], [17.0, 13.0, 14.0, 15.0, 14.0, 13.0, 14.0, 15.0, 13.0, 12.0], [15.0, 14.0, 14.0, 16.0, 12.0, 15.0, 14.0, 12.0, 15.0, 13.0], [14.0, 12.0, 12.0, 13.0, 13.0, 15.0, 15.0, 14.0, 19.0, 13.0], [16.0, 13.0, 10.0, 14.0, 16.0, 13.0, 16.0, 17.0, 10.0, 15.0]]</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>[[168.83996165156807, 123.59076141530063, 137.52389975446076, 156.56076627616952, 157.23945358979813, 102.19535536546157, 136.98234977747674, 148.11202772414816, 165.3966175086767, 168.1411905638944], [173.3778938221764, 121.08756093748445, 146.5913688266546, 154.40230569219315, 145.4947212627093, 103.72104361789681, 126.71084559796743, 151.73007906050145, 164.13194560985627, 156.0200638011278], [139.41539070961545, 114.54827561189082, 135.73475306205628, 140.81809021175053, 171.33152756667542, 119.20010596527693, 120.11723300749895, 148.21433184965375, 153.20138570473802, 156.95290611408822], [115.40154207344386, 89.81592503925985, 143.9484318186306, 167.27555292493275, 196.97953938222508, 68.16486543675677, 145.65137357476524, 149.6912349542489, 165.83173605452785, 185.4050771544179], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [155.30851665022445, 101.46766654749268, 157.67005968649443, 161.16074259334366, 147.0807205204198, 100.28855251190436, 152.95338094679695, 128.82601005018742, 171.6689462970614, 186.20394180285038], [151.49494337387458, 117.63970585649903, 163.36518294294515, 162.4387606206083, 155.6800257924122, 113.25638832677038, 117.6841561482807, 160.83878709456383, 159.34809118225894, 161.23989139159553], [155.31460127025164, 124.00260960556245, 148.60376550908018, 164.7376404534931, 161.71931721747035, 112.3850680839479, 114.1079803199717, 149.60165093783095, 157.59666266767624, 140.65031941257772], [116.75519767144029, 88.99311376250257, 147.25424111377666, 170.08749434033558, 210.62762868750434, 61.67641125468947, 143.08011862115282, 152.54965543170462, 163.87724299261785, 179.7845752589638], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705]]</t>
+          <t>[[160.82339156684048, 149.5985301891891, 159.72981834914225, 157.45251194028907, 157.44362326676634, 160.73272615210323, 177.69317795654624, 107.5732287002973, 135.14615937198818, 125.31700198676435], [131.9063534922431, 140.2029669861725, 155.9520446366828, 146.88842823519232, 154.09350117915173, 150.74762780168749, 149.7856648605115, 159.24468707826628, 148.31815237086576, 150.67263814891786], [155.4053984016226, 140.3690930249018, 161.61620080432874, 145.10325057591362, 134.36736594208364, 162.0699179734604, 162.02255332621226, 104.69801278048706, 153.19433600559702, 166.95647656014245], [133.28503119290986, 149.71323757852574, 130.57150548763033, 144.2766014805823, 131.61586104555596, 174.70996997603262, 174.79597787216443, 144.02018954174693, 154.64819889158906, 146.63331241847524], [163.43661653185353, 129.80257041273305, 103.01479418263983, 153.96294801551304, 162.1854262889534, 123.68940350458735, 162.26519920331216, 182.3635768591623, 84.47707502086726, 161.2524257048467]]</t>
         </is>
       </c>
     </row>
@@ -2781,14 +2781,14 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>13.973333333333333</t>
+          <t>14.0</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2798,7 +2798,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>143.74748647819948</t>
+          <t>149.26066201587366</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2808,12 +2808,12 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 12.0, 13.0, 16.0, 10.0, 14.0, 18.0, 20.0, 17.0], [10.0, 10.0, 17.0, 20.0, 18.0, 10.0, 10.0, 15.0, 14.0, 16.0], [12.0, 13.0, 17.0, 17.0, 17.0, 10.0, 10.0, 16.0, 18.0, 10.0], [10.0, 10.0, 12.0, 17.0, 17.0, 10.0, 13.0, 14.0, 20.0, 17.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [10.0, 10.0, 20.0, 15.0, 14.0, 10.0, 12.0, 13.0, 17.0, 19.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 16.0, 13.0, 18.0, 10.0, 10.0, 18.0, 18.0, 14.0], [10.0, 10.0, 17.0, 16.0, 15.0, 10.0, 10.0, 16.0, 19.0, 17.0], [10.0, 10.0, 14.0, 19.0, 17.0, 10.0, 13.0, 13.0, 17.0, 17.0], [10.0, 10.0, 17.0, 17.0, 13.0, 10.0, 13.0, 16.0, 16.0, 18.0], [13.0, 13.0, 10.0, 13.0, 13.0, 20.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 14.0, 18.0, 20.0, 10.0, 10.0, 20.0, 15.0, 13.0], [10.0, 10.0, 17.0, 14.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [10.0, 10.0, 18.0, 19.0, 15.0, 10.0, 13.0, 14.0, 18.0, 13.0]]</t>
+          <t>[[14.0, 12.0, 15.0, 14.0, 12.0, 16.0, 15.0, 15.0, 14.0, 13.0], [14.0, 14.0, 15.0, 12.0, 14.0, 16.0, 14.0, 15.0, 14.0, 12.0], [16.0, 15.0, 15.0, 15.0, 12.0, 14.0, 14.0, 12.0, 12.0, 15.0], [14.0, 15.0, 12.0, 16.0, 12.0, 14.0, 15.0, 14.0, 14.0, 14.0], [14.0, 15.0, 14.0, 14.0, 12.0, 15.0, 12.0, 16.0, 14.0, 14.0]]</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>[[168.83996165156807, 123.59076141530063, 137.52389975446076, 156.56076627616952, 157.23945358979813, 102.19535536546157, 136.98234977747674, 148.11202772414816, 165.3966175086767, 168.1411905638944], [173.3778938221764, 121.08756093748445, 146.5913688266546, 154.40230569219315, 145.4947212627093, 103.72104361789681, 126.71084559796743, 151.73007906050145, 164.13194560985627, 156.0200638011278], [139.41539070961545, 114.54827561189082, 135.73475306205628, 140.81809021175053, 171.33152756667542, 119.20010596527693, 120.11723300749895, 148.21433184965375, 153.20138570473802, 156.95290611408822], [115.40154207344386, 89.81592503925985, 143.9484318186306, 167.27555292493275, 196.97953938222508, 68.16486543675677, 145.65137357476524, 149.6912349542489, 165.83173605452785, 185.4050771544179], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [155.30851665022445, 101.46766654749268, 157.67005968649443, 161.16074259334366, 147.0807205204198, 100.28855251190436, 152.95338094679695, 128.82601005018742, 171.6689462970614, 186.20394180285038], [151.49494337387458, 117.63970585649903, 163.36518294294515, 162.4387606206083, 155.6800257924122, 113.25638832677038, 117.6841561482807, 160.83878709456383, 159.34809118225894, 161.23989139159553], [155.31460127025164, 124.00260960556245, 148.60376550908018, 164.7376404534931, 161.71931721747035, 112.3850680839479, 114.1079803199717, 149.60165093783095, 157.59666266767624, 140.65031941257772], [116.75519767144029, 88.99311376250257, 147.25424111377666, 170.08749434033558, 210.62762868750434, 61.67641125468947, 143.08011862115282, 152.54965543170462, 163.87724299261785, 179.7845752589638], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [122.54784555544693, 105.96315511038627, 157.97711386986117, 155.2254321890902, 174.64839198201918, 107.4048115793619, 131.48313009343553, 148.92290625266523, 157.07933065148725, 176.82477881731256], [146.20595012109717, 107.72606078634776, 127.61892564766411, 149.657659086279, 157.6312372947903, 117.64141321293776, 148.9797225611856, 157.30202446272347, 170.27970250153555, 171.94398144716365], [150.1993569665729, 131.99208731713904, 128.39741381245582, 160.87672932697532, 168.04061575136942, 132.62874187680404, 115.66162008336777, 159.92133798709102, 143.37137005344712, 128.6220526614146], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096]]</t>
+          <t>[[134.92146654623915, 140.6734557563938, 151.9567572410975, 122.95193146807895, 160.39513362670152, 176.04226690834867, 174.2567689266835, 142.54641897656003, 141.3694220760072, 147.33291254916895], [139.9350368193008, 146.20373151261512, 168.51487558091986, 157.78105041551433, 143.97059215753495, 147.95553086495474, 149.83626984829172, 152.85986374195537, 156.07588074797306, 130.91130248065699], [150.34124450271247, 145.93718907575712, 168.04991808244574, 148.69436586049673, 138.28212740018162, 161.7838730989635, 157.84904585110962, 126.82493779175657, 146.15068814257796, 150.4413113286041], [145.64589776237818, 157.76059899604206, 133.44443574732975, 151.42319832885357, 152.9389115075999, 162.74848386084807, 146.5382306638904, 143.2402765834958, 153.77470180116978, 147.06725947313998], [151.40333709740764, 151.90499744533895, 149.28210093785296, 168.6356054536115, 135.38873052243179, 159.88940166363778, 160.014126705302, 127.82130364454075, 136.26358035202742, 147.0025528671843]]</t>
         </is>
       </c>
     </row>
@@ -2834,14 +2834,14 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>13.979999999999999</t>
+          <t>14.0</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>143.26323327446192</t>
+          <t>148.83695539637603</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2861,12 +2861,12 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 12.0, 13.0, 16.0, 10.0, 14.0, 18.0, 20.0, 17.0], [10.0, 10.0, 17.0, 20.0, 18.0, 10.0, 10.0, 15.0, 14.0, 16.0], [12.0, 13.0, 17.0, 17.0, 17.0, 10.0, 10.0, 16.0, 18.0, 10.0], [10.0, 10.0, 12.0, 17.0, 17.0, 10.0, 13.0, 14.0, 20.0, 17.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [10.0, 10.0, 20.0, 15.0, 14.0, 10.0, 12.0, 13.0, 17.0, 19.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 16.0, 13.0, 18.0, 10.0, 10.0, 18.0, 18.0, 14.0], [10.0, 10.0, 17.0, 16.0, 15.0, 10.0, 10.0, 16.0, 19.0, 17.0], [10.0, 10.0, 14.0, 19.0, 17.0, 10.0, 13.0, 13.0, 17.0, 17.0], [10.0, 10.0, 17.0, 17.0, 13.0, 10.0, 13.0, 16.0, 16.0, 18.0], [13.0, 13.0, 10.0, 13.0, 13.0, 20.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 14.0, 18.0, 20.0, 10.0, 10.0, 20.0, 15.0, 13.0], [10.0, 10.0, 17.0, 14.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [10.0, 10.0, 18.0, 19.0, 15.0, 10.0, 13.0, 14.0, 18.0, 13.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 18.0, 16.0, 18.0, 13.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [13.0, 13.0, 16.0, 16.0, 14.0, 10.0, 10.0, 17.0, 18.0, 13.0], [18.0, 20.0, 10.0, 10.0, 15.0, 21.0, 16.0, 10.0, 10.0, 10.0], [20.0, 20.0, 13.0, 13.0, 14.0, 13.0, 10.0, 13.0, 14.0, 10.0]]</t>
+          <t>[[14.0, 14.0, 12.0, 14.0, 12.0, 15.0, 15.0, 15.0, 14.0, 15.0], [16.0, 12.0, 12.0, 15.0, 15.0, 14.0, 16.0, 12.0, 14.0, 14.0], [12.0, 14.0, 12.0, 16.0, 15.0, 14.0, 15.0, 12.0, 14.0, 16.0], [14.0, 16.0, 14.0, 15.0, 12.0, 13.0, 14.0, 15.0, 12.0, 15.0], [15.0, 12.0, 13.0, 12.0, 15.0, 15.0, 15.0, 19.0, 12.0, 12.0]]</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>[[168.83996165156807, 123.59076141530063, 137.52389975446076, 156.56076627616952, 157.23945358979813, 102.19535536546157, 136.98234977747674, 148.11202772414816, 165.3966175086767, 168.1411905638944], [173.3778938221764, 121.08756093748445, 146.5913688266546, 154.40230569219315, 145.4947212627093, 103.72104361789681, 126.71084559796743, 151.73007906050145, 164.13194560985627, 156.0200638011278], [139.41539070961545, 114.54827561189082, 135.73475306205628, 140.81809021175053, 171.33152756667542, 119.20010596527693, 120.11723300749895, 148.21433184965375, 153.20138570473802, 156.95290611408822], [115.40154207344386, 89.81592503925985, 143.9484318186306, 167.27555292493275, 196.97953938222508, 68.16486543675677, 145.65137357476524, 149.6912349542489, 165.83173605452785, 185.4050771544179], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [155.30851665022445, 101.46766654749268, 157.67005968649443, 161.16074259334366, 147.0807205204198, 100.28855251190436, 152.95338094679695, 128.82601005018742, 171.6689462970614, 186.20394180285038], [151.49494337387458, 117.63970585649903, 163.36518294294515, 162.4387606206083, 155.6800257924122, 113.25638832677038, 117.6841561482807, 160.83878709456383, 159.34809118225894, 161.23989139159553], [155.31460127025164, 124.00260960556245, 148.60376550908018, 164.7376404534931, 161.71931721747035, 112.3850680839479, 114.1079803199717, 149.60165093783095, 157.59666266767624, 140.65031941257772], [116.75519767144029, 88.99311376250257, 147.25424111377666, 170.08749434033558, 210.62762868750434, 61.67641125468947, 143.08011862115282, 152.54965543170462, 163.87724299261785, 179.7845752589638], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [122.54784555544693, 105.96315511038627, 157.97711386986117, 155.2254321890902, 174.64839198201918, 107.4048115793619, 131.48313009343553, 148.92290625266523, 157.07933065148725, 176.82477881731256], [146.20595012109717, 107.72606078634776, 127.61892564766411, 149.657659086279, 157.6312372947903, 117.64141321293776, 148.9797225611856, 157.30202446272347, 170.27970250153555, 171.94398144716365], [150.1993569665729, 131.99208731713904, 128.39741381245582, 160.87672932697532, 168.04061575136942, 132.62874187680404, 115.66162008336777, 159.92133798709102, 143.37137005344712, 128.6220526614146], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [171.25214622653692, 122.04092166869397, 163.28536700743373, 146.08131701827855, 166.3694233187611, 102.3003445816535, 113.49515031953875, 154.10183902835064, 153.28354180543303, 143.2839025143099], [183.9641110300671, 146.9571103426829, 82.42156374434263, 110.54738368811277, 161.45011086895678, 163.2299709311923, 110.01291484769432, 125.46488882332544, 121.24645626255418, 135.87043875544455], [154.87670501106774, 124.45712875915734, 157.33520915081402, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 150.72696126211756, 153.1866101146596, 155.4404734500336]]</t>
+          <t>[[156.35057508298263, 148.26591178045294, 151.53994971788958, 139.60814153797014, 129.907161542221, 164.71051978845952, 151.68164030511724, 151.19764183524273, 134.76605637155114, 164.47109152623258], [159.99421645243754, 123.96931596442384, 159.32021052212087, 170.96769422909023, 158.10626439867877, 146.36905987092092, 179.49884208230367, 97.62940177349658, 135.33666481567076, 158.49622709338192], [146.6419874077992, 153.15473636822102, 137.228150840678, 168.4224618051917, 154.5817588800562, 130.7874315641405, 137.6860615653221, 146.96207107010582, 148.57821554072515, 169.58311715352966], [147.55899043560535, 163.88878252843296, 158.51593608065443, 155.13611581197688, 146.33057292215176, 163.25197941721947, 144.46532674730153, 111.00667300055109, 130.78359802951263, 159.35771072806705], [149.18171329568042, 105.54147385385065, 182.22261633601704, 111.09585500241559, 166.32784418311687, 168.05802988164237, 178.19102724202122, 124.43821051864818, 149.97023288463265, 150.71250203289077]]</t>
         </is>
       </c>
     </row>
@@ -2887,14 +2887,14 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>13.984</t>
+          <t>14.0</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>143.0411847288978</t>
+          <t>148.8387886476361</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2914,12 +2914,12 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 12.0, 13.0, 16.0, 10.0, 14.0, 18.0, 20.0, 17.0], [10.0, 10.0, 17.0, 20.0, 18.0, 10.0, 10.0, 15.0, 14.0, 16.0], [12.0, 13.0, 17.0, 17.0, 17.0, 10.0, 10.0, 16.0, 18.0, 10.0], [10.0, 10.0, 12.0, 17.0, 17.0, 10.0, 13.0, 14.0, 20.0, 17.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [10.0, 10.0, 20.0, 15.0, 14.0, 10.0, 12.0, 13.0, 17.0, 19.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 16.0, 13.0, 18.0, 10.0, 10.0, 18.0, 18.0, 14.0], [10.0, 10.0, 17.0, 16.0, 15.0, 10.0, 10.0, 16.0, 19.0, 17.0], [10.0, 10.0, 14.0, 19.0, 17.0, 10.0, 13.0, 13.0, 17.0, 17.0], [10.0, 10.0, 17.0, 17.0, 13.0, 10.0, 13.0, 16.0, 16.0, 18.0], [13.0, 13.0, 10.0, 13.0, 13.0, 20.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 14.0, 18.0, 20.0, 10.0, 10.0, 20.0, 15.0, 13.0], [10.0, 10.0, 17.0, 14.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [10.0, 10.0, 18.0, 19.0, 15.0, 10.0, 13.0, 14.0, 18.0, 13.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 18.0, 16.0, 18.0, 13.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [13.0, 13.0, 16.0, 16.0, 14.0, 10.0, 10.0, 17.0, 18.0, 13.0], [18.0, 20.0, 10.0, 10.0, 15.0, 21.0, 16.0, 10.0, 10.0, 10.0], [20.0, 20.0, 13.0, 13.0, 14.0, 13.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 14.0, 19.0, 15.0, 10.0, 14.0, 14.0, 17.0, 17.0], [10.0, 10.0, 13.0, 18.0, 13.0, 10.0, 17.0, 17.0, 18.0, 14.0], [10.0, 15.0, 13.0, 16.0, 13.0, 10.0, 13.0, 16.0, 18.0, 16.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [20.0, 10.0, 16.0, 14.0, 13.0, 13.0, 12.0, 10.0, 17.0, 15.0]]</t>
+          <t>[[15.0, 14.0, 14.0, 14.0, 14.0, 14.0, 16.0, 14.0, 15.0, 10.0], [14.0, 15.0, 12.0, 15.0, 14.0, 15.0, 14.0, 13.0, 12.0, 16.0], [14.0, 14.0, 14.0, 16.0, 12.0, 14.0, 14.0, 13.0, 15.0, 14.0], [16.0, 15.0, 14.0, 16.0, 12.0, 14.0, 12.0, 14.0, 13.0, 14.0], [16.0, 17.0, 14.0, 14.0, 14.0, 12.0, 15.0, 11.0, 15.0, 12.0]]</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>[[168.83996165156807, 123.59076141530063, 137.52389975446076, 156.56076627616952, 157.23945358979813, 102.19535536546157, 136.98234977747674, 148.11202772414816, 165.3966175086767, 168.1411905638944], [173.3778938221764, 121.08756093748445, 146.5913688266546, 154.40230569219315, 145.4947212627093, 103.72104361789681, 126.71084559796743, 151.73007906050145, 164.13194560985627, 156.0200638011278], [139.41539070961545, 114.54827561189082, 135.73475306205628, 140.81809021175053, 171.33152756667542, 119.20010596527693, 120.11723300749895, 148.21433184965375, 153.20138570473802, 156.95290611408822], [115.40154207344386, 89.81592503925985, 143.9484318186306, 167.27555292493275, 196.97953938222508, 68.16486543675677, 145.65137357476524, 149.6912349542489, 165.83173605452785, 185.4050771544179], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [155.30851665022445, 101.46766654749268, 157.67005968649443, 161.16074259334366, 147.0807205204198, 100.28855251190436, 152.95338094679695, 128.82601005018742, 171.6689462970614, 186.20394180285038], [151.49494337387458, 117.63970585649903, 163.36518294294515, 162.4387606206083, 155.6800257924122, 113.25638832677038, 117.6841561482807, 160.83878709456383, 159.34809118225894, 161.23989139159553], [155.31460127025164, 124.00260960556245, 148.60376550908018, 164.7376404534931, 161.71931721747035, 112.3850680839479, 114.1079803199717, 149.60165093783095, 157.59666266767624, 140.65031941257772], [116.75519767144029, 88.99311376250257, 147.25424111377666, 170.08749434033558, 210.62762868750434, 61.67641125468947, 143.08011862115282, 152.54965543170462, 163.87724299261785, 179.7845752589638], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [122.54784555544693, 105.96315511038627, 157.97711386986117, 155.2254321890902, 174.64839198201918, 107.4048115793619, 131.48313009343553, 148.92290625266523, 157.07933065148725, 176.82477881731256], [146.20595012109717, 107.72606078634776, 127.61892564766411, 149.657659086279, 157.6312372947903, 117.64141321293776, 148.9797225611856, 157.30202446272347, 170.27970250153555, 171.94398144716365], [150.1993569665729, 131.99208731713904, 128.39741381245582, 160.87672932697532, 168.04061575136942, 132.62874187680404, 115.66162008336777, 159.92133798709102, 143.37137005344712, 128.6220526614146], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [171.25214622653692, 122.04092166869397, 163.28536700743373, 146.08131701827855, 166.3694233187611, 102.3003445816535, 113.49515031953875, 154.10183902835064, 153.28354180543303, 143.2839025143099], [183.9641110300671, 146.9571103426829, 82.42156374434263, 110.54738368811277, 161.45011086895678, 163.2299709311923, 110.01291484769432, 125.46488882332544, 121.24645626255418, 135.87043875544455], [154.87670501106774, 124.45712875915734, 157.33520915081402, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 150.72696126211756, 153.1866101146596, 155.4404734500336], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096], [132.6393307913183, 109.30686173945848, 145.99049101750552, 152.59811248205753, 165.52450200376143, 117.34929630919373, 129.6409490643926, 152.35447181627313, 157.37714922337852, 161.60798730295116], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [165.24117105960053, 133.77087149912916, 129.9614208259944, 121.00987965148478, 124.0617095913029, 124.99420175139073, 145.07648926363632, 125.14749257346011, 133.51187048282097, 194.0374710761797]]</t>
+          <t>[[137.90551498166093, 148.15493229829252, 158.11590535861788, 147.75756756156204, 146.37401634282762, 152.1741615429561, 159.9398196300095, 141.89753227369675, 163.67226322923085, 136.512716509715], [152.44003893105034, 158.6762766410598, 142.22472168602644, 144.36077851931967, 143.82685730984727, 162.95417409416024, 158.1389055776326, 113.43163108997784, 143.51559316319748, 174.11439856035108], [152.873869071206, 146.85592336551053, 153.2363276856136, 160.23956076557775, 154.16024241370744, 133.2940116641482, 155.857199307598, 136.88598022987316, 150.9676131358658, 150.40400927214048], [134.71819417977957, 156.4746932528745, 140.04651935023855, 185.73978056413927, 164.75730658005935, 159.5650090776096, 136.09437310572892, 131.41406993105247, 130.90863664854106, 155.0547377323752], [130.4811432992595, 144.14775173347772, 183.64932430997732, 125.95020652859137, 133.00368780522672, 162.74116867699883, 140.1184163420953, 165.94376489415382, 148.8085135100885, 131.35959264710425]]</t>
         </is>
       </c>
     </row>
@@ -2940,14 +2940,14 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>13.986666666666665</t>
+          <t>14.0</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>143.25368635785972</t>
+          <t>149.15979983572942</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2967,12 +2967,12 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 12.0, 13.0, 16.0, 10.0, 14.0, 18.0, 20.0, 17.0], [10.0, 10.0, 17.0, 20.0, 18.0, 10.0, 10.0, 15.0, 14.0, 16.0], [12.0, 13.0, 17.0, 17.0, 17.0, 10.0, 10.0, 16.0, 18.0, 10.0], [10.0, 10.0, 12.0, 17.0, 17.0, 10.0, 13.0, 14.0, 20.0, 17.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [10.0, 10.0, 20.0, 15.0, 14.0, 10.0, 12.0, 13.0, 17.0, 19.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 16.0, 13.0, 18.0, 10.0, 10.0, 18.0, 18.0, 14.0], [10.0, 10.0, 17.0, 16.0, 15.0, 10.0, 10.0, 16.0, 19.0, 17.0], [10.0, 10.0, 14.0, 19.0, 17.0, 10.0, 13.0, 13.0, 17.0, 17.0], [10.0, 10.0, 17.0, 17.0, 13.0, 10.0, 13.0, 16.0, 16.0, 18.0], [13.0, 13.0, 10.0, 13.0, 13.0, 20.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 14.0, 18.0, 20.0, 10.0, 10.0, 20.0, 15.0, 13.0], [10.0, 10.0, 17.0, 14.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [10.0, 10.0, 18.0, 19.0, 15.0, 10.0, 13.0, 14.0, 18.0, 13.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 18.0, 16.0, 18.0, 13.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [13.0, 13.0, 16.0, 16.0, 14.0, 10.0, 10.0, 17.0, 18.0, 13.0], [18.0, 20.0, 10.0, 10.0, 15.0, 21.0, 16.0, 10.0, 10.0, 10.0], [20.0, 20.0, 13.0, 13.0, 14.0, 13.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 14.0, 19.0, 15.0, 10.0, 14.0, 14.0, 17.0, 17.0], [10.0, 10.0, 13.0, 18.0, 13.0, 10.0, 17.0, 17.0, 18.0, 14.0], [10.0, 15.0, 13.0, 16.0, 13.0, 10.0, 13.0, 16.0, 18.0, 16.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [20.0, 10.0, 16.0, 14.0, 13.0, 13.0, 12.0, 10.0, 17.0, 15.0], [10.0, 10.0, 17.0, 14.0, 13.0, 10.0, 13.0, 18.0, 18.0, 17.0], [10.0, 13.0, 16.0, 19.0, 17.0, 10.0, 10.0, 13.0, 19.0, 13.0], [10.0, 13.0, 16.0, 19.0, 17.0, 10.0, 10.0, 13.0, 19.0, 13.0], [10.0, 15.0, 13.0, 16.0, 13.0, 10.0, 13.0, 16.0, 18.0, 16.0], [10.0, 10.0, 18.0, 22.0, 16.0, 10.0, 10.0, 11.0, 18.0, 15.0]]</t>
+          <t>[[14.0, 16.0, 14.0, 14.0, 12.0, 12.0, 14.0, 14.0, 16.0, 14.0], [14.0, 17.0, 12.0, 12.0, 14.0, 14.0, 15.0, 14.0, 14.0, 14.0], [14.0, 15.0, 12.0, 14.0, 12.0, 14.0, 15.0, 14.0, 14.0, 16.0], [15.0, 14.0, 12.0, 14.0, 14.0, 14.0, 15.0, 16.0, 14.0, 12.0], [15.0, 15.0, 15.0, 14.0, 12.0, 12.0, 14.0, 15.0, 14.0, 14.0]]</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>[[168.83996165156807, 123.59076141530063, 137.52389975446076, 156.56076627616952, 157.23945358979813, 102.19535536546157, 136.98234977747674, 148.11202772414816, 165.3966175086767, 168.1411905638944], [173.3778938221764, 121.08756093748445, 146.5913688266546, 154.40230569219315, 145.4947212627093, 103.72104361789681, 126.71084559796743, 151.73007906050145, 164.13194560985627, 156.0200638011278], [139.41539070961545, 114.54827561189082, 135.73475306205628, 140.81809021175053, 171.33152756667542, 119.20010596527693, 120.11723300749895, 148.21433184965375, 153.20138570473802, 156.95290611408822], [115.40154207344386, 89.81592503925985, 143.9484318186306, 167.27555292493275, 196.97953938222508, 68.16486543675677, 145.65137357476524, 149.6912349542489, 165.83173605452785, 185.4050771544179], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [155.30851665022445, 101.46766654749268, 157.67005968649443, 161.16074259334366, 147.0807205204198, 100.28855251190436, 152.95338094679695, 128.82601005018742, 171.6689462970614, 186.20394180285038], [151.49494337387458, 117.63970585649903, 163.36518294294515, 162.4387606206083, 155.6800257924122, 113.25638832677038, 117.6841561482807, 160.83878709456383, 159.34809118225894, 161.23989139159553], [155.31460127025164, 124.00260960556245, 148.60376550908018, 164.7376404534931, 161.71931721747035, 112.3850680839479, 114.1079803199717, 149.60165093783095, 157.59666266767624, 140.65031941257772], [116.75519767144029, 88.99311376250257, 147.25424111377666, 170.08749434033558, 210.62762868750434, 61.67641125468947, 143.08011862115282, 152.54965543170462, 163.87724299261785, 179.7845752589638], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [122.54784555544693, 105.96315511038627, 157.97711386986117, 155.2254321890902, 174.64839198201918, 107.4048115793619, 131.48313009343553, 148.92290625266523, 157.07933065148725, 176.82477881731256], [146.20595012109717, 107.72606078634776, 127.61892564766411, 149.657659086279, 157.6312372947903, 117.64141321293776, 148.9797225611856, 157.30202446272347, 170.27970250153555, 171.94398144716365], [150.1993569665729, 131.99208731713904, 128.39741381245582, 160.87672932697532, 168.04061575136942, 132.62874187680404, 115.66162008336777, 159.92133798709102, 143.37137005344712, 128.6220526614146], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [171.25214622653692, 122.04092166869397, 163.28536700743373, 146.08131701827855, 166.3694233187611, 102.3003445816535, 113.49515031953875, 154.10183902835064, 153.28354180543303, 143.2839025143099], [183.9641110300671, 146.9571103426829, 82.42156374434263, 110.54738368811277, 161.45011086895678, 163.2299709311923, 110.01291484769432, 125.46488882332544, 121.24645626255418, 135.87043875544455], [154.87670501106774, 124.45712875915734, 157.33520915081402, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 150.72696126211756, 153.1866101146596, 155.4404734500336], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096], [132.6393307913183, 109.30686173945848, 145.99049101750552, 152.59811248205753, 165.52450200376143, 117.34929630919373, 129.6409490643926, 152.35447181627313, 157.37714922337852, 161.60798730295116], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [165.24117105960053, 133.77087149912916, 129.9614208259944, 121.00987965148478, 124.0617095913029, 124.99420175139073, 145.07648926363632, 125.14749257346011, 133.51187048282097, 194.0374710761797], [148.65858587031735, 117.5537430787448, 152.7370674658746, 155.0185002942349, 147.46163154928857, 129.97949714189932, 132.1733655775968, 150.43382549066143, 156.29210499732608, 168.29369368023086], [154.87670501106774, 124.45712875915734, 157.33520915081402, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 150.72696126211756, 153.1866101146596, 155.4404734500336], [174.10245819655114, 127.80900078262174, 138.67139289299246, 148.41069607289663, 153.6350666551481, 103.46472832433717, 130.22281241842936, 147.4818180038071, 152.50682731933753, 157.6981277590819], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [163.82826724191202, 123.63300303116105, 162.8980670120787, 166.58612468713937, 158.67319842829247, 101.19007738890186, 123.85647903797361, 141.86796497619403, 159.9811243798996, 158.63953984939445]]</t>
+          <t>[[148.932802389076, 150.81260698370357, 150.982844922737, 145.90952901074, 140.24794182241484, 150.9250818153528, 158.5850450376021, 143.5297425383248, 157.6466338236241, 147.17725300747176], [139.39614513769592, 160.49961493364665, 141.93346615482503, 167.0802003478466, 156.77759237101816, 152.80563170479547, 145.7321715063759, 122.36744044245805, 141.6528870172137, 163.63897770607704], [138.2934282725598, 142.8115375212631, 151.47684242369832, 160.51738392545835, 143.438223032131, 150.2697548069707, 159.5949730190772, 143.595187395627, 153.9173819474224, 144.76431172566052], [151.84283284670394, 140.9735673902154, 161.04148344073496, 140.62871518512569, 154.09169330338975, 159.4933216829397, 158.80397815941018, 141.85666599542373, 147.30945119981342, 135.67697040893813], [132.799262203395, 167.70597618765058, 156.92141496910926, 141.8555632079008, 132.67515177739503, 171.33554258055545, 149.37210055425024, 131.46858483211582, 155.03814069541409, 151.78694242312207]]</t>
         </is>
       </c>
     </row>
@@ -2993,14 +2993,14 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>13.988571428571428</t>
+          <t>14.0</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>143.36864814470272</t>
+          <t>148.46679276173552</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3020,12 +3020,12 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 12.0, 13.0, 16.0, 10.0, 14.0, 18.0, 20.0, 17.0], [10.0, 10.0, 17.0, 20.0, 18.0, 10.0, 10.0, 15.0, 14.0, 16.0], [12.0, 13.0, 17.0, 17.0, 17.0, 10.0, 10.0, 16.0, 18.0, 10.0], [10.0, 10.0, 12.0, 17.0, 17.0, 10.0, 13.0, 14.0, 20.0, 17.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [10.0, 10.0, 20.0, 15.0, 14.0, 10.0, 12.0, 13.0, 17.0, 19.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 16.0, 13.0, 18.0, 10.0, 10.0, 18.0, 18.0, 14.0], [10.0, 10.0, 17.0, 16.0, 15.0, 10.0, 10.0, 16.0, 19.0, 17.0], [10.0, 10.0, 14.0, 19.0, 17.0, 10.0, 13.0, 13.0, 17.0, 17.0], [10.0, 10.0, 17.0, 17.0, 13.0, 10.0, 13.0, 16.0, 16.0, 18.0], [13.0, 13.0, 10.0, 13.0, 13.0, 20.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 14.0, 18.0, 20.0, 10.0, 10.0, 20.0, 15.0, 13.0], [10.0, 10.0, 17.0, 14.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [10.0, 10.0, 18.0, 19.0, 15.0, 10.0, 13.0, 14.0, 18.0, 13.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 18.0, 16.0, 18.0, 13.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [13.0, 13.0, 16.0, 16.0, 14.0, 10.0, 10.0, 17.0, 18.0, 13.0], [18.0, 20.0, 10.0, 10.0, 15.0, 21.0, 16.0, 10.0, 10.0, 10.0], [20.0, 20.0, 13.0, 13.0, 14.0, 13.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 14.0, 19.0, 15.0, 10.0, 14.0, 14.0, 17.0, 17.0], [10.0, 10.0, 13.0, 18.0, 13.0, 10.0, 17.0, 17.0, 18.0, 14.0], [10.0, 15.0, 13.0, 16.0, 13.0, 10.0, 13.0, 16.0, 18.0, 16.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [20.0, 10.0, 16.0, 14.0, 13.0, 13.0, 12.0, 10.0, 17.0, 15.0], [10.0, 10.0, 17.0, 14.0, 13.0, 10.0, 13.0, 18.0, 18.0, 17.0], [10.0, 13.0, 16.0, 19.0, 17.0, 10.0, 10.0, 13.0, 19.0, 13.0], [10.0, 13.0, 16.0, 19.0, 17.0, 10.0, 10.0, 13.0, 19.0, 13.0], [10.0, 15.0, 13.0, 16.0, 13.0, 10.0, 13.0, 16.0, 18.0, 16.0], [10.0, 10.0, 18.0, 22.0, 16.0, 10.0, 10.0, 11.0, 18.0, 15.0], [10.0, 13.0, 18.0, 16.0, 18.0, 10.0, 10.0, 17.0, 14.0, 14.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 17.0, 17.0, 18.0, 13.0], [10.0, 10.0, 18.0, 20.0, 16.0, 10.0, 10.0, 15.0, 14.0, 17.0], [10.0, 10.0, 16.0, 17.0, 13.0, 10.0, 13.0, 13.0, 20.0, 18.0], [14.0, 10.0, 13.0, 17.0, 13.0, 10.0, 13.0, 16.0, 16.0, 18.0]]</t>
+          <t>[[15.0, 14.0, 15.0, 15.0, 12.0, 15.0, 12.0, 14.0, 14.0, 14.0], [15.0, 14.0, 14.0, 14.0, 10.0, 14.0, 15.0, 14.0, 16.0, 14.0], [14.0, 15.0, 15.0, 13.0, 14.0, 13.0, 15.0, 14.0, 17.0, 10.0], [13.0, 14.0, 15.0, 10.0, 13.0, 19.0, 17.0, 13.0, 13.0, 13.0], [15.0, 15.0, 12.0, 14.0, 14.0, 14.0, 14.0, 15.0, 15.0, 12.0]]</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>[[168.83996165156807, 123.59076141530063, 137.52389975446076, 156.56076627616952, 157.23945358979813, 102.19535536546157, 136.98234977747674, 148.11202772414816, 165.3966175086767, 168.1411905638944], [173.3778938221764, 121.08756093748445, 146.5913688266546, 154.40230569219315, 145.4947212627093, 103.72104361789681, 126.71084559796743, 151.73007906050145, 164.13194560985627, 156.0200638011278], [139.41539070961545, 114.54827561189082, 135.73475306205628, 140.81809021175053, 171.33152756667542, 119.20010596527693, 120.11723300749895, 148.21433184965375, 153.20138570473802, 156.95290611408822], [115.40154207344386, 89.81592503925985, 143.9484318186306, 167.27555292493275, 196.97953938222508, 68.16486543675677, 145.65137357476524, 149.6912349542489, 165.83173605452785, 185.4050771544179], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [155.30851665022445, 101.46766654749268, 157.67005968649443, 161.16074259334366, 147.0807205204198, 100.28855251190436, 152.95338094679695, 128.82601005018742, 171.6689462970614, 186.20394180285038], [151.49494337387458, 117.63970585649903, 163.36518294294515, 162.4387606206083, 155.6800257924122, 113.25638832677038, 117.6841561482807, 160.83878709456383, 159.34809118225894, 161.23989139159553], [155.31460127025164, 124.00260960556245, 148.60376550908018, 164.7376404534931, 161.71931721747035, 112.3850680839479, 114.1079803199717, 149.60165093783095, 157.59666266767624, 140.65031941257772], [116.75519767144029, 88.99311376250257, 147.25424111377666, 170.08749434033558, 210.62762868750434, 61.67641125468947, 143.08011862115282, 152.54965543170462, 163.87724299261785, 179.7845752589638], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [122.54784555544693, 105.96315511038627, 157.97711386986117, 155.2254321890902, 174.64839198201918, 107.4048115793619, 131.48313009343553, 148.92290625266523, 157.07933065148725, 176.82477881731256], [146.20595012109717, 107.72606078634776, 127.61892564766411, 149.657659086279, 157.6312372947903, 117.64141321293776, 148.9797225611856, 157.30202446272347, 170.27970250153555, 171.94398144716365], [150.1993569665729, 131.99208731713904, 128.39741381245582, 160.87672932697532, 168.04061575136942, 132.62874187680404, 115.66162008336777, 159.92133798709102, 143.37137005344712, 128.6220526614146], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [171.25214622653692, 122.04092166869397, 163.28536700743373, 146.08131701827855, 166.3694233187611, 102.3003445816535, 113.49515031953875, 154.10183902835064, 153.28354180543303, 143.2839025143099], [183.9641110300671, 146.9571103426829, 82.42156374434263, 110.54738368811277, 161.45011086895678, 163.2299709311923, 110.01291484769432, 125.46488882332544, 121.24645626255418, 135.87043875544455], [154.87670501106774, 124.45712875915734, 157.33520915081402, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 150.72696126211756, 153.1866101146596, 155.4404734500336], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096], [132.6393307913183, 109.30686173945848, 145.99049101750552, 152.59811248205753, 165.52450200376143, 117.34929630919373, 129.6409490643926, 152.35447181627313, 157.37714922337852, 161.60798730295116], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [165.24117105960053, 133.77087149912916, 129.9614208259944, 121.00987965148478, 124.0617095913029, 124.99420175139073, 145.07648926363632, 125.14749257346011, 133.51187048282097, 194.0374710761797], [148.65858587031735, 117.5537430787448, 152.7370674658746, 155.0185002942349, 147.46163154928857, 129.97949714189932, 132.1733655775968, 150.43382549066143, 156.29210499732608, 168.29369368023086], [154.87670501106774, 124.45712875915734, 157.33520915081402, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 150.72696126211756, 153.1866101146596, 155.4404734500336], [174.10245819655114, 127.80900078262174, 138.67139289299246, 148.41069607289663, 153.6350666551481, 103.46472832433717, 130.22281241842936, 147.4818180038071, 152.50682731933753, 157.6981277590819], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [163.82826724191202, 123.63300303116105, 162.8980670120787, 166.58612468713937, 158.67319842829247, 101.19007738890186, 123.85647903797361, 141.86796497619403, 159.9811243798996, 158.63953984939445], [145.0072351499823, 115.99968345962576, 160.68230623339542, 152.3530590210606, 167.1076278296097, 131.08931955966278, 114.54546057653036, 150.04147491293364, 155.30290240960926, 140.86380002454607], [149.7529984808466, 108.80052007547977, 124.96810248186745, 146.0270227777066, 171.51514835196625, 98.79095122172545, 131.01688305315017, 147.11708785009412, 174.0852436128256, 192.9599715968946], [144.55856538564217, 117.02977381184573, 151.09093700806469, 170.31849702527362, 189.88602050509368, 111.78524265062529, 106.75016416033765, 149.20146450350555, 161.4668277430309, 146.78621271509914], [140.2268461963245, 116.71115157478997, 146.52034871887318, 146.389151580322, 152.9818486418794, 106.05265716177503, 131.3508218040346, 147.3827546710329, 173.23148359875637, 165.37466641996363], [154.2527428966532, 117.80024702535607, 164.2594332885985, 167.82531633195677, 150.90075080208038, 111.02924005724354, 99.95541985534355, 162.24143788372814, 165.1755696808328, 156.3585509104705]]</t>
+          <t>[[162.38121120862905, 142.26600362838582, 153.2111507276943, 155.1416496529073, 143.3733733413927, 139.1433116305153, 160.76613355835082, 125.60668781569949, 142.83119446522159, 157.66704765594173], [143.3419874086401, 143.51037687688626, 156.32354433434347, 152.22795193388666, 145.68972435514564, 152.7620752904703, 158.0624379932575, 138.15774317679578, 144.9154771756132, 159.14147336064698], [137.4493106473722, 155.1429912338824, 165.66615520996635, 159.24569684048487, 145.90657681009316, 152.5799550573537, 145.1540242335562, 136.82092105082813, 159.06901317516213, 136.2410572085491], [145.16772568175585, 145.4723639363083, 174.04880757047115, 146.95860756597492, 129.86227515669037, 159.90306097175483, 169.19715011785638, 123.73386596124466, 143.08476697751803, 136.04753911968885], [146.48074368604458, 146.89942129881987, 151.74236160594424, 150.2815467033126, 139.85573812236655, 128.4691737860238, 162.5246962741358, 158.9677122108108, 133.99475046852996, 160.85107381385217]]</t>
         </is>
       </c>
     </row>
@@ -3046,14 +3046,14 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>13.99</t>
+          <t>14.0</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3063,7 +3063,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>143.49739156822292</t>
+          <t>149.2272068804102</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3073,12 +3073,12 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 12.0, 13.0, 16.0, 10.0, 14.0, 18.0, 20.0, 17.0], [10.0, 10.0, 17.0, 20.0, 18.0, 10.0, 10.0, 15.0, 14.0, 16.0], [12.0, 13.0, 17.0, 17.0, 17.0, 10.0, 10.0, 16.0, 18.0, 10.0], [10.0, 10.0, 12.0, 17.0, 17.0, 10.0, 13.0, 14.0, 20.0, 17.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [10.0, 10.0, 20.0, 15.0, 14.0, 10.0, 12.0, 13.0, 17.0, 19.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 16.0, 13.0, 18.0, 10.0, 10.0, 18.0, 18.0, 14.0], [10.0, 10.0, 17.0, 16.0, 15.0, 10.0, 10.0, 16.0, 19.0, 17.0], [10.0, 10.0, 14.0, 19.0, 17.0, 10.0, 13.0, 13.0, 17.0, 17.0], [10.0, 10.0, 17.0, 17.0, 13.0, 10.0, 13.0, 16.0, 16.0, 18.0], [13.0, 13.0, 10.0, 13.0, 13.0, 20.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 14.0, 18.0, 20.0, 10.0, 10.0, 20.0, 15.0, 13.0], [10.0, 10.0, 17.0, 14.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [10.0, 10.0, 18.0, 19.0, 15.0, 10.0, 13.0, 14.0, 18.0, 13.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 18.0, 16.0, 18.0, 13.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [13.0, 13.0, 16.0, 16.0, 14.0, 10.0, 10.0, 17.0, 18.0, 13.0], [18.0, 20.0, 10.0, 10.0, 15.0, 21.0, 16.0, 10.0, 10.0, 10.0], [20.0, 20.0, 13.0, 13.0, 14.0, 13.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 14.0, 19.0, 15.0, 10.0, 14.0, 14.0, 17.0, 17.0], [10.0, 10.0, 13.0, 18.0, 13.0, 10.0, 17.0, 17.0, 18.0, 14.0], [10.0, 15.0, 13.0, 16.0, 13.0, 10.0, 13.0, 16.0, 18.0, 16.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [20.0, 10.0, 16.0, 14.0, 13.0, 13.0, 12.0, 10.0, 17.0, 15.0], [10.0, 10.0, 17.0, 14.0, 13.0, 10.0, 13.0, 18.0, 18.0, 17.0], [10.0, 13.0, 16.0, 19.0, 17.0, 10.0, 10.0, 13.0, 19.0, 13.0], [10.0, 13.0, 16.0, 19.0, 17.0, 10.0, 10.0, 13.0, 19.0, 13.0], [10.0, 15.0, 13.0, 16.0, 13.0, 10.0, 13.0, 16.0, 18.0, 16.0], [10.0, 10.0, 18.0, 22.0, 16.0, 10.0, 10.0, 11.0, 18.0, 15.0], [10.0, 13.0, 18.0, 16.0, 18.0, 10.0, 10.0, 17.0, 14.0, 14.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 17.0, 17.0, 18.0, 13.0], [10.0, 10.0, 18.0, 20.0, 16.0, 10.0, 10.0, 15.0, 14.0, 17.0], [10.0, 10.0, 16.0, 17.0, 13.0, 10.0, 13.0, 13.0, 20.0, 18.0], [14.0, 10.0, 13.0, 17.0, 13.0, 10.0, 13.0, 16.0, 16.0, 18.0], [13.0, 13.0, 16.0, 16.0, 14.0, 10.0, 10.0, 17.0, 18.0, 13.0], [10.0, 10.0, 17.0, 18.0, 14.0, 10.0, 13.0, 17.0, 14.0, 17.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [10.0, 10.0, 13.0, 18.0, 13.0, 10.0, 16.0, 17.0, 17.0, 16.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 17.0, 16.0, 19.0, 13.0]]</t>
+          <t>[[15.0, 15.0, 13.0, 13.0, 14.0, 13.0, 15.0, 13.0, 15.0, 14.0], [16.0, 13.0, 15.0, 14.0, 14.0, 15.0, 14.0, 15.0, 12.0, 12.0], [12.0, 15.0, 16.0, 16.0, 10.0, 17.0, 12.0, 12.0, 15.0, 15.0], [14.0, 17.0, 14.0, 14.0, 14.0, 11.0, 14.0, 14.0, 14.0, 14.0], [14.0, 14.0, 15.0, 15.0, 10.0, 14.0, 14.0, 12.0, 17.0, 15.0]]</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>[[168.83996165156807, 123.59076141530063, 137.52389975446076, 156.56076627616952, 157.23945358979813, 102.19535536546157, 136.98234977747674, 148.11202772414816, 165.3966175086767, 168.1411905638944], [173.3778938221764, 121.08756093748445, 146.5913688266546, 154.40230569219315, 145.4947212627093, 103.72104361789681, 126.71084559796743, 151.73007906050145, 164.13194560985627, 156.0200638011278], [139.41539070961545, 114.54827561189082, 135.73475306205628, 140.81809021175053, 171.33152756667542, 119.20010596527693, 120.11723300749895, 148.21433184965375, 153.20138570473802, 156.95290611408822], [115.40154207344386, 89.81592503925985, 143.9484318186306, 167.27555292493275, 196.97953938222508, 68.16486543675677, 145.65137357476524, 149.6912349542489, 165.83173605452785, 185.4050771544179], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [155.30851665022445, 101.46766654749268, 157.67005968649443, 161.16074259334366, 147.0807205204198, 100.28855251190436, 152.95338094679695, 128.82601005018742, 171.6689462970614, 186.20394180285038], [151.49494337387458, 117.63970585649903, 163.36518294294515, 162.4387606206083, 155.6800257924122, 113.25638832677038, 117.6841561482807, 160.83878709456383, 159.34809118225894, 161.23989139159553], [155.31460127025164, 124.00260960556245, 148.60376550908018, 164.7376404534931, 161.71931721747035, 112.3850680839479, 114.1079803199717, 149.60165093783095, 157.59666266767624, 140.65031941257772], [116.75519767144029, 88.99311376250257, 147.25424111377666, 170.08749434033558, 210.62762868750434, 61.67641125468947, 143.08011862115282, 152.54965543170462, 163.87724299261785, 179.7845752589638], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [122.54784555544693, 105.96315511038627, 157.97711386986117, 155.2254321890902, 174.64839198201918, 107.4048115793619, 131.48313009343553, 148.92290625266523, 157.07933065148725, 176.82477881731256], [146.20595012109717, 107.72606078634776, 127.61892564766411, 149.657659086279, 157.6312372947903, 117.64141321293776, 148.9797225611856, 157.30202446272347, 170.27970250153555, 171.94398144716365], [150.1993569665729, 131.99208731713904, 128.39741381245582, 160.87672932697532, 168.04061575136942, 132.62874187680404, 115.66162008336777, 159.92133798709102, 143.37137005344712, 128.6220526614146], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [171.25214622653692, 122.04092166869397, 163.28536700743373, 146.08131701827855, 166.3694233187611, 102.3003445816535, 113.49515031953875, 154.10183902835064, 153.28354180543303, 143.2839025143099], [183.9641110300671, 146.9571103426829, 82.42156374434263, 110.54738368811277, 161.45011086895678, 163.2299709311923, 110.01291484769432, 125.46488882332544, 121.24645626255418, 135.87043875544455], [154.87670501106774, 124.45712875915734, 157.33520915081402, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 150.72696126211756, 153.1866101146596, 155.4404734500336], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096], [132.6393307913183, 109.30686173945848, 145.99049101750552, 152.59811248205753, 165.52450200376143, 117.34929630919373, 129.6409490643926, 152.35447181627313, 157.37714922337852, 161.60798730295116], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [165.24117105960053, 133.77087149912916, 129.9614208259944, 121.00987965148478, 124.0617095913029, 124.99420175139073, 145.07648926363632, 125.14749257346011, 133.51187048282097, 194.0374710761797], [148.65858587031735, 117.5537430787448, 152.7370674658746, 155.0185002942349, 147.46163154928857, 129.97949714189932, 132.1733655775968, 150.43382549066143, 156.29210499732608, 168.29369368023086], [154.87670501106774, 124.45712875915734, 157.33520915081402, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 150.72696126211756, 153.1866101146596, 155.4404734500336], [174.10245819655114, 127.80900078262174, 138.67139289299246, 148.41069607289663, 153.6350666551481, 103.46472832433717, 130.22281241842936, 147.4818180038071, 152.50682731933753, 157.6981277590819], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [163.82826724191202, 123.63300303116105, 162.8980670120787, 166.58612468713937, 158.67319842829247, 101.19007738890186, 123.85647903797361, 141.86796497619403, 159.9811243798996, 158.63953984939445], [145.0072351499823, 115.99968345962576, 160.68230623339542, 152.3530590210606, 167.1076278296097, 131.08931955966278, 114.54546057653036, 150.04147491293364, 155.30290240960926, 140.86380002454607], [149.7529984808466, 108.80052007547977, 124.96810248186745, 146.0270227777066, 171.51514835196625, 98.79095122172545, 131.01688305315017, 147.11708785009412, 174.0852436128256, 192.9599715968946], [144.55856538564217, 117.02977381184573, 151.09093700806469, 170.31849702527362, 189.88602050509368, 111.78524265062529, 106.75016416033765, 149.20146450350555, 161.4668277430309, 146.78621271509914], [140.2268461963245, 116.71115157478997, 146.52034871887318, 146.389151580322, 152.9818486418794, 106.05265716177503, 131.3508218040346, 147.3827546710329, 173.23148359875637, 165.37466641996363], [154.2527428966532, 117.80024702535607, 164.2594332885985, 167.82531633195677, 150.90075080208038, 111.02924005724354, 99.95541985534355, 162.24143788372814, 165.1755696808328, 156.3585509104705], [146.68028294257556, 110.73139395055306, 159.36968986240163, 152.35051116574624, 174.90210786655473, 131.88990376903146, 109.6514739753097, 149.19676116288565, 154.1348794612632, 141.82027184671585], [132.6393307913183, 109.30686173945848, 145.99049101750552, 152.59811248205753, 165.52450200376143, 117.34929630919373, 129.6409490643926, 152.35447181627313, 157.37714922337852, 161.60798730295116], [169.16533358350605, 125.2512122003425, 124.36982905582596, 152.3431774421878, 164.55270315503893, 99.58614228205624, 138.9677058715599, 154.38699831564628, 167.33125598678217, 152.1864118047564], [151.3848407559981, 117.35033497131577, 159.26754100958533, 179.77760037675822, 149.5328415957601, 113.27968378965878, 123.670636716717, 153.30867936653834, 162.3419977297616, 155.28502904089973], [138.20605623854652, 107.42348781850717, 129.21584774205314, 142.2134787300486, 192.8664244086329, 96.20732846975696, 131.92385143024265, 156.3132038929684, 172.34092474542578, 184.7627903630174]]</t>
+          <t>[[151.5904775392701, 140.93997647537367, 182.34268053115142, 125.26539149020961, 156.17033981043602, 139.3234450804238, 161.91514672937646, 121.84641424414177, 164.48720643191052, 148.79759694354027], [137.8139116968595, 140.024602473143, 153.6301703941588, 137.55598113882863, 161.91691732492257, 153.35054557048392, 159.13582274127816, 129.0626600637646, 168.18969900218755, 153.23295666986388], [119.24348018897318, 140.6232476640788, 156.82330941144463, 150.88578355996657, 153.63350745236562, 141.97098956575928, 136.23247201817628, 136.28088045686994, 167.2024342486018, 188.09007117433518], [148.08448385490908, 169.23975747188229, 160.0760732327987, 137.41674538873897, 147.46242365783883, 150.092462404935, 140.8128454298999, 145.60045286765794, 144.52443153804833, 149.48934260561902], [156.4988620695711, 149.92914792978195, 167.92443652411157, 151.8357841959097, 151.72876979628322, 151.47218588299955, 153.95700462057863, 124.4819646762756, 131.92222113808893, 151.2328306426858]]</t>
         </is>
       </c>
     </row>
@@ -3099,14 +3099,14 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>13.991111111111113</t>
+          <t>14.0</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>143.50815983196094</t>
+          <t>149.17675015595498</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3126,118 +3126,12 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>[[10.0, 10.0, 12.0, 13.0, 16.0, 10.0, 14.0, 18.0, 20.0, 17.0], [10.0, 10.0, 17.0, 20.0, 18.0, 10.0, 10.0, 15.0, 14.0, 16.0], [12.0, 13.0, 17.0, 17.0, 17.0, 10.0, 10.0, 16.0, 18.0, 10.0], [10.0, 10.0, 12.0, 17.0, 17.0, 10.0, 13.0, 14.0, 20.0, 17.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [10.0, 10.0, 20.0, 15.0, 14.0, 10.0, 12.0, 13.0, 17.0, 19.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 16.0, 13.0, 18.0, 10.0, 10.0, 18.0, 18.0, 14.0], [10.0, 10.0, 17.0, 16.0, 15.0, 10.0, 10.0, 16.0, 19.0, 17.0], [10.0, 10.0, 14.0, 19.0, 17.0, 10.0, 13.0, 13.0, 17.0, 17.0], [10.0, 10.0, 17.0, 17.0, 13.0, 10.0, 13.0, 16.0, 16.0, 18.0], [13.0, 13.0, 10.0, 13.0, 13.0, 20.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 14.0, 18.0, 20.0, 10.0, 10.0, 20.0, 15.0, 13.0], [10.0, 10.0, 17.0, 14.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [10.0, 10.0, 18.0, 19.0, 15.0, 10.0, 13.0, 14.0, 18.0, 13.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 18.0, 16.0, 18.0, 13.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [13.0, 13.0, 16.0, 16.0, 14.0, 10.0, 10.0, 17.0, 18.0, 13.0], [18.0, 20.0, 10.0, 10.0, 15.0, 21.0, 16.0, 10.0, 10.0, 10.0], [20.0, 20.0, 13.0, 13.0, 14.0, 13.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 14.0, 19.0, 15.0, 10.0, 14.0, 14.0, 17.0, 17.0], [10.0, 10.0, 13.0, 18.0, 13.0, 10.0, 17.0, 17.0, 18.0, 14.0], [10.0, 15.0, 13.0, 16.0, 13.0, 10.0, 13.0, 16.0, 18.0, 16.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [20.0, 10.0, 16.0, 14.0, 13.0, 13.0, 12.0, 10.0, 17.0, 15.0], [10.0, 10.0, 17.0, 14.0, 13.0, 10.0, 13.0, 18.0, 18.0, 17.0], [10.0, 13.0, 16.0, 19.0, 17.0, 10.0, 10.0, 13.0, 19.0, 13.0], [10.0, 13.0, 16.0, 19.0, 17.0, 10.0, 10.0, 13.0, 19.0, 13.0], [10.0, 15.0, 13.0, 16.0, 13.0, 10.0, 13.0, 16.0, 18.0, 16.0], [10.0, 10.0, 18.0, 22.0, 16.0, 10.0, 10.0, 11.0, 18.0, 15.0], [10.0, 13.0, 18.0, 16.0, 18.0, 10.0, 10.0, 17.0, 14.0, 14.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 17.0, 17.0, 18.0, 13.0], [10.0, 10.0, 18.0, 20.0, 16.0, 10.0, 10.0, 15.0, 14.0, 17.0], [10.0, 10.0, 16.0, 17.0, 13.0, 10.0, 13.0, 13.0, 20.0, 18.0], [14.0, 10.0, 13.0, 17.0, 13.0, 10.0, 13.0, 16.0, 16.0, 18.0], [13.0, 13.0, 16.0, 16.0, 14.0, 10.0, 10.0, 17.0, 18.0, 13.0], [10.0, 10.0, 17.0, 18.0, 14.0, 10.0, 13.0, 17.0, 14.0, 17.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [10.0, 10.0, 13.0, 18.0, 13.0, 10.0, 16.0, 17.0, 17.0, 16.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 17.0, 16.0, 19.0, 13.0], [17.0, 10.0, 14.0, 15.0, 13.0, 15.0, 15.0, 14.0, 10.0, 17.0], [10.0, 10.0, 18.0, 16.0, 17.0, 10.0, 14.0, 18.0, 14.0, 13.0], [10.0, 13.0, 15.0, 17.0, 17.0, 10.0, 12.0, 16.0, 19.0, 11.0], [10.0, 10.0, 14.0, 18.0, 20.0, 10.0, 10.0, 20.0, 15.0, 13.0], [10.0, 10.0, 17.0, 14.0, 13.0, 10.0, 14.0, 18.0, 18.0, 16.0]]</t>
+          <t>[[13.0, 12.0, 13.0, 15.0, 15.0, 15.0, 14.0, 14.0, 16.0, 13.0], [13.0, 14.0, 12.0, 17.0, 14.0, 13.0, 14.0, 14.0, 14.0, 15.0], [15.0, 12.0, 15.0, 15.0, 14.0, 15.0, 13.0, 15.0, 14.0, 12.0], [15.0, 14.0, 15.0, 14.0, 14.0, 13.0, 15.0, 14.0, 14.0, 12.0], [13.0, 15.0, 12.0, 15.0, 14.0, 13.0, 14.0, 16.0, 14.0, 14.0]]</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>[[168.83996165156807, 123.59076141530063, 137.52389975446076, 156.56076627616952, 157.23945358979813, 102.19535536546157, 136.98234977747674, 148.11202772414816, 165.3966175086767, 168.1411905638944], [173.3778938221764, 121.08756093748445, 146.5913688266546, 154.40230569219315, 145.4947212627093, 103.72104361789681, 126.71084559796743, 151.73007906050145, 164.13194560985627, 156.0200638011278], [139.41539070961545, 114.54827561189082, 135.73475306205628, 140.81809021175053, 171.33152756667542, 119.20010596527693, 120.11723300749895, 148.21433184965375, 153.20138570473802, 156.95290611408822], [115.40154207344386, 89.81592503925985, 143.9484318186306, 167.27555292493275, 196.97953938222508, 68.16486543675677, 145.65137357476524, 149.6912349542489, 165.83173605452785, 185.4050771544179], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [155.30851665022445, 101.46766654749268, 157.67005968649443, 161.16074259334366, 147.0807205204198, 100.28855251190436, 152.95338094679695, 128.82601005018742, 171.6689462970614, 186.20394180285038], [151.49494337387458, 117.63970585649903, 163.36518294294515, 162.4387606206083, 155.6800257924122, 113.25638832677038, 117.6841561482807, 160.83878709456383, 159.34809118225894, 161.23989139159553], [155.31460127025164, 124.00260960556245, 148.60376550908018, 164.7376404534931, 161.71931721747035, 112.3850680839479, 114.1079803199717, 149.60165093783095, 157.59666266767624, 140.65031941257772], [116.75519767144029, 88.99311376250257, 147.25424111377666, 170.08749434033558, 210.62762868750434, 61.67641125468947, 143.08011862115282, 152.54965543170462, 163.87724299261785, 179.7845752589638], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [122.54784555544693, 105.96315511038627, 157.97711386986117, 155.2254321890902, 174.64839198201918, 107.4048115793619, 131.48313009343553, 148.92290625266523, 157.07933065148725, 176.82477881731256], [146.20595012109717, 107.72606078634776, 127.61892564766411, 149.657659086279, 157.6312372947903, 117.64141321293776, 148.9797225611856, 157.30202446272347, 170.27970250153555, 171.94398144716365], [150.1993569665729, 131.99208731713904, 128.39741381245582, 160.87672932697532, 168.04061575136942, 132.62874187680404, 115.66162008336777, 159.92133798709102, 143.37137005344712, 128.6220526614146], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [171.25214622653692, 122.04092166869397, 163.28536700743373, 146.08131701827855, 166.3694233187611, 102.3003445816535, 113.49515031953875, 154.10183902835064, 153.28354180543303, 143.2839025143099], [183.9641110300671, 146.9571103426829, 82.42156374434263, 110.54738368811277, 161.45011086895678, 163.2299709311923, 110.01291484769432, 125.46488882332544, 121.24645626255418, 135.87043875544455], [154.87670501106774, 124.45712875915734, 157.33520915081402, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 150.72696126211756, 153.1866101146596, 155.4404734500336], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096], [132.6393307913183, 109.30686173945848, 145.99049101750552, 152.59811248205753, 165.52450200376143, 117.34929630919373, 129.6409490643926, 152.35447181627313, 157.37714922337852, 161.60798730295116], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [165.24117105960053, 133.77087149912916, 129.9614208259944, 121.00987965148478, 124.0617095913029, 124.99420175139073, 145.07648926363632, 125.14749257346011, 133.51187048282097, 194.0374710761797], [148.65858587031735, 117.5537430787448, 152.7370674658746, 155.0185002942349, 147.46163154928857, 129.97949714189932, 132.1733655775968, 150.43382549066143, 156.29210499732608, 168.29369368023086], [154.87670501106774, 124.45712875915734, 157.33520915081402, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 150.72696126211756, 153.1866101146596, 155.4404734500336], [174.10245819655114, 127.80900078262174, 138.67139289299246, 148.41069607289663, 153.6350666551481, 103.46472832433717, 130.22281241842936, 147.4818180038071, 152.50682731933753, 157.6981277590819], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [163.82826724191202, 123.63300303116105, 162.8980670120787, 166.58612468713937, 158.67319842829247, 101.19007738890186, 123.85647903797361, 141.86796497619403, 159.9811243798996, 158.63953984939445], [145.0072351499823, 115.99968345962576, 160.68230623339542, 152.3530590210606, 167.1076278296097, 131.08931955966278, 114.54546057653036, 150.04147491293364, 155.30290240960926, 140.86380002454607], [149.7529984808466, 108.80052007547977, 124.96810248186745, 146.0270227777066, 171.51514835196625, 98.79095122172545, 131.01688305315017, 147.11708785009412, 174.0852436128256, 192.9599715968946], [144.55856538564217, 117.02977381184573, 151.09093700806469, 170.31849702527362, 189.88602050509368, 111.78524265062529, 106.75016416033765, 149.20146450350555, 161.4668277430309, 146.78621271509914], [140.2268461963245, 116.71115157478997, 146.52034871887318, 146.389151580322, 152.9818486418794, 106.05265716177503, 131.3508218040346, 147.3827546710329, 173.23148359875637, 165.37466641996363], [154.2527428966532, 117.80024702535607, 164.2594332885985, 167.82531633195677, 150.90075080208038, 111.02924005724354, 99.95541985534355, 162.24143788372814, 165.1755696808328, 156.3585509104705], [146.68028294257556, 110.73139395055306, 159.36968986240163, 152.35051116574624, 174.90210786655473, 131.88990376903146, 109.6514739753097, 149.19676116288565, 154.1348794612632, 141.82027184671585], [132.6393307913183, 109.30686173945848, 145.99049101750552, 152.59811248205753, 165.52450200376143, 117.34929630919373, 129.6409490643926, 152.35447181627313, 157.37714922337852, 161.60798730295116], [169.16533358350605, 125.2512122003425, 124.36982905582596, 152.3431774421878, 164.55270315503893, 99.58614228205624, 138.9677058715599, 154.38699831564628, 167.33125598678217, 152.1864118047564], [151.3848407559981, 117.35033497131577, 159.26754100958533, 179.77760037675822, 149.5328415957601, 113.27968378965878, 123.670636716717, 153.30867936653834, 162.3419977297616, 155.28502904089973], [138.20605623854652, 107.42348781850717, 129.21584774205314, 142.2134787300486, 192.8664244086329, 96.20732846975696, 131.92385143024265, 156.3132038929684, 172.34092474542578, 184.7627903630174], [155.31948812344817, 103.54968781024894, 155.54440994011514, 159.64573144883576, 147.03153222429555, 100.29278139457293, 152.96449306880106, 129.3847328892758, 172.26759503296182, 186.13756010516815], [124.60931392388997, 99.55757900064643, 161.99929959628253, 150.1285082839572, 186.11983693459018, 86.00430019489998, 119.13204577034072, 155.41436252761594, 169.16448238826908, 170.3493231523084], [155.31460127025164, 124.00260960556245, 148.60376550908018, 164.7376404534931, 161.71931721747035, 112.3850680839479, 114.1079803199717, 149.60165093783095, 157.59666266767624, 140.65031941257772], [153.1476310248567, 118.1329600449769, 129.3980487071801, 158.37058800553137, 170.7977841821514, 107.94684317141325, 122.26963812067054, 161.0180127552807, 144.70026811490482, 151.10468681449436], [149.0250338729308, 116.77434277151853, 162.14817871023328, 165.63041794718413, 164.30078521222296, 111.43165327141746, 95.09076225078535, 162.21262866457795, 165.63738490665054, 157.24096925588108]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>mixedSelfPlay.csv</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>[4, 3]</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>SelfPlay</t>
-        </is>
-      </c>
-      <c r="D52" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E52" t="b">
-        <v>0</v>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>13.992</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>NAN</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>143.6195111430212</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>NAN</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>[[10.0, 10.0, 12.0, 13.0, 16.0, 10.0, 14.0, 18.0, 20.0, 17.0], [10.0, 10.0, 17.0, 20.0, 18.0, 10.0, 10.0, 15.0, 14.0, 16.0], [12.0, 13.0, 17.0, 17.0, 17.0, 10.0, 10.0, 16.0, 18.0, 10.0], [10.0, 10.0, 12.0, 17.0, 17.0, 10.0, 13.0, 14.0, 20.0, 17.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [10.0, 10.0, 20.0, 15.0, 14.0, 10.0, 12.0, 13.0, 17.0, 19.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 16.0, 13.0, 18.0, 10.0, 10.0, 18.0, 18.0, 14.0], [10.0, 10.0, 17.0, 16.0, 15.0, 10.0, 10.0, 16.0, 19.0, 17.0], [10.0, 10.0, 14.0, 19.0, 17.0, 10.0, 13.0, 13.0, 17.0, 17.0], [10.0, 10.0, 17.0, 17.0, 13.0, 10.0, 13.0, 16.0, 16.0, 18.0], [13.0, 13.0, 10.0, 13.0, 13.0, 20.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 14.0, 18.0, 20.0, 10.0, 10.0, 20.0, 15.0, 13.0], [10.0, 10.0, 17.0, 14.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [10.0, 10.0, 18.0, 19.0, 15.0, 10.0, 13.0, 14.0, 18.0, 13.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 18.0, 16.0, 18.0, 13.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [13.0, 13.0, 16.0, 16.0, 14.0, 10.0, 10.0, 17.0, 18.0, 13.0], [18.0, 20.0, 10.0, 10.0, 15.0, 21.0, 16.0, 10.0, 10.0, 10.0], [20.0, 20.0, 13.0, 13.0, 14.0, 13.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 14.0, 19.0, 15.0, 10.0, 14.0, 14.0, 17.0, 17.0], [10.0, 10.0, 13.0, 18.0, 13.0, 10.0, 17.0, 17.0, 18.0, 14.0], [10.0, 15.0, 13.0, 16.0, 13.0, 10.0, 13.0, 16.0, 18.0, 16.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [20.0, 10.0, 16.0, 14.0, 13.0, 13.0, 12.0, 10.0, 17.0, 15.0], [10.0, 10.0, 17.0, 14.0, 13.0, 10.0, 13.0, 18.0, 18.0, 17.0], [10.0, 13.0, 16.0, 19.0, 17.0, 10.0, 10.0, 13.0, 19.0, 13.0], [10.0, 13.0, 16.0, 19.0, 17.0, 10.0, 10.0, 13.0, 19.0, 13.0], [10.0, 15.0, 13.0, 16.0, 13.0, 10.0, 13.0, 16.0, 18.0, 16.0], [10.0, 10.0, 18.0, 22.0, 16.0, 10.0, 10.0, 11.0, 18.0, 15.0], [10.0, 13.0, 18.0, 16.0, 18.0, 10.0, 10.0, 17.0, 14.0, 14.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 17.0, 17.0, 18.0, 13.0], [10.0, 10.0, 18.0, 20.0, 16.0, 10.0, 10.0, 15.0, 14.0, 17.0], [10.0, 10.0, 16.0, 17.0, 13.0, 10.0, 13.0, 13.0, 20.0, 18.0], [14.0, 10.0, 13.0, 17.0, 13.0, 10.0, 13.0, 16.0, 16.0, 18.0], [13.0, 13.0, 16.0, 16.0, 14.0, 10.0, 10.0, 17.0, 18.0, 13.0], [10.0, 10.0, 17.0, 18.0, 14.0, 10.0, 13.0, 17.0, 14.0, 17.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [10.0, 10.0, 13.0, 18.0, 13.0, 10.0, 16.0, 17.0, 17.0, 16.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 17.0, 16.0, 19.0, 13.0], [17.0, 10.0, 14.0, 15.0, 13.0, 15.0, 15.0, 14.0, 10.0, 17.0], [10.0, 10.0, 18.0, 16.0, 17.0, 10.0, 14.0, 18.0, 14.0, 13.0], [10.0, 13.0, 15.0, 17.0, 17.0, 10.0, 12.0, 16.0, 19.0, 11.0], [10.0, 10.0, 14.0, 18.0, 20.0, 10.0, 10.0, 20.0, 15.0, 13.0], [10.0, 10.0, 17.0, 14.0, 13.0, 10.0, 14.0, 18.0, 18.0, 16.0], [10.0, 10.0, 13.0, 18.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [18.0, 16.0, 13.0, 14.0, 10.0, 16.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 10.0, 14.0, 18.0, 20.0, 10.0, 10.0, 20.0, 15.0, 13.0], [10.0, 10.0, 14.0, 20.0, 16.0, 10.0, 10.0, 15.0, 18.0, 17.0]]</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>[[168.83996165156807, 123.59076141530063, 137.52389975446076, 156.56076627616952, 157.23945358979813, 102.19535536546157, 136.98234977747674, 148.11202772414816, 165.3966175086767, 168.1411905638944], [173.3778938221764, 121.08756093748445, 146.5913688266546, 154.40230569219315, 145.4947212627093, 103.72104361789681, 126.71084559796743, 151.73007906050145, 164.13194560985627, 156.0200638011278], [139.41539070961545, 114.54827561189082, 135.73475306205628, 140.81809021175053, 171.33152756667542, 119.20010596527693, 120.11723300749895, 148.21433184965375, 153.20138570473802, 156.95290611408822], [115.40154207344386, 89.81592503925985, 143.9484318186306, 167.27555292493275, 196.97953938222508, 68.16486543675677, 145.65137357476524, 149.6912349542489, 165.83173605452785, 185.4050771544179], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [155.30851665022445, 101.46766654749268, 157.67005968649443, 161.16074259334366, 147.0807205204198, 100.28855251190436, 152.95338094679695, 128.82601005018742, 171.6689462970614, 186.20394180285038], [151.49494337387458, 117.63970585649903, 163.36518294294515, 162.4387606206083, 155.6800257924122, 113.25638832677038, 117.6841561482807, 160.83878709456383, 159.34809118225894, 161.23989139159553], [155.31460127025164, 124.00260960556245, 148.60376550908018, 164.7376404534931, 161.71931721747035, 112.3850680839479, 114.1079803199717, 149.60165093783095, 157.59666266767624, 140.65031941257772], [116.75519767144029, 88.99311376250257, 147.25424111377666, 170.08749434033558, 210.62762868750434, 61.67641125468947, 143.08011862115282, 152.54965543170462, 163.87724299261785, 179.7845752589638], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [122.54784555544693, 105.96315511038627, 157.97711386986117, 155.2254321890902, 174.64839198201918, 107.4048115793619, 131.48313009343553, 148.92290625266523, 157.07933065148725, 176.82477881731256], [146.20595012109717, 107.72606078634776, 127.61892564766411, 149.657659086279, 157.6312372947903, 117.64141321293776, 148.9797225611856, 157.30202446272347, 170.27970250153555, 171.94398144716365], [150.1993569665729, 131.99208731713904, 128.39741381245582, 160.87672932697532, 168.04061575136942, 132.62874187680404, 115.66162008336777, 159.92133798709102, 143.37137005344712, 128.6220526614146], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [171.25214622653692, 122.04092166869397, 163.28536700743373, 146.08131701827855, 166.3694233187611, 102.3003445816535, 113.49515031953875, 154.10183902835064, 153.28354180543303, 143.2839025143099], [183.9641110300671, 146.9571103426829, 82.42156374434263, 110.54738368811277, 161.45011086895678, 163.2299709311923, 110.01291484769432, 125.46488882332544, 121.24645626255418, 135.87043875544455], [154.87670501106774, 124.45712875915734, 157.33520915081402, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 150.72696126211756, 153.1866101146596, 155.4404734500336], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096], [132.6393307913183, 109.30686173945848, 145.99049101750552, 152.59811248205753, 165.52450200376143, 117.34929630919373, 129.6409490643926, 152.35447181627313, 157.37714922337852, 161.60798730295116], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [165.24117105960053, 133.77087149912916, 129.9614208259944, 121.00987965148478, 124.0617095913029, 124.99420175139073, 145.07648926363632, 125.14749257346011, 133.51187048282097, 194.0374710761797], [148.65858587031735, 117.5537430787448, 152.7370674658746, 155.0185002942349, 147.46163154928857, 129.97949714189932, 132.1733655775968, 150.43382549066143, 156.29210499732608, 168.29369368023086], [154.87670501106774, 124.45712875915734, 157.33520915081402, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 150.72696126211756, 153.1866101146596, 155.4404734500336], [174.10245819655114, 127.80900078262174, 138.67139289299246, 148.41069607289663, 153.6350666551481, 103.46472832433717, 130.22281241842936, 147.4818180038071, 152.50682731933753, 157.6981277590819], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [163.82826724191202, 123.63300303116105, 162.8980670120787, 166.58612468713937, 158.67319842829247, 101.19007738890186, 123.85647903797361, 141.86796497619403, 159.9811243798996, 158.63953984939445], [145.0072351499823, 115.99968345962576, 160.68230623339542, 152.3530590210606, 167.1076278296097, 131.08931955966278, 114.54546057653036, 150.04147491293364, 155.30290240960926, 140.86380002454607], [149.7529984808466, 108.80052007547977, 124.96810248186745, 146.0270227777066, 171.51514835196625, 98.79095122172545, 131.01688305315017, 147.11708785009412, 174.0852436128256, 192.9599715968946], [144.55856538564217, 117.02977381184573, 151.09093700806469, 170.31849702527362, 189.88602050509368, 111.78524265062529, 106.75016416033765, 149.20146450350555, 161.4668277430309, 146.78621271509914], [140.2268461963245, 116.71115157478997, 146.52034871887318, 146.389151580322, 152.9818486418794, 106.05265716177503, 131.3508218040346, 147.3827546710329, 173.23148359875637, 165.37466641996363], [154.2527428966532, 117.80024702535607, 164.2594332885985, 167.82531633195677, 150.90075080208038, 111.02924005724354, 99.95541985534355, 162.24143788372814, 165.1755696808328, 156.3585509104705], [146.68028294257556, 110.73139395055306, 159.36968986240163, 152.35051116574624, 174.90210786655473, 131.88990376903146, 109.6514739753097, 149.19676116288565, 154.1348794612632, 141.82027184671585], [132.6393307913183, 109.30686173945848, 145.99049101750552, 152.59811248205753, 165.52450200376143, 117.34929630919373, 129.6409490643926, 152.35447181627313, 157.37714922337852, 161.60798730295116], [169.16533358350605, 125.2512122003425, 124.36982905582596, 152.3431774421878, 164.55270315503893, 99.58614228205624, 138.9677058715599, 154.38699831564628, 167.33125598678217, 152.1864118047564], [151.3848407559981, 117.35033497131577, 159.26754100958533, 179.77760037675822, 149.5328415957601, 113.27968378965878, 123.670636716717, 153.30867936653834, 162.3419977297616, 155.28502904089973], [138.20605623854652, 107.42348781850717, 129.21584774205314, 142.2134787300486, 192.8664244086329, 96.20732846975696, 131.92385143024265, 156.3132038929684, 172.34092474542578, 184.7627903630174], [155.31948812344817, 103.54968781024894, 155.54440994011514, 159.64573144883576, 147.03153222429555, 100.29278139457293, 152.96449306880106, 129.3847328892758, 172.26759503296182, 186.13756010516815], [124.60931392388997, 99.55757900064643, 161.99929959628253, 150.1285082839572, 186.11983693459018, 86.00430019489998, 119.13204577034072, 155.41436252761594, 169.16448238826908, 170.3493231523084], [155.31460127025164, 124.00260960556245, 148.60376550908018, 164.7376404534931, 161.71931721747035, 112.3850680839479, 114.1079803199717, 149.60165093783095, 157.59666266767624, 140.65031941257772], [153.1476310248567, 118.1329600449769, 129.3980487071801, 158.37058800553137, 170.7977841821514, 107.94684317141325, 122.26963812067054, 161.0180127552807, 144.70026811490482, 151.10468681449436], [149.0250338729308, 116.77434277151853, 162.14817871023328, 165.63041794718413, 164.30078521222296, 111.43165327141746, 95.09076225078535, 162.21262866457795, 165.63738490665054, 157.24096925588108], [167.0289090491371, 124.30893920494574, 153.50285471754952, 158.8221000494878, 140.38758830030181, 101.42229138743608, 136.09796166251127, 155.39385433707233, 159.10033495026562, 159.92079055338738], [167.0289090491371, 124.30893920494574, 153.50285471754952, 158.8221000494878, 140.38758830030181, 101.42229138743608, 136.09796166251127, 155.39385433707233, 159.10033495026562, 159.92079055338738], [151.49494337387458, 117.63970585649903, 163.36518294294515, 162.4387606206083, 155.6800257924122, 113.25638832677038, 117.6841561482807, 160.83878709456383, 159.34809118225894, 161.23989139159553], [152.7282052709074, 130.41874324998875, 125.82420113609076, 156.97943007117505, 157.16274510072986, 126.51035377237639, 132.61048893821945, 159.55495885505314, 143.6280207101792, 136.0236397347833], [116.75519767144029, 88.99311376250257, 147.25424111377666, 170.08749434033558, 210.62762868750434, 61.67641125468947, 143.08011862115282, 152.54965543170462, 163.87724299261785, 179.7845752589638]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>mixedSelfPlay.csv</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>[4, 3]</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>SelfPlay</t>
-        </is>
-      </c>
-      <c r="D53" t="n">
-        <v>1</v>
-      </c>
-      <c r="E53" t="b">
-        <v>0</v>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>13.992727272727274</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>NAN</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>143.64991954971873</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>NAN</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>[[10.0, 10.0, 12.0, 13.0, 16.0, 10.0, 14.0, 18.0, 20.0, 17.0], [10.0, 10.0, 17.0, 20.0, 18.0, 10.0, 10.0, 15.0, 14.0, 16.0], [12.0, 13.0, 17.0, 17.0, 17.0, 10.0, 10.0, 16.0, 18.0, 10.0], [10.0, 10.0, 12.0, 17.0, 17.0, 10.0, 13.0, 14.0, 20.0, 17.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [10.0, 10.0, 20.0, 15.0, 14.0, 10.0, 12.0, 13.0, 17.0, 19.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 13.0, 16.0, 13.0, 18.0, 10.0, 10.0, 18.0, 18.0, 14.0], [10.0, 10.0, 17.0, 16.0, 15.0, 10.0, 10.0, 16.0, 19.0, 17.0], [10.0, 10.0, 14.0, 19.0, 17.0, 10.0, 13.0, 13.0, 17.0, 17.0], [10.0, 10.0, 17.0, 17.0, 13.0, 10.0, 13.0, 16.0, 16.0, 18.0], [13.0, 13.0, 10.0, 13.0, 13.0, 20.0, 13.0, 13.0, 15.0, 13.0], [10.0, 10.0, 14.0, 18.0, 20.0, 10.0, 10.0, 20.0, 15.0, 13.0], [10.0, 10.0, 17.0, 14.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [10.0, 10.0, 18.0, 19.0, 15.0, 10.0, 13.0, 14.0, 18.0, 13.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 18.0, 16.0, 18.0, 13.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [13.0, 13.0, 16.0, 16.0, 14.0, 10.0, 10.0, 17.0, 18.0, 13.0], [18.0, 20.0, 10.0, 10.0, 15.0, 21.0, 16.0, 10.0, 10.0, 10.0], [20.0, 20.0, 13.0, 13.0, 14.0, 13.0, 10.0, 13.0, 14.0, 10.0], [10.0, 10.0, 14.0, 19.0, 15.0, 10.0, 14.0, 14.0, 17.0, 17.0], [10.0, 10.0, 13.0, 18.0, 13.0, 10.0, 17.0, 17.0, 18.0, 14.0], [10.0, 15.0, 13.0, 16.0, 13.0, 10.0, 13.0, 16.0, 18.0, 16.0], [14.0, 14.0, 16.0, 10.0, 14.0, 14.0, 12.0, 10.0, 17.0, 19.0], [20.0, 10.0, 16.0, 14.0, 13.0, 13.0, 12.0, 10.0, 17.0, 15.0], [10.0, 10.0, 17.0, 14.0, 13.0, 10.0, 13.0, 18.0, 18.0, 17.0], [10.0, 13.0, 16.0, 19.0, 17.0, 10.0, 10.0, 13.0, 19.0, 13.0], [10.0, 13.0, 16.0, 19.0, 17.0, 10.0, 10.0, 13.0, 19.0, 13.0], [10.0, 15.0, 13.0, 16.0, 13.0, 10.0, 13.0, 16.0, 18.0, 16.0], [10.0, 10.0, 18.0, 22.0, 16.0, 10.0, 10.0, 11.0, 18.0, 15.0], [10.0, 13.0, 18.0, 16.0, 18.0, 10.0, 10.0, 17.0, 14.0, 14.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 17.0, 17.0, 18.0, 13.0], [10.0, 10.0, 18.0, 20.0, 16.0, 10.0, 10.0, 15.0, 14.0, 17.0], [10.0, 10.0, 16.0, 17.0, 13.0, 10.0, 13.0, 13.0, 20.0, 18.0], [14.0, 10.0, 13.0, 17.0, 13.0, 10.0, 13.0, 16.0, 16.0, 18.0], [13.0, 13.0, 16.0, 16.0, 14.0, 10.0, 10.0, 17.0, 18.0, 13.0], [10.0, 10.0, 17.0, 18.0, 14.0, 10.0, 13.0, 17.0, 14.0, 17.0], [10.0, 10.0, 14.0, 17.0, 17.0, 10.0, 13.0, 17.0, 15.0, 17.0], [10.0, 10.0, 13.0, 18.0, 13.0, 10.0, 16.0, 17.0, 17.0, 16.0], [10.0, 10.0, 13.0, 16.0, 16.0, 10.0, 17.0, 16.0, 19.0, 13.0], [17.0, 10.0, 14.0, 15.0, 13.0, 15.0, 15.0, 14.0, 10.0, 17.0], [10.0, 10.0, 18.0, 16.0, 17.0, 10.0, 14.0, 18.0, 14.0, 13.0], [10.0, 13.0, 15.0, 17.0, 17.0, 10.0, 12.0, 16.0, 19.0, 11.0], [10.0, 10.0, 14.0, 18.0, 20.0, 10.0, 10.0, 20.0, 15.0, 13.0], [10.0, 10.0, 17.0, 14.0, 13.0, 10.0, 14.0, 18.0, 18.0, 16.0], [10.0, 10.0, 13.0, 18.0, 14.0, 10.0, 13.0, 17.0, 18.0, 17.0], [18.0, 16.0, 13.0, 14.0, 10.0, 16.0, 13.0, 13.0, 14.0, 13.0], [10.0, 10.0, 17.0, 20.0, 13.0, 10.0, 13.0, 13.0, 18.0, 16.0], [10.0, 10.0, 14.0, 18.0, 20.0, 10.0, 10.0, 20.0, 15.0, 13.0], [10.0, 10.0, 14.0, 20.0, 16.0, 10.0, 10.0, 15.0, 18.0, 17.0], [13.0, 10.0, 18.0, 17.0, 14.0, 10.0, 10.0, 18.0, 13.0, 17.0], [16.0, 15.0, 14.0, 17.0, 14.0, 10.0, 16.0, 15.0, 10.0, 13.0], [10.0, 10.0, 13.0, 17.0, 16.0, 10.0, 17.0, 16.0, 18.0, 13.0], [10.0, 10.0, 16.0, 19.0, 13.0, 10.0, 16.0, 16.0, 17.0, 13.0], [10.0, 10.0, 12.0, 13.0, 17.0, 10.0, 14.0, 18.0, 19.0, 17.0]]</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>[[168.83996165156807, 123.59076141530063, 137.52389975446076, 156.56076627616952, 157.23945358979813, 102.19535536546157, 136.98234977747674, 148.11202772414816, 165.3966175086767, 168.1411905638944], [173.3778938221764, 121.08756093748445, 146.5913688266546, 154.40230569219315, 145.4947212627093, 103.72104361789681, 126.71084559796743, 151.73007906050145, 164.13194560985627, 156.0200638011278], [139.41539070961545, 114.54827561189082, 135.73475306205628, 140.81809021175053, 171.33152756667542, 119.20010596527693, 120.11723300749895, 148.21433184965375, 153.20138570473802, 156.95290611408822], [115.40154207344386, 89.81592503925985, 143.9484318186306, 167.27555292493275, 196.97953938222508, 68.16486543675677, 145.65137357476524, 149.6912349542489, 165.83173605452785, 185.4050771544179], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [155.30851665022445, 101.46766654749268, 157.67005968649443, 161.16074259334366, 147.0807205204198, 100.28855251190436, 152.95338094679695, 128.82601005018742, 171.6689462970614, 186.20394180285038], [151.49494337387458, 117.63970585649903, 163.36518294294515, 162.4387606206083, 155.6800257924122, 113.25638832677038, 117.6841561482807, 160.83878709456383, 159.34809118225894, 161.23989139159553], [155.31460127025164, 124.00260960556245, 148.60376550908018, 164.7376404534931, 161.71931721747035, 112.3850680839479, 114.1079803199717, 149.60165093783095, 157.59666266767624, 140.65031941257772], [116.75519767144029, 88.99311376250257, 147.25424111377666, 170.08749434033558, 210.62762868750434, 61.67641125468947, 143.08011862115282, 152.54965543170462, 163.87724299261785, 179.7845752589638], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [122.54784555544693, 105.96315511038627, 157.97711386986117, 155.2254321890902, 174.64839198201918, 107.4048115793619, 131.48313009343553, 148.92290625266523, 157.07933065148725, 176.82477881731256], [146.20595012109717, 107.72606078634776, 127.61892564766411, 149.657659086279, 157.6312372947903, 117.64141321293776, 148.9797225611856, 157.30202446272347, 170.27970250153555, 171.94398144716365], [150.1993569665729, 131.99208731713904, 128.39741381245582, 160.87672932697532, 168.04061575136942, 132.62874187680404, 115.66162008336777, 159.92133798709102, 143.37137005344712, 128.6220526614146], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006], [171.25214622653692, 122.04092166869397, 163.28536700743373, 146.08131701827855, 166.3694233187611, 102.3003445816535, 113.49515031953875, 154.10183902835064, 153.28354180543303, 143.2839025143099], [183.9641110300671, 146.9571103426829, 82.42156374434263, 110.54738368811277, 161.45011086895678, 163.2299709311923, 110.01291484769432, 125.46488882332544, 121.24645626255418, 135.87043875544455], [154.87670501106774, 124.45712875915734, 157.33520915081402, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 150.72696126211756, 153.1866101146596, 155.4404734500336], [157.39431967157654, 118.72621855108888, 165.0467816984108, 168.3072369000775, 154.37664116275025, 114.51332186490818, 123.15215301127888, 128.67365323558175, 168.4348448525051, 160.21040114328096], [132.6393307913183, 109.30686173945848, 145.99049101750552, 152.59811248205753, 165.52450200376143, 117.34929630919373, 129.6409490643926, 152.35447181627313, 157.37714922337852, 161.60798730295116], [114.81208960698191, 87.37079030560386, 151.91364086278085, 155.88443549023452, 207.6215621572906, 67.56721883738453, 141.12963570062718, 155.44837157647052, 153.36883424895083, 192.04893929564705], [156.67370056557374, 124.99374425683207, 141.71845826734344, 137.26118395166182, 129.8751358858144, 135.04516650593146, 134.92129063968494, 126.20359047162871, 131.26678890750526, 182.48764818137406], [165.24117105960053, 133.77087149912916, 129.9614208259944, 121.00987965148478, 124.0617095913029, 124.99420175139073, 145.07648926363632, 125.14749257346011, 133.51187048282097, 194.0374710761797], [148.65858587031735, 117.5537430787448, 152.7370674658746, 155.0185002942349, 147.46163154928857, 129.97949714189932, 132.1733655775968, 150.43382549066143, 156.29210499732608, 168.29369368023086], [154.87670501106774, 124.45712875915734, 157.33520915081402, 139.44618970864255, 162.91689858892633, 112.69313077614252, 112.64060886497516, 150.72696126211756, 153.1866101146596, 155.4404734500336], [174.10245819655114, 127.80900078262174, 138.67139289299246, 148.41069607289663, 153.6350666551481, 103.46472832433717, 130.22281241842936, 147.4818180038071, 152.50682731933753, 157.6981277590819], [114.73266608848746, 89.39802544766577, 158.94539134495167, 152.6694368363921, 216.76711179742992, 67.24104216623691, 139.9800325976516, 152.85502811046752, 160.06957993685043, 185.67270551646817], [163.82826724191202, 123.63300303116105, 162.8980670120787, 166.58612468713937, 158.67319842829247, 101.19007738890186, 123.85647903797361, 141.86796497619403, 159.9811243798996, 158.63953984939445], [145.0072351499823, 115.99968345962576, 160.68230623339542, 152.3530590210606, 167.1076278296097, 131.08931955966278, 114.54546057653036, 150.04147491293364, 155.30290240960926, 140.86380002454607], [149.7529984808466, 108.80052007547977, 124.96810248186745, 146.0270227777066, 171.51514835196625, 98.79095122172545, 131.01688305315017, 147.11708785009412, 174.0852436128256, 192.9599715968946], [144.55856538564217, 117.02977381184573, 151.09093700806469, 170.31849702527362, 189.88602050509368, 111.78524265062529, 106.75016416033765, 149.20146450350555, 161.4668277430309, 146.78621271509914], [140.2268461963245, 116.71115157478997, 146.52034871887318, 146.389151580322, 152.9818486418794, 106.05265716177503, 131.3508218040346, 147.3827546710329, 173.23148359875637, 165.37466641996363], [154.2527428966532, 117.80024702535607, 164.2594332885985, 167.82531633195677, 150.90075080208038, 111.02924005724354, 99.95541985534355, 162.24143788372814, 165.1755696808328, 156.3585509104705], [146.68028294257556, 110.73139395055306, 159.36968986240163, 152.35051116574624, 174.90210786655473, 131.88990376903146, 109.6514739753097, 149.19676116288565, 154.1348794612632, 141.82027184671585], [132.6393307913183, 109.30686173945848, 145.99049101750552, 152.59811248205753, 165.52450200376143, 117.34929630919373, 129.6409490643926, 152.35447181627313, 157.37714922337852, 161.60798730295116], [169.16533358350605, 125.2512122003425, 124.36982905582596, 152.3431774421878, 164.55270315503893, 99.58614228205624, 138.9677058715599, 154.38699831564628, 167.33125598678217, 152.1864118047564], [151.3848407559981, 117.35033497131577, 159.26754100958533, 179.77760037675822, 149.5328415957601, 113.27968378965878, 123.670636716717, 153.30867936653834, 162.3419977297616, 155.28502904089973], [138.20605623854652, 107.42348781850717, 129.21584774205314, 142.2134787300486, 192.8664244086329, 96.20732846975696, 131.92385143024265, 156.3132038929684, 172.34092474542578, 184.7627903630174], [155.31948812344817, 103.54968781024894, 155.54440994011514, 159.64573144883576, 147.03153222429555, 100.29278139457293, 152.96449306880106, 129.3847328892758, 172.26759503296182, 186.13756010516815], [124.60931392388997, 99.55757900064643, 161.99929959628253, 150.1285082839572, 186.11983693459018, 86.00430019489998, 119.13204577034072, 155.41436252761594, 169.16448238826908, 170.3493231523084], [155.31460127025164, 124.00260960556245, 148.60376550908018, 164.7376404534931, 161.71931721747035, 112.3850680839479, 114.1079803199717, 149.60165093783095, 157.59666266767624, 140.65031941257772], [153.1476310248567, 118.1329600449769, 129.3980487071801, 158.37058800553137, 170.7977841821514, 107.94684317141325, 122.26963812067054, 161.0180127552807, 144.70026811490482, 151.10468681449436], [149.0250338729308, 116.77434277151853, 162.14817871023328, 165.63041794718413, 164.30078521222296, 111.43165327141746, 95.09076225078535, 162.21262866457795, 165.63738490665054, 157.24096925588108], [167.0289090491371, 124.30893920494574, 153.50285471754952, 158.8221000494878, 140.38758830030181, 101.42229138743608, 136.09796166251127, 155.39385433707233, 159.10033495026562, 159.92079055338738], [167.0289090491371, 124.30893920494574, 153.50285471754952, 158.8221000494878, 140.38758830030181, 101.42229138743608, 136.09796166251127, 155.39385433707233, 159.10033495026562, 159.92079055338738], [151.49494337387458, 117.63970585649903, 163.36518294294515, 162.4387606206083, 155.6800257924122, 113.25638832677038, 117.6841561482807, 160.83878709456383, 159.34809118225894, 161.23989139159553], [152.7282052709074, 130.41874324998875, 125.82420113609076, 156.97943007117505, 157.16274510072986, 126.51035377237639, 132.61048893821945, 159.55495885505314, 143.6280207101792, 136.0236397347833], [116.75519767144029, 88.99311376250257, 147.25424111377666, 170.08749434033558, 210.62762868750434, 61.67641125468947, 143.08011862115282, 152.54965543170462, 163.87724299261785, 179.7845752589638], [181.393153961203, 136.65303694070522, 125.90506986307487, 151.23293415828567, 167.04522306488312, 103.96871006288565, 114.83430969632307, 160.9344401999319, 142.79236673817732, 131.87396315470303], [153.1476310248567, 118.1329600449769, 129.3980487071801, 158.37058800553137, 170.7977841821514, 107.94684317141325, 122.26963812067054, 161.0180127552807, 144.70026811490482, 151.10468681449436], [149.27816962680123, 108.37247732346466, 138.71329142679446, 152.99701822494, 183.85670983256415, 98.26543736382182, 127.5550170615973, 153.75067512774277, 157.57839871208935, 183.54169965397787], [151.3848407559981, 117.35033497131577, 159.26754100958533, 179.77760037675822, 149.5328415957601, 113.27968378965878, 123.670636716717, 153.30867936653834, 162.3419977297616, 155.28502904089973], [152.58831894614698, 110.97678531179112, 128.30784401390054, 140.0858619551157, 178.4893576609055, 101.31091038534413, 122.7854912698353, 155.3982510541831, 171.3023709881371, 183.82724076092006]]</t>
+          <t>[[146.32011168648035, 144.67145252432897, 142.73890362706453, 154.79845436333184, 159.45171898896723, 150.62662250278504, 157.51393343833843, 135.9279498414939, 174.53941573285547, 126.13743609401969], [151.35497286393942, 160.76870351660634, 141.5898180137468, 170.37891849752756, 144.76198125641537, 148.17369689738956, 155.41589728594445, 137.2068043654447, 130.08918788169967, 153.9947816423278], [151.71309806276054, 145.84060177663494, 151.0469631011355, 131.9515453373102, 154.73099956302778, 164.21354992089942, 152.72615359751535, 147.85801245832903, 157.57612107093095, 132.14042270360883], [129.05400767791087, 157.96633614306174, 159.2189293568144, 160.1591176794438, 153.0674498817814, 143.42886777327604, 150.21460051626906, 143.56065688302098, 140.91813557529593, 156.13445446783376], [120.62656642720097, 144.9759834615558, 159.77335578927378, 150.25641588389664, 160.23553851735193, 151.5489200543449, 157.35802626153247, 137.74758779652467, 148.29729094968408, 158.03703808881704]]</t>
         </is>
       </c>
     </row>

</xml_diff>